<commit_message>
feat: add a config per standard grid cell and a run record
E0 step 23 (D70). configs/grid/ holds cells 1, 2, 5, 6, 5' and 6':
open-ended, 300 steps, $50 ceiling, empty-handed like FLE's open_play,
differing only in model, human backend and cell label (a test enforces
it). Cells 3, 4, 7, 8 wait for the E2 harness, which is refused until
then. Every trajectory now opens with a run record holding the goal,
the full resolved config and the git commit, and annotation validation
checks cell, harness and human against it.

Also updates the codebook workbook to D69 (unstuck computed on export,
column P grey, grid-cell drop-down), with openpyxl as a dev dependency
for editing it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/codebook-v0.xlsx
+++ b/docs/codebook-v0.xlsx
@@ -66,7 +66,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -86,6 +86,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -116,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -149,6 +154,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -605,7 +616,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>One row per stuck event - every time the stuck detector fires, whether or not a human answered. Stuck events in no-human runs (grid cells 1, 4, 5, 8) get error codes only.</t>
+          <t>One row per stuck event - every time the stuck detector fires, whether or not a human answered. Stuck events in no-human runs (grid cells 1, 4, 5, 8 and 5', 8') get error codes only.</t>
         </is>
       </c>
     </row>
@@ -617,7 +628,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>1) Open the run's trajectory; list its intervention records (each is one stuck event). 2) Read the ~5 steps before the event: the policy code, execution errors and verifier reasons. 3) Pick ONE primary error code (the root cause) and optionally one secondary. 4) If a human answered, paste the text verbatim and code it the same way. 5) Fill 'unstuck' with the rule below. 6) Record codebook version and your initials.</t>
+          <t>1) Open the run's trajectory; list its intervention records (each is one stuck event). 2) Read the ~5 steps before the event: the policy code, execution errors and verifier reasons. 3) Pick ONE primary error code (the root cause) and optionally one secondary. 4) If a human answered, code the guidance the same way (the text itself is copied from the trajectory on export). 5) Leave 'unstuck' blank - it is computed on export (rule below). 6) Record codebook version and your initials. 7) Export and validate: python -m factorio_maxxing.annotations export</t>
         </is>
       </c>
     </row>
@@ -636,12 +647,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Unstuck rule (draft)</t>
+          <t>Unstuck rule</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>'yes' if, within k steps after the event, the Scorer records a new milestone OR the stuck detector does not fire again; 'no' otherwise; 'n/a' if the run ended within k steps. Draft wording - for the research lead to confirm.</t>
+          <t>Computed on export from the Scorer (decisions D69): 'yes' if a milestone is first reached within k steps after the event; 'n/a' if the run ended sooner; 'no' otherwise. A milestone first reached at the event's own step does not count. If you do type a value in column P it must match, or the export stops.</t>
         </is>
       </c>
     </row>
@@ -675,7 +686,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Yellow cells are the ones you fill in (Annotations sheet, and k above). The 'Worked examples' sheet shows the expected format with real stuck events from the goal-5 rescue run.</t>
+          <t>Yellow cells are the ones you fill in (Annotations sheet, and k above). Grey column P is computed on export. Columns C, G, H and N are for reading only: export copies policy model, intervention_index, stuck_reason and guidance text verbatim from the trajectory. The 'Worked examples' sheet shows the expected format with real stuck events from the goal-5 rescue run.</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1509,7 @@
       <c r="M2" s="8" t="n"/>
       <c r="N2" s="8" t="n"/>
       <c r="O2" s="8" t="n"/>
-      <c r="P2" s="8" t="n"/>
+      <c r="P2" s="16" t="n"/>
       <c r="Q2" s="8" t="n"/>
       <c r="R2" s="8" t="n"/>
       <c r="S2" s="8" t="n"/>
@@ -1519,7 +1530,7 @@
       <c r="M3" s="8" t="n"/>
       <c r="N3" s="8" t="n"/>
       <c r="O3" s="8" t="n"/>
-      <c r="P3" s="8" t="n"/>
+      <c r="P3" s="16" t="n"/>
       <c r="Q3" s="8" t="n"/>
       <c r="R3" s="8" t="n"/>
       <c r="S3" s="8" t="n"/>
@@ -1540,7 +1551,7 @@
       <c r="M4" s="8" t="n"/>
       <c r="N4" s="8" t="n"/>
       <c r="O4" s="8" t="n"/>
-      <c r="P4" s="8" t="n"/>
+      <c r="P4" s="16" t="n"/>
       <c r="Q4" s="8" t="n"/>
       <c r="R4" s="8" t="n"/>
       <c r="S4" s="8" t="n"/>
@@ -1561,7 +1572,7 @@
       <c r="M5" s="8" t="n"/>
       <c r="N5" s="8" t="n"/>
       <c r="O5" s="8" t="n"/>
-      <c r="P5" s="8" t="n"/>
+      <c r="P5" s="16" t="n"/>
       <c r="Q5" s="8" t="n"/>
       <c r="R5" s="8" t="n"/>
       <c r="S5" s="8" t="n"/>
@@ -1582,7 +1593,7 @@
       <c r="M6" s="8" t="n"/>
       <c r="N6" s="8" t="n"/>
       <c r="O6" s="8" t="n"/>
-      <c r="P6" s="8" t="n"/>
+      <c r="P6" s="16" t="n"/>
       <c r="Q6" s="8" t="n"/>
       <c r="R6" s="8" t="n"/>
       <c r="S6" s="8" t="n"/>
@@ -1603,7 +1614,7 @@
       <c r="M7" s="8" t="n"/>
       <c r="N7" s="8" t="n"/>
       <c r="O7" s="8" t="n"/>
-      <c r="P7" s="8" t="n"/>
+      <c r="P7" s="16" t="n"/>
       <c r="Q7" s="8" t="n"/>
       <c r="R7" s="8" t="n"/>
       <c r="S7" s="8" t="n"/>
@@ -1624,7 +1635,7 @@
       <c r="M8" s="8" t="n"/>
       <c r="N8" s="8" t="n"/>
       <c r="O8" s="8" t="n"/>
-      <c r="P8" s="8" t="n"/>
+      <c r="P8" s="16" t="n"/>
       <c r="Q8" s="8" t="n"/>
       <c r="R8" s="8" t="n"/>
       <c r="S8" s="8" t="n"/>
@@ -1645,7 +1656,7 @@
       <c r="M9" s="8" t="n"/>
       <c r="N9" s="8" t="n"/>
       <c r="O9" s="8" t="n"/>
-      <c r="P9" s="8" t="n"/>
+      <c r="P9" s="16" t="n"/>
       <c r="Q9" s="8" t="n"/>
       <c r="R9" s="8" t="n"/>
       <c r="S9" s="8" t="n"/>
@@ -1666,7 +1677,7 @@
       <c r="M10" s="8" t="n"/>
       <c r="N10" s="8" t="n"/>
       <c r="O10" s="8" t="n"/>
-      <c r="P10" s="8" t="n"/>
+      <c r="P10" s="16" t="n"/>
       <c r="Q10" s="8" t="n"/>
       <c r="R10" s="8" t="n"/>
       <c r="S10" s="8" t="n"/>
@@ -1687,7 +1698,7 @@
       <c r="M11" s="8" t="n"/>
       <c r="N11" s="8" t="n"/>
       <c r="O11" s="8" t="n"/>
-      <c r="P11" s="8" t="n"/>
+      <c r="P11" s="16" t="n"/>
       <c r="Q11" s="8" t="n"/>
       <c r="R11" s="8" t="n"/>
       <c r="S11" s="8" t="n"/>
@@ -1708,7 +1719,7 @@
       <c r="M12" s="8" t="n"/>
       <c r="N12" s="8" t="n"/>
       <c r="O12" s="8" t="n"/>
-      <c r="P12" s="8" t="n"/>
+      <c r="P12" s="16" t="n"/>
       <c r="Q12" s="8" t="n"/>
       <c r="R12" s="8" t="n"/>
       <c r="S12" s="8" t="n"/>
@@ -1729,7 +1740,7 @@
       <c r="M13" s="8" t="n"/>
       <c r="N13" s="8" t="n"/>
       <c r="O13" s="8" t="n"/>
-      <c r="P13" s="8" t="n"/>
+      <c r="P13" s="16" t="n"/>
       <c r="Q13" s="8" t="n"/>
       <c r="R13" s="8" t="n"/>
       <c r="S13" s="8" t="n"/>
@@ -1750,7 +1761,7 @@
       <c r="M14" s="8" t="n"/>
       <c r="N14" s="8" t="n"/>
       <c r="O14" s="8" t="n"/>
-      <c r="P14" s="8" t="n"/>
+      <c r="P14" s="16" t="n"/>
       <c r="Q14" s="8" t="n"/>
       <c r="R14" s="8" t="n"/>
       <c r="S14" s="8" t="n"/>
@@ -1771,7 +1782,7 @@
       <c r="M15" s="8" t="n"/>
       <c r="N15" s="8" t="n"/>
       <c r="O15" s="8" t="n"/>
-      <c r="P15" s="8" t="n"/>
+      <c r="P15" s="16" t="n"/>
       <c r="Q15" s="8" t="n"/>
       <c r="R15" s="8" t="n"/>
       <c r="S15" s="8" t="n"/>
@@ -1792,7 +1803,7 @@
       <c r="M16" s="8" t="n"/>
       <c r="N16" s="8" t="n"/>
       <c r="O16" s="8" t="n"/>
-      <c r="P16" s="8" t="n"/>
+      <c r="P16" s="16" t="n"/>
       <c r="Q16" s="8" t="n"/>
       <c r="R16" s="8" t="n"/>
       <c r="S16" s="8" t="n"/>
@@ -1813,7 +1824,7 @@
       <c r="M17" s="8" t="n"/>
       <c r="N17" s="8" t="n"/>
       <c r="O17" s="8" t="n"/>
-      <c r="P17" s="8" t="n"/>
+      <c r="P17" s="16" t="n"/>
       <c r="Q17" s="8" t="n"/>
       <c r="R17" s="8" t="n"/>
       <c r="S17" s="8" t="n"/>
@@ -1834,7 +1845,7 @@
       <c r="M18" s="8" t="n"/>
       <c r="N18" s="8" t="n"/>
       <c r="O18" s="8" t="n"/>
-      <c r="P18" s="8" t="n"/>
+      <c r="P18" s="16" t="n"/>
       <c r="Q18" s="8" t="n"/>
       <c r="R18" s="8" t="n"/>
       <c r="S18" s="8" t="n"/>
@@ -1855,7 +1866,7 @@
       <c r="M19" s="8" t="n"/>
       <c r="N19" s="8" t="n"/>
       <c r="O19" s="8" t="n"/>
-      <c r="P19" s="8" t="n"/>
+      <c r="P19" s="16" t="n"/>
       <c r="Q19" s="8" t="n"/>
       <c r="R19" s="8" t="n"/>
       <c r="S19" s="8" t="n"/>
@@ -1876,7 +1887,7 @@
       <c r="M20" s="8" t="n"/>
       <c r="N20" s="8" t="n"/>
       <c r="O20" s="8" t="n"/>
-      <c r="P20" s="8" t="n"/>
+      <c r="P20" s="16" t="n"/>
       <c r="Q20" s="8" t="n"/>
       <c r="R20" s="8" t="n"/>
       <c r="S20" s="8" t="n"/>
@@ -1897,7 +1908,7 @@
       <c r="M21" s="8" t="n"/>
       <c r="N21" s="8" t="n"/>
       <c r="O21" s="8" t="n"/>
-      <c r="P21" s="8" t="n"/>
+      <c r="P21" s="16" t="n"/>
       <c r="Q21" s="8" t="n"/>
       <c r="R21" s="8" t="n"/>
       <c r="S21" s="8" t="n"/>
@@ -1918,7 +1929,7 @@
       <c r="M22" s="9" t="n"/>
       <c r="N22" s="9" t="n"/>
       <c r="O22" s="9" t="n"/>
-      <c r="P22" s="9" t="n"/>
+      <c r="P22" s="17" t="n"/>
       <c r="Q22" s="9" t="n"/>
       <c r="R22" s="9" t="n"/>
       <c r="S22" s="9" t="n"/>
@@ -1939,7 +1950,7 @@
       <c r="M23" s="9" t="n"/>
       <c r="N23" s="9" t="n"/>
       <c r="O23" s="9" t="n"/>
-      <c r="P23" s="9" t="n"/>
+      <c r="P23" s="17" t="n"/>
       <c r="Q23" s="9" t="n"/>
       <c r="R23" s="9" t="n"/>
       <c r="S23" s="9" t="n"/>
@@ -1960,7 +1971,7 @@
       <c r="M24" s="9" t="n"/>
       <c r="N24" s="9" t="n"/>
       <c r="O24" s="9" t="n"/>
-      <c r="P24" s="9" t="n"/>
+      <c r="P24" s="17" t="n"/>
       <c r="Q24" s="9" t="n"/>
       <c r="R24" s="9" t="n"/>
       <c r="S24" s="9" t="n"/>
@@ -1981,7 +1992,7 @@
       <c r="M25" s="9" t="n"/>
       <c r="N25" s="9" t="n"/>
       <c r="O25" s="9" t="n"/>
-      <c r="P25" s="9" t="n"/>
+      <c r="P25" s="17" t="n"/>
       <c r="Q25" s="9" t="n"/>
       <c r="R25" s="9" t="n"/>
       <c r="S25" s="9" t="n"/>
@@ -2002,7 +2013,7 @@
       <c r="M26" s="9" t="n"/>
       <c r="N26" s="9" t="n"/>
       <c r="O26" s="9" t="n"/>
-      <c r="P26" s="9" t="n"/>
+      <c r="P26" s="17" t="n"/>
       <c r="Q26" s="9" t="n"/>
       <c r="R26" s="9" t="n"/>
       <c r="S26" s="9" t="n"/>
@@ -2023,7 +2034,7 @@
       <c r="M27" s="9" t="n"/>
       <c r="N27" s="9" t="n"/>
       <c r="O27" s="9" t="n"/>
-      <c r="P27" s="9" t="n"/>
+      <c r="P27" s="17" t="n"/>
       <c r="Q27" s="9" t="n"/>
       <c r="R27" s="9" t="n"/>
       <c r="S27" s="9" t="n"/>
@@ -2044,7 +2055,7 @@
       <c r="M28" s="9" t="n"/>
       <c r="N28" s="9" t="n"/>
       <c r="O28" s="9" t="n"/>
-      <c r="P28" s="9" t="n"/>
+      <c r="P28" s="17" t="n"/>
       <c r="Q28" s="9" t="n"/>
       <c r="R28" s="9" t="n"/>
       <c r="S28" s="9" t="n"/>
@@ -2065,7 +2076,7 @@
       <c r="M29" s="9" t="n"/>
       <c r="N29" s="9" t="n"/>
       <c r="O29" s="9" t="n"/>
-      <c r="P29" s="9" t="n"/>
+      <c r="P29" s="17" t="n"/>
       <c r="Q29" s="9" t="n"/>
       <c r="R29" s="9" t="n"/>
       <c r="S29" s="9" t="n"/>
@@ -2086,7 +2097,7 @@
       <c r="M30" s="9" t="n"/>
       <c r="N30" s="9" t="n"/>
       <c r="O30" s="9" t="n"/>
-      <c r="P30" s="9" t="n"/>
+      <c r="P30" s="17" t="n"/>
       <c r="Q30" s="9" t="n"/>
       <c r="R30" s="9" t="n"/>
       <c r="S30" s="9" t="n"/>
@@ -2107,7 +2118,7 @@
       <c r="M31" s="9" t="n"/>
       <c r="N31" s="9" t="n"/>
       <c r="O31" s="9" t="n"/>
-      <c r="P31" s="9" t="n"/>
+      <c r="P31" s="17" t="n"/>
       <c r="Q31" s="9" t="n"/>
       <c r="R31" s="9" t="n"/>
       <c r="S31" s="9" t="n"/>
@@ -2128,7 +2139,7 @@
       <c r="M32" s="9" t="n"/>
       <c r="N32" s="9" t="n"/>
       <c r="O32" s="9" t="n"/>
-      <c r="P32" s="9" t="n"/>
+      <c r="P32" s="17" t="n"/>
       <c r="Q32" s="9" t="n"/>
       <c r="R32" s="9" t="n"/>
       <c r="S32" s="9" t="n"/>
@@ -2149,7 +2160,7 @@
       <c r="M33" s="9" t="n"/>
       <c r="N33" s="9" t="n"/>
       <c r="O33" s="9" t="n"/>
-      <c r="P33" s="9" t="n"/>
+      <c r="P33" s="17" t="n"/>
       <c r="Q33" s="9" t="n"/>
       <c r="R33" s="9" t="n"/>
       <c r="S33" s="9" t="n"/>
@@ -2170,7 +2181,7 @@
       <c r="M34" s="9" t="n"/>
       <c r="N34" s="9" t="n"/>
       <c r="O34" s="9" t="n"/>
-      <c r="P34" s="9" t="n"/>
+      <c r="P34" s="17" t="n"/>
       <c r="Q34" s="9" t="n"/>
       <c r="R34" s="9" t="n"/>
       <c r="S34" s="9" t="n"/>
@@ -2191,7 +2202,7 @@
       <c r="M35" s="9" t="n"/>
       <c r="N35" s="9" t="n"/>
       <c r="O35" s="9" t="n"/>
-      <c r="P35" s="9" t="n"/>
+      <c r="P35" s="17" t="n"/>
       <c r="Q35" s="9" t="n"/>
       <c r="R35" s="9" t="n"/>
       <c r="S35" s="9" t="n"/>
@@ -2212,7 +2223,7 @@
       <c r="M36" s="9" t="n"/>
       <c r="N36" s="9" t="n"/>
       <c r="O36" s="9" t="n"/>
-      <c r="P36" s="9" t="n"/>
+      <c r="P36" s="17" t="n"/>
       <c r="Q36" s="9" t="n"/>
       <c r="R36" s="9" t="n"/>
       <c r="S36" s="9" t="n"/>
@@ -2233,7 +2244,7 @@
       <c r="M37" s="9" t="n"/>
       <c r="N37" s="9" t="n"/>
       <c r="O37" s="9" t="n"/>
-      <c r="P37" s="9" t="n"/>
+      <c r="P37" s="17" t="n"/>
       <c r="Q37" s="9" t="n"/>
       <c r="R37" s="9" t="n"/>
       <c r="S37" s="9" t="n"/>
@@ -2254,7 +2265,7 @@
       <c r="M38" s="9" t="n"/>
       <c r="N38" s="9" t="n"/>
       <c r="O38" s="9" t="n"/>
-      <c r="P38" s="9" t="n"/>
+      <c r="P38" s="17" t="n"/>
       <c r="Q38" s="9" t="n"/>
       <c r="R38" s="9" t="n"/>
       <c r="S38" s="9" t="n"/>
@@ -2275,7 +2286,7 @@
       <c r="M39" s="9" t="n"/>
       <c r="N39" s="9" t="n"/>
       <c r="O39" s="9" t="n"/>
-      <c r="P39" s="9" t="n"/>
+      <c r="P39" s="17" t="n"/>
       <c r="Q39" s="9" t="n"/>
       <c r="R39" s="9" t="n"/>
       <c r="S39" s="9" t="n"/>
@@ -2296,7 +2307,7 @@
       <c r="M40" s="9" t="n"/>
       <c r="N40" s="9" t="n"/>
       <c r="O40" s="9" t="n"/>
-      <c r="P40" s="9" t="n"/>
+      <c r="P40" s="17" t="n"/>
       <c r="Q40" s="9" t="n"/>
       <c r="R40" s="9" t="n"/>
       <c r="S40" s="9" t="n"/>
@@ -2317,7 +2328,7 @@
       <c r="M41" s="9" t="n"/>
       <c r="N41" s="9" t="n"/>
       <c r="O41" s="9" t="n"/>
-      <c r="P41" s="9" t="n"/>
+      <c r="P41" s="17" t="n"/>
       <c r="Q41" s="9" t="n"/>
       <c r="R41" s="9" t="n"/>
       <c r="S41" s="9" t="n"/>
@@ -2338,7 +2349,7 @@
       <c r="M42" s="9" t="n"/>
       <c r="N42" s="9" t="n"/>
       <c r="O42" s="9" t="n"/>
-      <c r="P42" s="9" t="n"/>
+      <c r="P42" s="17" t="n"/>
       <c r="Q42" s="9" t="n"/>
       <c r="R42" s="9" t="n"/>
       <c r="S42" s="9" t="n"/>
@@ -2359,7 +2370,7 @@
       <c r="M43" s="9" t="n"/>
       <c r="N43" s="9" t="n"/>
       <c r="O43" s="9" t="n"/>
-      <c r="P43" s="9" t="n"/>
+      <c r="P43" s="17" t="n"/>
       <c r="Q43" s="9" t="n"/>
       <c r="R43" s="9" t="n"/>
       <c r="S43" s="9" t="n"/>
@@ -2380,7 +2391,7 @@
       <c r="M44" s="9" t="n"/>
       <c r="N44" s="9" t="n"/>
       <c r="O44" s="9" t="n"/>
-      <c r="P44" s="9" t="n"/>
+      <c r="P44" s="17" t="n"/>
       <c r="Q44" s="9" t="n"/>
       <c r="R44" s="9" t="n"/>
       <c r="S44" s="9" t="n"/>
@@ -2401,7 +2412,7 @@
       <c r="M45" s="9" t="n"/>
       <c r="N45" s="9" t="n"/>
       <c r="O45" s="9" t="n"/>
-      <c r="P45" s="9" t="n"/>
+      <c r="P45" s="17" t="n"/>
       <c r="Q45" s="9" t="n"/>
       <c r="R45" s="9" t="n"/>
       <c r="S45" s="9" t="n"/>
@@ -2422,7 +2433,7 @@
       <c r="M46" s="9" t="n"/>
       <c r="N46" s="9" t="n"/>
       <c r="O46" s="9" t="n"/>
-      <c r="P46" s="9" t="n"/>
+      <c r="P46" s="17" t="n"/>
       <c r="Q46" s="9" t="n"/>
       <c r="R46" s="9" t="n"/>
       <c r="S46" s="9" t="n"/>
@@ -2443,7 +2454,7 @@
       <c r="M47" s="9" t="n"/>
       <c r="N47" s="9" t="n"/>
       <c r="O47" s="9" t="n"/>
-      <c r="P47" s="9" t="n"/>
+      <c r="P47" s="17" t="n"/>
       <c r="Q47" s="9" t="n"/>
       <c r="R47" s="9" t="n"/>
       <c r="S47" s="9" t="n"/>
@@ -2464,7 +2475,7 @@
       <c r="M48" s="9" t="n"/>
       <c r="N48" s="9" t="n"/>
       <c r="O48" s="9" t="n"/>
-      <c r="P48" s="9" t="n"/>
+      <c r="P48" s="17" t="n"/>
       <c r="Q48" s="9" t="n"/>
       <c r="R48" s="9" t="n"/>
       <c r="S48" s="9" t="n"/>
@@ -2485,7 +2496,7 @@
       <c r="M49" s="9" t="n"/>
       <c r="N49" s="9" t="n"/>
       <c r="O49" s="9" t="n"/>
-      <c r="P49" s="9" t="n"/>
+      <c r="P49" s="17" t="n"/>
       <c r="Q49" s="9" t="n"/>
       <c r="R49" s="9" t="n"/>
       <c r="S49" s="9" t="n"/>
@@ -2506,7 +2517,7 @@
       <c r="M50" s="9" t="n"/>
       <c r="N50" s="9" t="n"/>
       <c r="O50" s="9" t="n"/>
-      <c r="P50" s="9" t="n"/>
+      <c r="P50" s="17" t="n"/>
       <c r="Q50" s="9" t="n"/>
       <c r="R50" s="9" t="n"/>
       <c r="S50" s="9" t="n"/>
@@ -2527,7 +2538,7 @@
       <c r="M51" s="9" t="n"/>
       <c r="N51" s="9" t="n"/>
       <c r="O51" s="9" t="n"/>
-      <c r="P51" s="9" t="n"/>
+      <c r="P51" s="17" t="n"/>
       <c r="Q51" s="9" t="n"/>
       <c r="R51" s="9" t="n"/>
       <c r="S51" s="9" t="n"/>
@@ -2548,7 +2559,7 @@
       <c r="M52" s="9" t="n"/>
       <c r="N52" s="9" t="n"/>
       <c r="O52" s="9" t="n"/>
-      <c r="P52" s="9" t="n"/>
+      <c r="P52" s="17" t="n"/>
       <c r="Q52" s="9" t="n"/>
       <c r="R52" s="9" t="n"/>
       <c r="S52" s="9" t="n"/>
@@ -2569,7 +2580,7 @@
       <c r="M53" s="9" t="n"/>
       <c r="N53" s="9" t="n"/>
       <c r="O53" s="9" t="n"/>
-      <c r="P53" s="9" t="n"/>
+      <c r="P53" s="17" t="n"/>
       <c r="Q53" s="9" t="n"/>
       <c r="R53" s="9" t="n"/>
       <c r="S53" s="9" t="n"/>
@@ -2590,7 +2601,7 @@
       <c r="M54" s="9" t="n"/>
       <c r="N54" s="9" t="n"/>
       <c r="O54" s="9" t="n"/>
-      <c r="P54" s="9" t="n"/>
+      <c r="P54" s="17" t="n"/>
       <c r="Q54" s="9" t="n"/>
       <c r="R54" s="9" t="n"/>
       <c r="S54" s="9" t="n"/>
@@ -2611,7 +2622,7 @@
       <c r="M55" s="9" t="n"/>
       <c r="N55" s="9" t="n"/>
       <c r="O55" s="9" t="n"/>
-      <c r="P55" s="9" t="n"/>
+      <c r="P55" s="17" t="n"/>
       <c r="Q55" s="9" t="n"/>
       <c r="R55" s="9" t="n"/>
       <c r="S55" s="9" t="n"/>
@@ -2632,7 +2643,7 @@
       <c r="M56" s="9" t="n"/>
       <c r="N56" s="9" t="n"/>
       <c r="O56" s="9" t="n"/>
-      <c r="P56" s="9" t="n"/>
+      <c r="P56" s="17" t="n"/>
       <c r="Q56" s="9" t="n"/>
       <c r="R56" s="9" t="n"/>
       <c r="S56" s="9" t="n"/>
@@ -2653,7 +2664,7 @@
       <c r="M57" s="9" t="n"/>
       <c r="N57" s="9" t="n"/>
       <c r="O57" s="9" t="n"/>
-      <c r="P57" s="9" t="n"/>
+      <c r="P57" s="17" t="n"/>
       <c r="Q57" s="9" t="n"/>
       <c r="R57" s="9" t="n"/>
       <c r="S57" s="9" t="n"/>
@@ -2674,7 +2685,7 @@
       <c r="M58" s="9" t="n"/>
       <c r="N58" s="9" t="n"/>
       <c r="O58" s="9" t="n"/>
-      <c r="P58" s="9" t="n"/>
+      <c r="P58" s="17" t="n"/>
       <c r="Q58" s="9" t="n"/>
       <c r="R58" s="9" t="n"/>
       <c r="S58" s="9" t="n"/>
@@ -2695,7 +2706,7 @@
       <c r="M59" s="9" t="n"/>
       <c r="N59" s="9" t="n"/>
       <c r="O59" s="9" t="n"/>
-      <c r="P59" s="9" t="n"/>
+      <c r="P59" s="17" t="n"/>
       <c r="Q59" s="9" t="n"/>
       <c r="R59" s="9" t="n"/>
       <c r="S59" s="9" t="n"/>
@@ -2716,7 +2727,7 @@
       <c r="M60" s="9" t="n"/>
       <c r="N60" s="9" t="n"/>
       <c r="O60" s="9" t="n"/>
-      <c r="P60" s="9" t="n"/>
+      <c r="P60" s="17" t="n"/>
       <c r="Q60" s="9" t="n"/>
       <c r="R60" s="9" t="n"/>
       <c r="S60" s="9" t="n"/>
@@ -2737,7 +2748,7 @@
       <c r="M61" s="9" t="n"/>
       <c r="N61" s="9" t="n"/>
       <c r="O61" s="9" t="n"/>
-      <c r="P61" s="9" t="n"/>
+      <c r="P61" s="17" t="n"/>
       <c r="Q61" s="9" t="n"/>
       <c r="R61" s="9" t="n"/>
       <c r="S61" s="9" t="n"/>
@@ -2758,7 +2769,7 @@
       <c r="M62" s="9" t="n"/>
       <c r="N62" s="9" t="n"/>
       <c r="O62" s="9" t="n"/>
-      <c r="P62" s="9" t="n"/>
+      <c r="P62" s="17" t="n"/>
       <c r="Q62" s="9" t="n"/>
       <c r="R62" s="9" t="n"/>
       <c r="S62" s="9" t="n"/>
@@ -2779,7 +2790,7 @@
       <c r="M63" s="9" t="n"/>
       <c r="N63" s="9" t="n"/>
       <c r="O63" s="9" t="n"/>
-      <c r="P63" s="9" t="n"/>
+      <c r="P63" s="17" t="n"/>
       <c r="Q63" s="9" t="n"/>
       <c r="R63" s="9" t="n"/>
       <c r="S63" s="9" t="n"/>
@@ -2800,7 +2811,7 @@
       <c r="M64" s="9" t="n"/>
       <c r="N64" s="9" t="n"/>
       <c r="O64" s="9" t="n"/>
-      <c r="P64" s="9" t="n"/>
+      <c r="P64" s="17" t="n"/>
       <c r="Q64" s="9" t="n"/>
       <c r="R64" s="9" t="n"/>
       <c r="S64" s="9" t="n"/>
@@ -2821,7 +2832,7 @@
       <c r="M65" s="9" t="n"/>
       <c r="N65" s="9" t="n"/>
       <c r="O65" s="9" t="n"/>
-      <c r="P65" s="9" t="n"/>
+      <c r="P65" s="17" t="n"/>
       <c r="Q65" s="9" t="n"/>
       <c r="R65" s="9" t="n"/>
       <c r="S65" s="9" t="n"/>
@@ -2842,7 +2853,7 @@
       <c r="M66" s="9" t="n"/>
       <c r="N66" s="9" t="n"/>
       <c r="O66" s="9" t="n"/>
-      <c r="P66" s="9" t="n"/>
+      <c r="P66" s="17" t="n"/>
       <c r="Q66" s="9" t="n"/>
       <c r="R66" s="9" t="n"/>
       <c r="S66" s="9" t="n"/>
@@ -2863,7 +2874,7 @@
       <c r="M67" s="9" t="n"/>
       <c r="N67" s="9" t="n"/>
       <c r="O67" s="9" t="n"/>
-      <c r="P67" s="9" t="n"/>
+      <c r="P67" s="17" t="n"/>
       <c r="Q67" s="9" t="n"/>
       <c r="R67" s="9" t="n"/>
       <c r="S67" s="9" t="n"/>
@@ -2884,7 +2895,7 @@
       <c r="M68" s="9" t="n"/>
       <c r="N68" s="9" t="n"/>
       <c r="O68" s="9" t="n"/>
-      <c r="P68" s="9" t="n"/>
+      <c r="P68" s="17" t="n"/>
       <c r="Q68" s="9" t="n"/>
       <c r="R68" s="9" t="n"/>
       <c r="S68" s="9" t="n"/>
@@ -2905,7 +2916,7 @@
       <c r="M69" s="9" t="n"/>
       <c r="N69" s="9" t="n"/>
       <c r="O69" s="9" t="n"/>
-      <c r="P69" s="9" t="n"/>
+      <c r="P69" s="17" t="n"/>
       <c r="Q69" s="9" t="n"/>
       <c r="R69" s="9" t="n"/>
       <c r="S69" s="9" t="n"/>
@@ -2926,7 +2937,7 @@
       <c r="M70" s="9" t="n"/>
       <c r="N70" s="9" t="n"/>
       <c r="O70" s="9" t="n"/>
-      <c r="P70" s="9" t="n"/>
+      <c r="P70" s="17" t="n"/>
       <c r="Q70" s="9" t="n"/>
       <c r="R70" s="9" t="n"/>
       <c r="S70" s="9" t="n"/>
@@ -2947,7 +2958,7 @@
       <c r="M71" s="9" t="n"/>
       <c r="N71" s="9" t="n"/>
       <c r="O71" s="9" t="n"/>
-      <c r="P71" s="9" t="n"/>
+      <c r="P71" s="17" t="n"/>
       <c r="Q71" s="9" t="n"/>
       <c r="R71" s="9" t="n"/>
       <c r="S71" s="9" t="n"/>
@@ -2968,7 +2979,7 @@
       <c r="M72" s="9" t="n"/>
       <c r="N72" s="9" t="n"/>
       <c r="O72" s="9" t="n"/>
-      <c r="P72" s="9" t="n"/>
+      <c r="P72" s="17" t="n"/>
       <c r="Q72" s="9" t="n"/>
       <c r="R72" s="9" t="n"/>
       <c r="S72" s="9" t="n"/>
@@ -2989,7 +3000,7 @@
       <c r="M73" s="9" t="n"/>
       <c r="N73" s="9" t="n"/>
       <c r="O73" s="9" t="n"/>
-      <c r="P73" s="9" t="n"/>
+      <c r="P73" s="17" t="n"/>
       <c r="Q73" s="9" t="n"/>
       <c r="R73" s="9" t="n"/>
       <c r="S73" s="9" t="n"/>
@@ -3010,7 +3021,7 @@
       <c r="M74" s="9" t="n"/>
       <c r="N74" s="9" t="n"/>
       <c r="O74" s="9" t="n"/>
-      <c r="P74" s="9" t="n"/>
+      <c r="P74" s="17" t="n"/>
       <c r="Q74" s="9" t="n"/>
       <c r="R74" s="9" t="n"/>
       <c r="S74" s="9" t="n"/>
@@ -3031,7 +3042,7 @@
       <c r="M75" s="9" t="n"/>
       <c r="N75" s="9" t="n"/>
       <c r="O75" s="9" t="n"/>
-      <c r="P75" s="9" t="n"/>
+      <c r="P75" s="17" t="n"/>
       <c r="Q75" s="9" t="n"/>
       <c r="R75" s="9" t="n"/>
       <c r="S75" s="9" t="n"/>
@@ -3052,7 +3063,7 @@
       <c r="M76" s="9" t="n"/>
       <c r="N76" s="9" t="n"/>
       <c r="O76" s="9" t="n"/>
-      <c r="P76" s="9" t="n"/>
+      <c r="P76" s="17" t="n"/>
       <c r="Q76" s="9" t="n"/>
       <c r="R76" s="9" t="n"/>
       <c r="S76" s="9" t="n"/>
@@ -3073,7 +3084,7 @@
       <c r="M77" s="9" t="n"/>
       <c r="N77" s="9" t="n"/>
       <c r="O77" s="9" t="n"/>
-      <c r="P77" s="9" t="n"/>
+      <c r="P77" s="17" t="n"/>
       <c r="Q77" s="9" t="n"/>
       <c r="R77" s="9" t="n"/>
       <c r="S77" s="9" t="n"/>
@@ -3094,7 +3105,7 @@
       <c r="M78" s="9" t="n"/>
       <c r="N78" s="9" t="n"/>
       <c r="O78" s="9" t="n"/>
-      <c r="P78" s="9" t="n"/>
+      <c r="P78" s="17" t="n"/>
       <c r="Q78" s="9" t="n"/>
       <c r="R78" s="9" t="n"/>
       <c r="S78" s="9" t="n"/>
@@ -3115,7 +3126,7 @@
       <c r="M79" s="9" t="n"/>
       <c r="N79" s="9" t="n"/>
       <c r="O79" s="9" t="n"/>
-      <c r="P79" s="9" t="n"/>
+      <c r="P79" s="17" t="n"/>
       <c r="Q79" s="9" t="n"/>
       <c r="R79" s="9" t="n"/>
       <c r="S79" s="9" t="n"/>
@@ -3136,7 +3147,7 @@
       <c r="M80" s="9" t="n"/>
       <c r="N80" s="9" t="n"/>
       <c r="O80" s="9" t="n"/>
-      <c r="P80" s="9" t="n"/>
+      <c r="P80" s="17" t="n"/>
       <c r="Q80" s="9" t="n"/>
       <c r="R80" s="9" t="n"/>
       <c r="S80" s="9" t="n"/>
@@ -3157,7 +3168,7 @@
       <c r="M81" s="9" t="n"/>
       <c r="N81" s="9" t="n"/>
       <c r="O81" s="9" t="n"/>
-      <c r="P81" s="9" t="n"/>
+      <c r="P81" s="17" t="n"/>
       <c r="Q81" s="9" t="n"/>
       <c r="R81" s="9" t="n"/>
       <c r="S81" s="9" t="n"/>
@@ -3178,7 +3189,7 @@
       <c r="M82" s="9" t="n"/>
       <c r="N82" s="9" t="n"/>
       <c r="O82" s="9" t="n"/>
-      <c r="P82" s="9" t="n"/>
+      <c r="P82" s="17" t="n"/>
       <c r="Q82" s="9" t="n"/>
       <c r="R82" s="9" t="n"/>
       <c r="S82" s="9" t="n"/>
@@ -3199,7 +3210,7 @@
       <c r="M83" s="9" t="n"/>
       <c r="N83" s="9" t="n"/>
       <c r="O83" s="9" t="n"/>
-      <c r="P83" s="9" t="n"/>
+      <c r="P83" s="17" t="n"/>
       <c r="Q83" s="9" t="n"/>
       <c r="R83" s="9" t="n"/>
       <c r="S83" s="9" t="n"/>
@@ -3220,7 +3231,7 @@
       <c r="M84" s="9" t="n"/>
       <c r="N84" s="9" t="n"/>
       <c r="O84" s="9" t="n"/>
-      <c r="P84" s="9" t="n"/>
+      <c r="P84" s="17" t="n"/>
       <c r="Q84" s="9" t="n"/>
       <c r="R84" s="9" t="n"/>
       <c r="S84" s="9" t="n"/>
@@ -3241,7 +3252,7 @@
       <c r="M85" s="9" t="n"/>
       <c r="N85" s="9" t="n"/>
       <c r="O85" s="9" t="n"/>
-      <c r="P85" s="9" t="n"/>
+      <c r="P85" s="17" t="n"/>
       <c r="Q85" s="9" t="n"/>
       <c r="R85" s="9" t="n"/>
       <c r="S85" s="9" t="n"/>
@@ -3262,7 +3273,7 @@
       <c r="M86" s="9" t="n"/>
       <c r="N86" s="9" t="n"/>
       <c r="O86" s="9" t="n"/>
-      <c r="P86" s="9" t="n"/>
+      <c r="P86" s="17" t="n"/>
       <c r="Q86" s="9" t="n"/>
       <c r="R86" s="9" t="n"/>
       <c r="S86" s="9" t="n"/>
@@ -3283,7 +3294,7 @@
       <c r="M87" s="9" t="n"/>
       <c r="N87" s="9" t="n"/>
       <c r="O87" s="9" t="n"/>
-      <c r="P87" s="9" t="n"/>
+      <c r="P87" s="17" t="n"/>
       <c r="Q87" s="9" t="n"/>
       <c r="R87" s="9" t="n"/>
       <c r="S87" s="9" t="n"/>
@@ -3304,7 +3315,7 @@
       <c r="M88" s="9" t="n"/>
       <c r="N88" s="9" t="n"/>
       <c r="O88" s="9" t="n"/>
-      <c r="P88" s="9" t="n"/>
+      <c r="P88" s="17" t="n"/>
       <c r="Q88" s="9" t="n"/>
       <c r="R88" s="9" t="n"/>
       <c r="S88" s="9" t="n"/>
@@ -3325,7 +3336,7 @@
       <c r="M89" s="9" t="n"/>
       <c r="N89" s="9" t="n"/>
       <c r="O89" s="9" t="n"/>
-      <c r="P89" s="9" t="n"/>
+      <c r="P89" s="17" t="n"/>
       <c r="Q89" s="9" t="n"/>
       <c r="R89" s="9" t="n"/>
       <c r="S89" s="9" t="n"/>
@@ -3346,7 +3357,7 @@
       <c r="M90" s="9" t="n"/>
       <c r="N90" s="9" t="n"/>
       <c r="O90" s="9" t="n"/>
-      <c r="P90" s="9" t="n"/>
+      <c r="P90" s="17" t="n"/>
       <c r="Q90" s="9" t="n"/>
       <c r="R90" s="9" t="n"/>
       <c r="S90" s="9" t="n"/>
@@ -3367,7 +3378,7 @@
       <c r="M91" s="9" t="n"/>
       <c r="N91" s="9" t="n"/>
       <c r="O91" s="9" t="n"/>
-      <c r="P91" s="9" t="n"/>
+      <c r="P91" s="17" t="n"/>
       <c r="Q91" s="9" t="n"/>
       <c r="R91" s="9" t="n"/>
       <c r="S91" s="9" t="n"/>
@@ -3388,7 +3399,7 @@
       <c r="M92" s="9" t="n"/>
       <c r="N92" s="9" t="n"/>
       <c r="O92" s="9" t="n"/>
-      <c r="P92" s="9" t="n"/>
+      <c r="P92" s="17" t="n"/>
       <c r="Q92" s="9" t="n"/>
       <c r="R92" s="9" t="n"/>
       <c r="S92" s="9" t="n"/>
@@ -3409,7 +3420,7 @@
       <c r="M93" s="9" t="n"/>
       <c r="N93" s="9" t="n"/>
       <c r="O93" s="9" t="n"/>
-      <c r="P93" s="9" t="n"/>
+      <c r="P93" s="17" t="n"/>
       <c r="Q93" s="9" t="n"/>
       <c r="R93" s="9" t="n"/>
       <c r="S93" s="9" t="n"/>
@@ -3430,7 +3441,7 @@
       <c r="M94" s="9" t="n"/>
       <c r="N94" s="9" t="n"/>
       <c r="O94" s="9" t="n"/>
-      <c r="P94" s="9" t="n"/>
+      <c r="P94" s="17" t="n"/>
       <c r="Q94" s="9" t="n"/>
       <c r="R94" s="9" t="n"/>
       <c r="S94" s="9" t="n"/>
@@ -3451,7 +3462,7 @@
       <c r="M95" s="9" t="n"/>
       <c r="N95" s="9" t="n"/>
       <c r="O95" s="9" t="n"/>
-      <c r="P95" s="9" t="n"/>
+      <c r="P95" s="17" t="n"/>
       <c r="Q95" s="9" t="n"/>
       <c r="R95" s="9" t="n"/>
       <c r="S95" s="9" t="n"/>
@@ -3472,7 +3483,7 @@
       <c r="M96" s="9" t="n"/>
       <c r="N96" s="9" t="n"/>
       <c r="O96" s="9" t="n"/>
-      <c r="P96" s="9" t="n"/>
+      <c r="P96" s="17" t="n"/>
       <c r="Q96" s="9" t="n"/>
       <c r="R96" s="9" t="n"/>
       <c r="S96" s="9" t="n"/>
@@ -3493,7 +3504,7 @@
       <c r="M97" s="9" t="n"/>
       <c r="N97" s="9" t="n"/>
       <c r="O97" s="9" t="n"/>
-      <c r="P97" s="9" t="n"/>
+      <c r="P97" s="17" t="n"/>
       <c r="Q97" s="9" t="n"/>
       <c r="R97" s="9" t="n"/>
       <c r="S97" s="9" t="n"/>
@@ -3514,7 +3525,7 @@
       <c r="M98" s="9" t="n"/>
       <c r="N98" s="9" t="n"/>
       <c r="O98" s="9" t="n"/>
-      <c r="P98" s="9" t="n"/>
+      <c r="P98" s="17" t="n"/>
       <c r="Q98" s="9" t="n"/>
       <c r="R98" s="9" t="n"/>
       <c r="S98" s="9" t="n"/>
@@ -3535,7 +3546,7 @@
       <c r="M99" s="9" t="n"/>
       <c r="N99" s="9" t="n"/>
       <c r="O99" s="9" t="n"/>
-      <c r="P99" s="9" t="n"/>
+      <c r="P99" s="17" t="n"/>
       <c r="Q99" s="9" t="n"/>
       <c r="R99" s="9" t="n"/>
       <c r="S99" s="9" t="n"/>
@@ -3556,7 +3567,7 @@
       <c r="M100" s="9" t="n"/>
       <c r="N100" s="9" t="n"/>
       <c r="O100" s="9" t="n"/>
-      <c r="P100" s="9" t="n"/>
+      <c r="P100" s="17" t="n"/>
       <c r="Q100" s="9" t="n"/>
       <c r="R100" s="9" t="n"/>
       <c r="S100" s="9" t="n"/>
@@ -3577,7 +3588,7 @@
       <c r="M101" s="9" t="n"/>
       <c r="N101" s="9" t="n"/>
       <c r="O101" s="9" t="n"/>
-      <c r="P101" s="9" t="n"/>
+      <c r="P101" s="17" t="n"/>
       <c r="Q101" s="9" t="n"/>
       <c r="R101" s="9" t="n"/>
       <c r="S101" s="9" t="n"/>
@@ -3598,7 +3609,7 @@
       <c r="M102" s="9" t="n"/>
       <c r="N102" s="9" t="n"/>
       <c r="O102" s="9" t="n"/>
-      <c r="P102" s="9" t="n"/>
+      <c r="P102" s="17" t="n"/>
       <c r="Q102" s="9" t="n"/>
       <c r="R102" s="9" t="n"/>
       <c r="S102" s="9" t="n"/>
@@ -3619,7 +3630,7 @@
       <c r="M103" s="9" t="n"/>
       <c r="N103" s="9" t="n"/>
       <c r="O103" s="9" t="n"/>
-      <c r="P103" s="9" t="n"/>
+      <c r="P103" s="17" t="n"/>
       <c r="Q103" s="9" t="n"/>
       <c r="R103" s="9" t="n"/>
       <c r="S103" s="9" t="n"/>
@@ -3640,7 +3651,7 @@
       <c r="M104" s="9" t="n"/>
       <c r="N104" s="9" t="n"/>
       <c r="O104" s="9" t="n"/>
-      <c r="P104" s="9" t="n"/>
+      <c r="P104" s="17" t="n"/>
       <c r="Q104" s="9" t="n"/>
       <c r="R104" s="9" t="n"/>
       <c r="S104" s="9" t="n"/>
@@ -3661,7 +3672,7 @@
       <c r="M105" s="9" t="n"/>
       <c r="N105" s="9" t="n"/>
       <c r="O105" s="9" t="n"/>
-      <c r="P105" s="9" t="n"/>
+      <c r="P105" s="17" t="n"/>
       <c r="Q105" s="9" t="n"/>
       <c r="R105" s="9" t="n"/>
       <c r="S105" s="9" t="n"/>
@@ -3682,7 +3693,7 @@
       <c r="M106" s="9" t="n"/>
       <c r="N106" s="9" t="n"/>
       <c r="O106" s="9" t="n"/>
-      <c r="P106" s="9" t="n"/>
+      <c r="P106" s="17" t="n"/>
       <c r="Q106" s="9" t="n"/>
       <c r="R106" s="9" t="n"/>
       <c r="S106" s="9" t="n"/>
@@ -3703,7 +3714,7 @@
       <c r="M107" s="9" t="n"/>
       <c r="N107" s="9" t="n"/>
       <c r="O107" s="9" t="n"/>
-      <c r="P107" s="9" t="n"/>
+      <c r="P107" s="17" t="n"/>
       <c r="Q107" s="9" t="n"/>
       <c r="R107" s="9" t="n"/>
       <c r="S107" s="9" t="n"/>
@@ -3724,7 +3735,7 @@
       <c r="M108" s="9" t="n"/>
       <c r="N108" s="9" t="n"/>
       <c r="O108" s="9" t="n"/>
-      <c r="P108" s="9" t="n"/>
+      <c r="P108" s="17" t="n"/>
       <c r="Q108" s="9" t="n"/>
       <c r="R108" s="9" t="n"/>
       <c r="S108" s="9" t="n"/>
@@ -3745,7 +3756,7 @@
       <c r="M109" s="9" t="n"/>
       <c r="N109" s="9" t="n"/>
       <c r="O109" s="9" t="n"/>
-      <c r="P109" s="9" t="n"/>
+      <c r="P109" s="17" t="n"/>
       <c r="Q109" s="9" t="n"/>
       <c r="R109" s="9" t="n"/>
       <c r="S109" s="9" t="n"/>
@@ -3766,7 +3777,7 @@
       <c r="M110" s="9" t="n"/>
       <c r="N110" s="9" t="n"/>
       <c r="O110" s="9" t="n"/>
-      <c r="P110" s="9" t="n"/>
+      <c r="P110" s="17" t="n"/>
       <c r="Q110" s="9" t="n"/>
       <c r="R110" s="9" t="n"/>
       <c r="S110" s="9" t="n"/>
@@ -3787,7 +3798,7 @@
       <c r="M111" s="9" t="n"/>
       <c r="N111" s="9" t="n"/>
       <c r="O111" s="9" t="n"/>
-      <c r="P111" s="9" t="n"/>
+      <c r="P111" s="17" t="n"/>
       <c r="Q111" s="9" t="n"/>
       <c r="R111" s="9" t="n"/>
       <c r="S111" s="9" t="n"/>
@@ -3808,7 +3819,7 @@
       <c r="M112" s="9" t="n"/>
       <c r="N112" s="9" t="n"/>
       <c r="O112" s="9" t="n"/>
-      <c r="P112" s="9" t="n"/>
+      <c r="P112" s="17" t="n"/>
       <c r="Q112" s="9" t="n"/>
       <c r="R112" s="9" t="n"/>
       <c r="S112" s="9" t="n"/>
@@ -3829,7 +3840,7 @@
       <c r="M113" s="9" t="n"/>
       <c r="N113" s="9" t="n"/>
       <c r="O113" s="9" t="n"/>
-      <c r="P113" s="9" t="n"/>
+      <c r="P113" s="17" t="n"/>
       <c r="Q113" s="9" t="n"/>
       <c r="R113" s="9" t="n"/>
       <c r="S113" s="9" t="n"/>
@@ -3850,7 +3861,7 @@
       <c r="M114" s="9" t="n"/>
       <c r="N114" s="9" t="n"/>
       <c r="O114" s="9" t="n"/>
-      <c r="P114" s="9" t="n"/>
+      <c r="P114" s="17" t="n"/>
       <c r="Q114" s="9" t="n"/>
       <c r="R114" s="9" t="n"/>
       <c r="S114" s="9" t="n"/>
@@ -3871,7 +3882,7 @@
       <c r="M115" s="9" t="n"/>
       <c r="N115" s="9" t="n"/>
       <c r="O115" s="9" t="n"/>
-      <c r="P115" s="9" t="n"/>
+      <c r="P115" s="17" t="n"/>
       <c r="Q115" s="9" t="n"/>
       <c r="R115" s="9" t="n"/>
       <c r="S115" s="9" t="n"/>
@@ -3892,7 +3903,7 @@
       <c r="M116" s="9" t="n"/>
       <c r="N116" s="9" t="n"/>
       <c r="O116" s="9" t="n"/>
-      <c r="P116" s="9" t="n"/>
+      <c r="P116" s="17" t="n"/>
       <c r="Q116" s="9" t="n"/>
       <c r="R116" s="9" t="n"/>
       <c r="S116" s="9" t="n"/>
@@ -3913,7 +3924,7 @@
       <c r="M117" s="9" t="n"/>
       <c r="N117" s="9" t="n"/>
       <c r="O117" s="9" t="n"/>
-      <c r="P117" s="9" t="n"/>
+      <c r="P117" s="17" t="n"/>
       <c r="Q117" s="9" t="n"/>
       <c r="R117" s="9" t="n"/>
       <c r="S117" s="9" t="n"/>
@@ -3934,7 +3945,7 @@
       <c r="M118" s="9" t="n"/>
       <c r="N118" s="9" t="n"/>
       <c r="O118" s="9" t="n"/>
-      <c r="P118" s="9" t="n"/>
+      <c r="P118" s="17" t="n"/>
       <c r="Q118" s="9" t="n"/>
       <c r="R118" s="9" t="n"/>
       <c r="S118" s="9" t="n"/>
@@ -3955,7 +3966,7 @@
       <c r="M119" s="9" t="n"/>
       <c r="N119" s="9" t="n"/>
       <c r="O119" s="9" t="n"/>
-      <c r="P119" s="9" t="n"/>
+      <c r="P119" s="17" t="n"/>
       <c r="Q119" s="9" t="n"/>
       <c r="R119" s="9" t="n"/>
       <c r="S119" s="9" t="n"/>
@@ -3976,7 +3987,7 @@
       <c r="M120" s="9" t="n"/>
       <c r="N120" s="9" t="n"/>
       <c r="O120" s="9" t="n"/>
-      <c r="P120" s="9" t="n"/>
+      <c r="P120" s="17" t="n"/>
       <c r="Q120" s="9" t="n"/>
       <c r="R120" s="9" t="n"/>
       <c r="S120" s="9" t="n"/>
@@ -3997,7 +4008,7 @@
       <c r="M121" s="9" t="n"/>
       <c r="N121" s="9" t="n"/>
       <c r="O121" s="9" t="n"/>
-      <c r="P121" s="9" t="n"/>
+      <c r="P121" s="17" t="n"/>
       <c r="Q121" s="9" t="n"/>
       <c r="R121" s="9" t="n"/>
       <c r="S121" s="9" t="n"/>
@@ -4018,7 +4029,7 @@
       <c r="M122" s="9" t="n"/>
       <c r="N122" s="9" t="n"/>
       <c r="O122" s="9" t="n"/>
-      <c r="P122" s="9" t="n"/>
+      <c r="P122" s="17" t="n"/>
       <c r="Q122" s="9" t="n"/>
       <c r="R122" s="9" t="n"/>
       <c r="S122" s="9" t="n"/>
@@ -4039,7 +4050,7 @@
       <c r="M123" s="9" t="n"/>
       <c r="N123" s="9" t="n"/>
       <c r="O123" s="9" t="n"/>
-      <c r="P123" s="9" t="n"/>
+      <c r="P123" s="17" t="n"/>
       <c r="Q123" s="9" t="n"/>
       <c r="R123" s="9" t="n"/>
       <c r="S123" s="9" t="n"/>
@@ -4060,7 +4071,7 @@
       <c r="M124" s="9" t="n"/>
       <c r="N124" s="9" t="n"/>
       <c r="O124" s="9" t="n"/>
-      <c r="P124" s="9" t="n"/>
+      <c r="P124" s="17" t="n"/>
       <c r="Q124" s="9" t="n"/>
       <c r="R124" s="9" t="n"/>
       <c r="S124" s="9" t="n"/>
@@ -4081,7 +4092,7 @@
       <c r="M125" s="9" t="n"/>
       <c r="N125" s="9" t="n"/>
       <c r="O125" s="9" t="n"/>
-      <c r="P125" s="9" t="n"/>
+      <c r="P125" s="17" t="n"/>
       <c r="Q125" s="9" t="n"/>
       <c r="R125" s="9" t="n"/>
       <c r="S125" s="9" t="n"/>
@@ -4102,7 +4113,7 @@
       <c r="M126" s="9" t="n"/>
       <c r="N126" s="9" t="n"/>
       <c r="O126" s="9" t="n"/>
-      <c r="P126" s="9" t="n"/>
+      <c r="P126" s="17" t="n"/>
       <c r="Q126" s="9" t="n"/>
       <c r="R126" s="9" t="n"/>
       <c r="S126" s="9" t="n"/>
@@ -4123,7 +4134,7 @@
       <c r="M127" s="9" t="n"/>
       <c r="N127" s="9" t="n"/>
       <c r="O127" s="9" t="n"/>
-      <c r="P127" s="9" t="n"/>
+      <c r="P127" s="17" t="n"/>
       <c r="Q127" s="9" t="n"/>
       <c r="R127" s="9" t="n"/>
       <c r="S127" s="9" t="n"/>
@@ -4144,7 +4155,7 @@
       <c r="M128" s="9" t="n"/>
       <c r="N128" s="9" t="n"/>
       <c r="O128" s="9" t="n"/>
-      <c r="P128" s="9" t="n"/>
+      <c r="P128" s="17" t="n"/>
       <c r="Q128" s="9" t="n"/>
       <c r="R128" s="9" t="n"/>
       <c r="S128" s="9" t="n"/>
@@ -4165,7 +4176,7 @@
       <c r="M129" s="9" t="n"/>
       <c r="N129" s="9" t="n"/>
       <c r="O129" s="9" t="n"/>
-      <c r="P129" s="9" t="n"/>
+      <c r="P129" s="17" t="n"/>
       <c r="Q129" s="9" t="n"/>
       <c r="R129" s="9" t="n"/>
       <c r="S129" s="9" t="n"/>
@@ -4186,7 +4197,7 @@
       <c r="M130" s="9" t="n"/>
       <c r="N130" s="9" t="n"/>
       <c r="O130" s="9" t="n"/>
-      <c r="P130" s="9" t="n"/>
+      <c r="P130" s="17" t="n"/>
       <c r="Q130" s="9" t="n"/>
       <c r="R130" s="9" t="n"/>
       <c r="S130" s="9" t="n"/>
@@ -4207,7 +4218,7 @@
       <c r="M131" s="9" t="n"/>
       <c r="N131" s="9" t="n"/>
       <c r="O131" s="9" t="n"/>
-      <c r="P131" s="9" t="n"/>
+      <c r="P131" s="17" t="n"/>
       <c r="Q131" s="9" t="n"/>
       <c r="R131" s="9" t="n"/>
       <c r="S131" s="9" t="n"/>
@@ -4228,7 +4239,7 @@
       <c r="M132" s="9" t="n"/>
       <c r="N132" s="9" t="n"/>
       <c r="O132" s="9" t="n"/>
-      <c r="P132" s="9" t="n"/>
+      <c r="P132" s="17" t="n"/>
       <c r="Q132" s="9" t="n"/>
       <c r="R132" s="9" t="n"/>
       <c r="S132" s="9" t="n"/>
@@ -4249,7 +4260,7 @@
       <c r="M133" s="9" t="n"/>
       <c r="N133" s="9" t="n"/>
       <c r="O133" s="9" t="n"/>
-      <c r="P133" s="9" t="n"/>
+      <c r="P133" s="17" t="n"/>
       <c r="Q133" s="9" t="n"/>
       <c r="R133" s="9" t="n"/>
       <c r="S133" s="9" t="n"/>
@@ -4270,7 +4281,7 @@
       <c r="M134" s="9" t="n"/>
       <c r="N134" s="9" t="n"/>
       <c r="O134" s="9" t="n"/>
-      <c r="P134" s="9" t="n"/>
+      <c r="P134" s="17" t="n"/>
       <c r="Q134" s="9" t="n"/>
       <c r="R134" s="9" t="n"/>
       <c r="S134" s="9" t="n"/>
@@ -4291,7 +4302,7 @@
       <c r="M135" s="9" t="n"/>
       <c r="N135" s="9" t="n"/>
       <c r="O135" s="9" t="n"/>
-      <c r="P135" s="9" t="n"/>
+      <c r="P135" s="17" t="n"/>
       <c r="Q135" s="9" t="n"/>
       <c r="R135" s="9" t="n"/>
       <c r="S135" s="9" t="n"/>
@@ -4312,7 +4323,7 @@
       <c r="M136" s="9" t="n"/>
       <c r="N136" s="9" t="n"/>
       <c r="O136" s="9" t="n"/>
-      <c r="P136" s="9" t="n"/>
+      <c r="P136" s="17" t="n"/>
       <c r="Q136" s="9" t="n"/>
       <c r="R136" s="9" t="n"/>
       <c r="S136" s="9" t="n"/>
@@ -4333,7 +4344,7 @@
       <c r="M137" s="9" t="n"/>
       <c r="N137" s="9" t="n"/>
       <c r="O137" s="9" t="n"/>
-      <c r="P137" s="9" t="n"/>
+      <c r="P137" s="17" t="n"/>
       <c r="Q137" s="9" t="n"/>
       <c r="R137" s="9" t="n"/>
       <c r="S137" s="9" t="n"/>
@@ -4354,7 +4365,7 @@
       <c r="M138" s="9" t="n"/>
       <c r="N138" s="9" t="n"/>
       <c r="O138" s="9" t="n"/>
-      <c r="P138" s="9" t="n"/>
+      <c r="P138" s="17" t="n"/>
       <c r="Q138" s="9" t="n"/>
       <c r="R138" s="9" t="n"/>
       <c r="S138" s="9" t="n"/>
@@ -4375,7 +4386,7 @@
       <c r="M139" s="9" t="n"/>
       <c r="N139" s="9" t="n"/>
       <c r="O139" s="9" t="n"/>
-      <c r="P139" s="9" t="n"/>
+      <c r="P139" s="17" t="n"/>
       <c r="Q139" s="9" t="n"/>
       <c r="R139" s="9" t="n"/>
       <c r="S139" s="9" t="n"/>
@@ -4396,7 +4407,7 @@
       <c r="M140" s="9" t="n"/>
       <c r="N140" s="9" t="n"/>
       <c r="O140" s="9" t="n"/>
-      <c r="P140" s="9" t="n"/>
+      <c r="P140" s="17" t="n"/>
       <c r="Q140" s="9" t="n"/>
       <c r="R140" s="9" t="n"/>
       <c r="S140" s="9" t="n"/>
@@ -4417,7 +4428,7 @@
       <c r="M141" s="9" t="n"/>
       <c r="N141" s="9" t="n"/>
       <c r="O141" s="9" t="n"/>
-      <c r="P141" s="9" t="n"/>
+      <c r="P141" s="17" t="n"/>
       <c r="Q141" s="9" t="n"/>
       <c r="R141" s="9" t="n"/>
       <c r="S141" s="9" t="n"/>
@@ -4438,7 +4449,7 @@
       <c r="M142" s="9" t="n"/>
       <c r="N142" s="9" t="n"/>
       <c r="O142" s="9" t="n"/>
-      <c r="P142" s="9" t="n"/>
+      <c r="P142" s="17" t="n"/>
       <c r="Q142" s="9" t="n"/>
       <c r="R142" s="9" t="n"/>
       <c r="S142" s="9" t="n"/>
@@ -4459,7 +4470,7 @@
       <c r="M143" s="9" t="n"/>
       <c r="N143" s="9" t="n"/>
       <c r="O143" s="9" t="n"/>
-      <c r="P143" s="9" t="n"/>
+      <c r="P143" s="17" t="n"/>
       <c r="Q143" s="9" t="n"/>
       <c r="R143" s="9" t="n"/>
       <c r="S143" s="9" t="n"/>
@@ -4480,7 +4491,7 @@
       <c r="M144" s="9" t="n"/>
       <c r="N144" s="9" t="n"/>
       <c r="O144" s="9" t="n"/>
-      <c r="P144" s="9" t="n"/>
+      <c r="P144" s="17" t="n"/>
       <c r="Q144" s="9" t="n"/>
       <c r="R144" s="9" t="n"/>
       <c r="S144" s="9" t="n"/>
@@ -4501,7 +4512,7 @@
       <c r="M145" s="9" t="n"/>
       <c r="N145" s="9" t="n"/>
       <c r="O145" s="9" t="n"/>
-      <c r="P145" s="9" t="n"/>
+      <c r="P145" s="17" t="n"/>
       <c r="Q145" s="9" t="n"/>
       <c r="R145" s="9" t="n"/>
       <c r="S145" s="9" t="n"/>
@@ -4522,7 +4533,7 @@
       <c r="M146" s="9" t="n"/>
       <c r="N146" s="9" t="n"/>
       <c r="O146" s="9" t="n"/>
-      <c r="P146" s="9" t="n"/>
+      <c r="P146" s="17" t="n"/>
       <c r="Q146" s="9" t="n"/>
       <c r="R146" s="9" t="n"/>
       <c r="S146" s="9" t="n"/>
@@ -4543,7 +4554,7 @@
       <c r="M147" s="9" t="n"/>
       <c r="N147" s="9" t="n"/>
       <c r="O147" s="9" t="n"/>
-      <c r="P147" s="9" t="n"/>
+      <c r="P147" s="17" t="n"/>
       <c r="Q147" s="9" t="n"/>
       <c r="R147" s="9" t="n"/>
       <c r="S147" s="9" t="n"/>
@@ -4564,7 +4575,7 @@
       <c r="M148" s="9" t="n"/>
       <c r="N148" s="9" t="n"/>
       <c r="O148" s="9" t="n"/>
-      <c r="P148" s="9" t="n"/>
+      <c r="P148" s="17" t="n"/>
       <c r="Q148" s="9" t="n"/>
       <c r="R148" s="9" t="n"/>
       <c r="S148" s="9" t="n"/>
@@ -4585,7 +4596,7 @@
       <c r="M149" s="9" t="n"/>
       <c r="N149" s="9" t="n"/>
       <c r="O149" s="9" t="n"/>
-      <c r="P149" s="9" t="n"/>
+      <c r="P149" s="17" t="n"/>
       <c r="Q149" s="9" t="n"/>
       <c r="R149" s="9" t="n"/>
       <c r="S149" s="9" t="n"/>
@@ -4606,7 +4617,7 @@
       <c r="M150" s="9" t="n"/>
       <c r="N150" s="9" t="n"/>
       <c r="O150" s="9" t="n"/>
-      <c r="P150" s="9" t="n"/>
+      <c r="P150" s="17" t="n"/>
       <c r="Q150" s="9" t="n"/>
       <c r="R150" s="9" t="n"/>
       <c r="S150" s="9" t="n"/>
@@ -4627,7 +4638,7 @@
       <c r="M151" s="9" t="n"/>
       <c r="N151" s="9" t="n"/>
       <c r="O151" s="9" t="n"/>
-      <c r="P151" s="9" t="n"/>
+      <c r="P151" s="17" t="n"/>
       <c r="Q151" s="9" t="n"/>
       <c r="R151" s="9" t="n"/>
       <c r="S151" s="9" t="n"/>
@@ -4648,7 +4659,7 @@
       <c r="M152" s="9" t="n"/>
       <c r="N152" s="9" t="n"/>
       <c r="O152" s="9" t="n"/>
-      <c r="P152" s="9" t="n"/>
+      <c r="P152" s="17" t="n"/>
       <c r="Q152" s="9" t="n"/>
       <c r="R152" s="9" t="n"/>
       <c r="S152" s="9" t="n"/>
@@ -4669,7 +4680,7 @@
       <c r="M153" s="9" t="n"/>
       <c r="N153" s="9" t="n"/>
       <c r="O153" s="9" t="n"/>
-      <c r="P153" s="9" t="n"/>
+      <c r="P153" s="17" t="n"/>
       <c r="Q153" s="9" t="n"/>
       <c r="R153" s="9" t="n"/>
       <c r="S153" s="9" t="n"/>
@@ -4690,7 +4701,7 @@
       <c r="M154" s="9" t="n"/>
       <c r="N154" s="9" t="n"/>
       <c r="O154" s="9" t="n"/>
-      <c r="P154" s="9" t="n"/>
+      <c r="P154" s="17" t="n"/>
       <c r="Q154" s="9" t="n"/>
       <c r="R154" s="9" t="n"/>
       <c r="S154" s="9" t="n"/>
@@ -4711,7 +4722,7 @@
       <c r="M155" s="9" t="n"/>
       <c r="N155" s="9" t="n"/>
       <c r="O155" s="9" t="n"/>
-      <c r="P155" s="9" t="n"/>
+      <c r="P155" s="17" t="n"/>
       <c r="Q155" s="9" t="n"/>
       <c r="R155" s="9" t="n"/>
       <c r="S155" s="9" t="n"/>
@@ -4732,7 +4743,7 @@
       <c r="M156" s="9" t="n"/>
       <c r="N156" s="9" t="n"/>
       <c r="O156" s="9" t="n"/>
-      <c r="P156" s="9" t="n"/>
+      <c r="P156" s="17" t="n"/>
       <c r="Q156" s="9" t="n"/>
       <c r="R156" s="9" t="n"/>
       <c r="S156" s="9" t="n"/>
@@ -4753,7 +4764,7 @@
       <c r="M157" s="9" t="n"/>
       <c r="N157" s="9" t="n"/>
       <c r="O157" s="9" t="n"/>
-      <c r="P157" s="9" t="n"/>
+      <c r="P157" s="17" t="n"/>
       <c r="Q157" s="9" t="n"/>
       <c r="R157" s="9" t="n"/>
       <c r="S157" s="9" t="n"/>
@@ -4774,7 +4785,7 @@
       <c r="M158" s="9" t="n"/>
       <c r="N158" s="9" t="n"/>
       <c r="O158" s="9" t="n"/>
-      <c r="P158" s="9" t="n"/>
+      <c r="P158" s="17" t="n"/>
       <c r="Q158" s="9" t="n"/>
       <c r="R158" s="9" t="n"/>
       <c r="S158" s="9" t="n"/>
@@ -4795,7 +4806,7 @@
       <c r="M159" s="9" t="n"/>
       <c r="N159" s="9" t="n"/>
       <c r="O159" s="9" t="n"/>
-      <c r="P159" s="9" t="n"/>
+      <c r="P159" s="17" t="n"/>
       <c r="Q159" s="9" t="n"/>
       <c r="R159" s="9" t="n"/>
       <c r="S159" s="9" t="n"/>
@@ -4816,7 +4827,7 @@
       <c r="M160" s="9" t="n"/>
       <c r="N160" s="9" t="n"/>
       <c r="O160" s="9" t="n"/>
-      <c r="P160" s="9" t="n"/>
+      <c r="P160" s="17" t="n"/>
       <c r="Q160" s="9" t="n"/>
       <c r="R160" s="9" t="n"/>
       <c r="S160" s="9" t="n"/>
@@ -4837,7 +4848,7 @@
       <c r="M161" s="9" t="n"/>
       <c r="N161" s="9" t="n"/>
       <c r="O161" s="9" t="n"/>
-      <c r="P161" s="9" t="n"/>
+      <c r="P161" s="17" t="n"/>
       <c r="Q161" s="9" t="n"/>
       <c r="R161" s="9" t="n"/>
       <c r="S161" s="9" t="n"/>
@@ -4858,7 +4869,7 @@
       <c r="M162" s="9" t="n"/>
       <c r="N162" s="9" t="n"/>
       <c r="O162" s="9" t="n"/>
-      <c r="P162" s="9" t="n"/>
+      <c r="P162" s="17" t="n"/>
       <c r="Q162" s="9" t="n"/>
       <c r="R162" s="9" t="n"/>
       <c r="S162" s="9" t="n"/>
@@ -4879,7 +4890,7 @@
       <c r="M163" s="9" t="n"/>
       <c r="N163" s="9" t="n"/>
       <c r="O163" s="9" t="n"/>
-      <c r="P163" s="9" t="n"/>
+      <c r="P163" s="17" t="n"/>
       <c r="Q163" s="9" t="n"/>
       <c r="R163" s="9" t="n"/>
       <c r="S163" s="9" t="n"/>
@@ -4900,7 +4911,7 @@
       <c r="M164" s="9" t="n"/>
       <c r="N164" s="9" t="n"/>
       <c r="O164" s="9" t="n"/>
-      <c r="P164" s="9" t="n"/>
+      <c r="P164" s="17" t="n"/>
       <c r="Q164" s="9" t="n"/>
       <c r="R164" s="9" t="n"/>
       <c r="S164" s="9" t="n"/>
@@ -4921,7 +4932,7 @@
       <c r="M165" s="9" t="n"/>
       <c r="N165" s="9" t="n"/>
       <c r="O165" s="9" t="n"/>
-      <c r="P165" s="9" t="n"/>
+      <c r="P165" s="17" t="n"/>
       <c r="Q165" s="9" t="n"/>
       <c r="R165" s="9" t="n"/>
       <c r="S165" s="9" t="n"/>
@@ -4942,7 +4953,7 @@
       <c r="M166" s="9" t="n"/>
       <c r="N166" s="9" t="n"/>
       <c r="O166" s="9" t="n"/>
-      <c r="P166" s="9" t="n"/>
+      <c r="P166" s="17" t="n"/>
       <c r="Q166" s="9" t="n"/>
       <c r="R166" s="9" t="n"/>
       <c r="S166" s="9" t="n"/>
@@ -4963,7 +4974,7 @@
       <c r="M167" s="9" t="n"/>
       <c r="N167" s="9" t="n"/>
       <c r="O167" s="9" t="n"/>
-      <c r="P167" s="9" t="n"/>
+      <c r="P167" s="17" t="n"/>
       <c r="Q167" s="9" t="n"/>
       <c r="R167" s="9" t="n"/>
       <c r="S167" s="9" t="n"/>
@@ -4984,7 +4995,7 @@
       <c r="M168" s="9" t="n"/>
       <c r="N168" s="9" t="n"/>
       <c r="O168" s="9" t="n"/>
-      <c r="P168" s="9" t="n"/>
+      <c r="P168" s="17" t="n"/>
       <c r="Q168" s="9" t="n"/>
       <c r="R168" s="9" t="n"/>
       <c r="S168" s="9" t="n"/>
@@ -5005,7 +5016,7 @@
       <c r="M169" s="9" t="n"/>
       <c r="N169" s="9" t="n"/>
       <c r="O169" s="9" t="n"/>
-      <c r="P169" s="9" t="n"/>
+      <c r="P169" s="17" t="n"/>
       <c r="Q169" s="9" t="n"/>
       <c r="R169" s="9" t="n"/>
       <c r="S169" s="9" t="n"/>
@@ -5026,7 +5037,7 @@
       <c r="M170" s="9" t="n"/>
       <c r="N170" s="9" t="n"/>
       <c r="O170" s="9" t="n"/>
-      <c r="P170" s="9" t="n"/>
+      <c r="P170" s="17" t="n"/>
       <c r="Q170" s="9" t="n"/>
       <c r="R170" s="9" t="n"/>
       <c r="S170" s="9" t="n"/>
@@ -5047,7 +5058,7 @@
       <c r="M171" s="9" t="n"/>
       <c r="N171" s="9" t="n"/>
       <c r="O171" s="9" t="n"/>
-      <c r="P171" s="9" t="n"/>
+      <c r="P171" s="17" t="n"/>
       <c r="Q171" s="9" t="n"/>
       <c r="R171" s="9" t="n"/>
       <c r="S171" s="9" t="n"/>
@@ -5068,7 +5079,7 @@
       <c r="M172" s="9" t="n"/>
       <c r="N172" s="9" t="n"/>
       <c r="O172" s="9" t="n"/>
-      <c r="P172" s="9" t="n"/>
+      <c r="P172" s="17" t="n"/>
       <c r="Q172" s="9" t="n"/>
       <c r="R172" s="9" t="n"/>
       <c r="S172" s="9" t="n"/>
@@ -5089,7 +5100,7 @@
       <c r="M173" s="9" t="n"/>
       <c r="N173" s="9" t="n"/>
       <c r="O173" s="9" t="n"/>
-      <c r="P173" s="9" t="n"/>
+      <c r="P173" s="17" t="n"/>
       <c r="Q173" s="9" t="n"/>
       <c r="R173" s="9" t="n"/>
       <c r="S173" s="9" t="n"/>
@@ -5110,7 +5121,7 @@
       <c r="M174" s="9" t="n"/>
       <c r="N174" s="9" t="n"/>
       <c r="O174" s="9" t="n"/>
-      <c r="P174" s="9" t="n"/>
+      <c r="P174" s="17" t="n"/>
       <c r="Q174" s="9" t="n"/>
       <c r="R174" s="9" t="n"/>
       <c r="S174" s="9" t="n"/>
@@ -5131,7 +5142,7 @@
       <c r="M175" s="9" t="n"/>
       <c r="N175" s="9" t="n"/>
       <c r="O175" s="9" t="n"/>
-      <c r="P175" s="9" t="n"/>
+      <c r="P175" s="17" t="n"/>
       <c r="Q175" s="9" t="n"/>
       <c r="R175" s="9" t="n"/>
       <c r="S175" s="9" t="n"/>
@@ -5152,7 +5163,7 @@
       <c r="M176" s="9" t="n"/>
       <c r="N176" s="9" t="n"/>
       <c r="O176" s="9" t="n"/>
-      <c r="P176" s="9" t="n"/>
+      <c r="P176" s="17" t="n"/>
       <c r="Q176" s="9" t="n"/>
       <c r="R176" s="9" t="n"/>
       <c r="S176" s="9" t="n"/>
@@ -5173,7 +5184,7 @@
       <c r="M177" s="9" t="n"/>
       <c r="N177" s="9" t="n"/>
       <c r="O177" s="9" t="n"/>
-      <c r="P177" s="9" t="n"/>
+      <c r="P177" s="17" t="n"/>
       <c r="Q177" s="9" t="n"/>
       <c r="R177" s="9" t="n"/>
       <c r="S177" s="9" t="n"/>
@@ -5194,7 +5205,7 @@
       <c r="M178" s="9" t="n"/>
       <c r="N178" s="9" t="n"/>
       <c r="O178" s="9" t="n"/>
-      <c r="P178" s="9" t="n"/>
+      <c r="P178" s="17" t="n"/>
       <c r="Q178" s="9" t="n"/>
       <c r="R178" s="9" t="n"/>
       <c r="S178" s="9" t="n"/>
@@ -5215,7 +5226,7 @@
       <c r="M179" s="9" t="n"/>
       <c r="N179" s="9" t="n"/>
       <c r="O179" s="9" t="n"/>
-      <c r="P179" s="9" t="n"/>
+      <c r="P179" s="17" t="n"/>
       <c r="Q179" s="9" t="n"/>
       <c r="R179" s="9" t="n"/>
       <c r="S179" s="9" t="n"/>
@@ -5236,7 +5247,7 @@
       <c r="M180" s="9" t="n"/>
       <c r="N180" s="9" t="n"/>
       <c r="O180" s="9" t="n"/>
-      <c r="P180" s="9" t="n"/>
+      <c r="P180" s="17" t="n"/>
       <c r="Q180" s="9" t="n"/>
       <c r="R180" s="9" t="n"/>
       <c r="S180" s="9" t="n"/>
@@ -5257,7 +5268,7 @@
       <c r="M181" s="9" t="n"/>
       <c r="N181" s="9" t="n"/>
       <c r="O181" s="9" t="n"/>
-      <c r="P181" s="9" t="n"/>
+      <c r="P181" s="17" t="n"/>
       <c r="Q181" s="9" t="n"/>
       <c r="R181" s="9" t="n"/>
       <c r="S181" s="9" t="n"/>
@@ -5278,7 +5289,7 @@
       <c r="M182" s="9" t="n"/>
       <c r="N182" s="9" t="n"/>
       <c r="O182" s="9" t="n"/>
-      <c r="P182" s="9" t="n"/>
+      <c r="P182" s="17" t="n"/>
       <c r="Q182" s="9" t="n"/>
       <c r="R182" s="9" t="n"/>
       <c r="S182" s="9" t="n"/>
@@ -5299,7 +5310,7 @@
       <c r="M183" s="9" t="n"/>
       <c r="N183" s="9" t="n"/>
       <c r="O183" s="9" t="n"/>
-      <c r="P183" s="9" t="n"/>
+      <c r="P183" s="17" t="n"/>
       <c r="Q183" s="9" t="n"/>
       <c r="R183" s="9" t="n"/>
       <c r="S183" s="9" t="n"/>
@@ -5320,7 +5331,7 @@
       <c r="M184" s="9" t="n"/>
       <c r="N184" s="9" t="n"/>
       <c r="O184" s="9" t="n"/>
-      <c r="P184" s="9" t="n"/>
+      <c r="P184" s="17" t="n"/>
       <c r="Q184" s="9" t="n"/>
       <c r="R184" s="9" t="n"/>
       <c r="S184" s="9" t="n"/>
@@ -5341,7 +5352,7 @@
       <c r="M185" s="9" t="n"/>
       <c r="N185" s="9" t="n"/>
       <c r="O185" s="9" t="n"/>
-      <c r="P185" s="9" t="n"/>
+      <c r="P185" s="17" t="n"/>
       <c r="Q185" s="9" t="n"/>
       <c r="R185" s="9" t="n"/>
       <c r="S185" s="9" t="n"/>
@@ -5362,7 +5373,7 @@
       <c r="M186" s="9" t="n"/>
       <c r="N186" s="9" t="n"/>
       <c r="O186" s="9" t="n"/>
-      <c r="P186" s="9" t="n"/>
+      <c r="P186" s="17" t="n"/>
       <c r="Q186" s="9" t="n"/>
       <c r="R186" s="9" t="n"/>
       <c r="S186" s="9" t="n"/>
@@ -5383,7 +5394,7 @@
       <c r="M187" s="9" t="n"/>
       <c r="N187" s="9" t="n"/>
       <c r="O187" s="9" t="n"/>
-      <c r="P187" s="9" t="n"/>
+      <c r="P187" s="17" t="n"/>
       <c r="Q187" s="9" t="n"/>
       <c r="R187" s="9" t="n"/>
       <c r="S187" s="9" t="n"/>
@@ -5404,7 +5415,7 @@
       <c r="M188" s="9" t="n"/>
       <c r="N188" s="9" t="n"/>
       <c r="O188" s="9" t="n"/>
-      <c r="P188" s="9" t="n"/>
+      <c r="P188" s="17" t="n"/>
       <c r="Q188" s="9" t="n"/>
       <c r="R188" s="9" t="n"/>
       <c r="S188" s="9" t="n"/>
@@ -5425,7 +5436,7 @@
       <c r="M189" s="9" t="n"/>
       <c r="N189" s="9" t="n"/>
       <c r="O189" s="9" t="n"/>
-      <c r="P189" s="9" t="n"/>
+      <c r="P189" s="17" t="n"/>
       <c r="Q189" s="9" t="n"/>
       <c r="R189" s="9" t="n"/>
       <c r="S189" s="9" t="n"/>
@@ -5446,7 +5457,7 @@
       <c r="M190" s="9" t="n"/>
       <c r="N190" s="9" t="n"/>
       <c r="O190" s="9" t="n"/>
-      <c r="P190" s="9" t="n"/>
+      <c r="P190" s="17" t="n"/>
       <c r="Q190" s="9" t="n"/>
       <c r="R190" s="9" t="n"/>
       <c r="S190" s="9" t="n"/>
@@ -5467,7 +5478,7 @@
       <c r="M191" s="9" t="n"/>
       <c r="N191" s="9" t="n"/>
       <c r="O191" s="9" t="n"/>
-      <c r="P191" s="9" t="n"/>
+      <c r="P191" s="17" t="n"/>
       <c r="Q191" s="9" t="n"/>
       <c r="R191" s="9" t="n"/>
       <c r="S191" s="9" t="n"/>
@@ -5488,7 +5499,7 @@
       <c r="M192" s="9" t="n"/>
       <c r="N192" s="9" t="n"/>
       <c r="O192" s="9" t="n"/>
-      <c r="P192" s="9" t="n"/>
+      <c r="P192" s="17" t="n"/>
       <c r="Q192" s="9" t="n"/>
       <c r="R192" s="9" t="n"/>
       <c r="S192" s="9" t="n"/>
@@ -5509,7 +5520,7 @@
       <c r="M193" s="9" t="n"/>
       <c r="N193" s="9" t="n"/>
       <c r="O193" s="9" t="n"/>
-      <c r="P193" s="9" t="n"/>
+      <c r="P193" s="17" t="n"/>
       <c r="Q193" s="9" t="n"/>
       <c r="R193" s="9" t="n"/>
       <c r="S193" s="9" t="n"/>
@@ -5530,7 +5541,7 @@
       <c r="M194" s="9" t="n"/>
       <c r="N194" s="9" t="n"/>
       <c r="O194" s="9" t="n"/>
-      <c r="P194" s="9" t="n"/>
+      <c r="P194" s="17" t="n"/>
       <c r="Q194" s="9" t="n"/>
       <c r="R194" s="9" t="n"/>
       <c r="S194" s="9" t="n"/>
@@ -5551,7 +5562,7 @@
       <c r="M195" s="9" t="n"/>
       <c r="N195" s="9" t="n"/>
       <c r="O195" s="9" t="n"/>
-      <c r="P195" s="9" t="n"/>
+      <c r="P195" s="17" t="n"/>
       <c r="Q195" s="9" t="n"/>
       <c r="R195" s="9" t="n"/>
       <c r="S195" s="9" t="n"/>
@@ -5572,7 +5583,7 @@
       <c r="M196" s="9" t="n"/>
       <c r="N196" s="9" t="n"/>
       <c r="O196" s="9" t="n"/>
-      <c r="P196" s="9" t="n"/>
+      <c r="P196" s="17" t="n"/>
       <c r="Q196" s="9" t="n"/>
       <c r="R196" s="9" t="n"/>
       <c r="S196" s="9" t="n"/>
@@ -5593,7 +5604,7 @@
       <c r="M197" s="9" t="n"/>
       <c r="N197" s="9" t="n"/>
       <c r="O197" s="9" t="n"/>
-      <c r="P197" s="9" t="n"/>
+      <c r="P197" s="17" t="n"/>
       <c r="Q197" s="9" t="n"/>
       <c r="R197" s="9" t="n"/>
       <c r="S197" s="9" t="n"/>
@@ -5614,7 +5625,7 @@
       <c r="M198" s="9" t="n"/>
       <c r="N198" s="9" t="n"/>
       <c r="O198" s="9" t="n"/>
-      <c r="P198" s="9" t="n"/>
+      <c r="P198" s="17" t="n"/>
       <c r="Q198" s="9" t="n"/>
       <c r="R198" s="9" t="n"/>
       <c r="S198" s="9" t="n"/>
@@ -5635,7 +5646,7 @@
       <c r="M199" s="9" t="n"/>
       <c r="N199" s="9" t="n"/>
       <c r="O199" s="9" t="n"/>
-      <c r="P199" s="9" t="n"/>
+      <c r="P199" s="17" t="n"/>
       <c r="Q199" s="9" t="n"/>
       <c r="R199" s="9" t="n"/>
       <c r="S199" s="9" t="n"/>
@@ -5656,7 +5667,7 @@
       <c r="M200" s="9" t="n"/>
       <c r="N200" s="9" t="n"/>
       <c r="O200" s="9" t="n"/>
-      <c r="P200" s="9" t="n"/>
+      <c r="P200" s="17" t="n"/>
       <c r="Q200" s="9" t="n"/>
       <c r="R200" s="9" t="n"/>
       <c r="S200" s="9" t="n"/>
@@ -5677,7 +5688,7 @@
       <c r="M201" s="9" t="n"/>
       <c r="N201" s="9" t="n"/>
       <c r="O201" s="9" t="n"/>
-      <c r="P201" s="9" t="n"/>
+      <c r="P201" s="17" t="n"/>
       <c r="Q201" s="9" t="n"/>
       <c r="R201" s="9" t="n"/>
       <c r="S201" s="9" t="n"/>
@@ -5698,7 +5709,7 @@
       <c r="M202" s="9" t="n"/>
       <c r="N202" s="9" t="n"/>
       <c r="O202" s="9" t="n"/>
-      <c r="P202" s="9" t="n"/>
+      <c r="P202" s="17" t="n"/>
       <c r="Q202" s="9" t="n"/>
       <c r="R202" s="9" t="n"/>
       <c r="S202" s="9" t="n"/>
@@ -5719,7 +5730,7 @@
       <c r="M203" s="9" t="n"/>
       <c r="N203" s="9" t="n"/>
       <c r="O203" s="9" t="n"/>
-      <c r="P203" s="9" t="n"/>
+      <c r="P203" s="17" t="n"/>
       <c r="Q203" s="9" t="n"/>
       <c r="R203" s="9" t="n"/>
       <c r="S203" s="9" t="n"/>
@@ -5740,7 +5751,7 @@
       <c r="M204" s="9" t="n"/>
       <c r="N204" s="9" t="n"/>
       <c r="O204" s="9" t="n"/>
-      <c r="P204" s="9" t="n"/>
+      <c r="P204" s="17" t="n"/>
       <c r="Q204" s="9" t="n"/>
       <c r="R204" s="9" t="n"/>
       <c r="S204" s="9" t="n"/>
@@ -5761,7 +5772,7 @@
       <c r="M205" s="9" t="n"/>
       <c r="N205" s="9" t="n"/>
       <c r="O205" s="9" t="n"/>
-      <c r="P205" s="9" t="n"/>
+      <c r="P205" s="17" t="n"/>
       <c r="Q205" s="9" t="n"/>
       <c r="R205" s="9" t="n"/>
       <c r="S205" s="9" t="n"/>
@@ -5782,7 +5793,7 @@
       <c r="M206" s="9" t="n"/>
       <c r="N206" s="9" t="n"/>
       <c r="O206" s="9" t="n"/>
-      <c r="P206" s="9" t="n"/>
+      <c r="P206" s="17" t="n"/>
       <c r="Q206" s="9" t="n"/>
       <c r="R206" s="9" t="n"/>
       <c r="S206" s="9" t="n"/>
@@ -5803,7 +5814,7 @@
       <c r="M207" s="9" t="n"/>
       <c r="N207" s="9" t="n"/>
       <c r="O207" s="9" t="n"/>
-      <c r="P207" s="9" t="n"/>
+      <c r="P207" s="17" t="n"/>
       <c r="Q207" s="9" t="n"/>
       <c r="R207" s="9" t="n"/>
       <c r="S207" s="9" t="n"/>
@@ -5824,7 +5835,7 @@
       <c r="M208" s="9" t="n"/>
       <c r="N208" s="9" t="n"/>
       <c r="O208" s="9" t="n"/>
-      <c r="P208" s="9" t="n"/>
+      <c r="P208" s="17" t="n"/>
       <c r="Q208" s="9" t="n"/>
       <c r="R208" s="9" t="n"/>
       <c r="S208" s="9" t="n"/>
@@ -5845,7 +5856,7 @@
       <c r="M209" s="9" t="n"/>
       <c r="N209" s="9" t="n"/>
       <c r="O209" s="9" t="n"/>
-      <c r="P209" s="9" t="n"/>
+      <c r="P209" s="17" t="n"/>
       <c r="Q209" s="9" t="n"/>
       <c r="R209" s="9" t="n"/>
       <c r="S209" s="9" t="n"/>
@@ -5866,7 +5877,7 @@
       <c r="M210" s="9" t="n"/>
       <c r="N210" s="9" t="n"/>
       <c r="O210" s="9" t="n"/>
-      <c r="P210" s="9" t="n"/>
+      <c r="P210" s="17" t="n"/>
       <c r="Q210" s="9" t="n"/>
       <c r="R210" s="9" t="n"/>
       <c r="S210" s="9" t="n"/>
@@ -5887,7 +5898,7 @@
       <c r="M211" s="9" t="n"/>
       <c r="N211" s="9" t="n"/>
       <c r="O211" s="9" t="n"/>
-      <c r="P211" s="9" t="n"/>
+      <c r="P211" s="17" t="n"/>
       <c r="Q211" s="9" t="n"/>
       <c r="R211" s="9" t="n"/>
       <c r="S211" s="9" t="n"/>
@@ -5908,7 +5919,7 @@
       <c r="M212" s="9" t="n"/>
       <c r="N212" s="9" t="n"/>
       <c r="O212" s="9" t="n"/>
-      <c r="P212" s="9" t="n"/>
+      <c r="P212" s="17" t="n"/>
       <c r="Q212" s="9" t="n"/>
       <c r="R212" s="9" t="n"/>
       <c r="S212" s="9" t="n"/>
@@ -5929,7 +5940,7 @@
       <c r="M213" s="9" t="n"/>
       <c r="N213" s="9" t="n"/>
       <c r="O213" s="9" t="n"/>
-      <c r="P213" s="9" t="n"/>
+      <c r="P213" s="17" t="n"/>
       <c r="Q213" s="9" t="n"/>
       <c r="R213" s="9" t="n"/>
       <c r="S213" s="9" t="n"/>
@@ -5950,7 +5961,7 @@
       <c r="M214" s="9" t="n"/>
       <c r="N214" s="9" t="n"/>
       <c r="O214" s="9" t="n"/>
-      <c r="P214" s="9" t="n"/>
+      <c r="P214" s="17" t="n"/>
       <c r="Q214" s="9" t="n"/>
       <c r="R214" s="9" t="n"/>
       <c r="S214" s="9" t="n"/>
@@ -5971,7 +5982,7 @@
       <c r="M215" s="9" t="n"/>
       <c r="N215" s="9" t="n"/>
       <c r="O215" s="9" t="n"/>
-      <c r="P215" s="9" t="n"/>
+      <c r="P215" s="17" t="n"/>
       <c r="Q215" s="9" t="n"/>
       <c r="R215" s="9" t="n"/>
       <c r="S215" s="9" t="n"/>
@@ -5992,7 +6003,7 @@
       <c r="M216" s="9" t="n"/>
       <c r="N216" s="9" t="n"/>
       <c r="O216" s="9" t="n"/>
-      <c r="P216" s="9" t="n"/>
+      <c r="P216" s="17" t="n"/>
       <c r="Q216" s="9" t="n"/>
       <c r="R216" s="9" t="n"/>
       <c r="S216" s="9" t="n"/>
@@ -6013,7 +6024,7 @@
       <c r="M217" s="9" t="n"/>
       <c r="N217" s="9" t="n"/>
       <c r="O217" s="9" t="n"/>
-      <c r="P217" s="9" t="n"/>
+      <c r="P217" s="17" t="n"/>
       <c r="Q217" s="9" t="n"/>
       <c r="R217" s="9" t="n"/>
       <c r="S217" s="9" t="n"/>
@@ -6034,7 +6045,7 @@
       <c r="M218" s="9" t="n"/>
       <c r="N218" s="9" t="n"/>
       <c r="O218" s="9" t="n"/>
-      <c r="P218" s="9" t="n"/>
+      <c r="P218" s="17" t="n"/>
       <c r="Q218" s="9" t="n"/>
       <c r="R218" s="9" t="n"/>
       <c r="S218" s="9" t="n"/>
@@ -6055,7 +6066,7 @@
       <c r="M219" s="9" t="n"/>
       <c r="N219" s="9" t="n"/>
       <c r="O219" s="9" t="n"/>
-      <c r="P219" s="9" t="n"/>
+      <c r="P219" s="17" t="n"/>
       <c r="Q219" s="9" t="n"/>
       <c r="R219" s="9" t="n"/>
       <c r="S219" s="9" t="n"/>
@@ -6076,7 +6087,7 @@
       <c r="M220" s="9" t="n"/>
       <c r="N220" s="9" t="n"/>
       <c r="O220" s="9" t="n"/>
-      <c r="P220" s="9" t="n"/>
+      <c r="P220" s="17" t="n"/>
       <c r="Q220" s="9" t="n"/>
       <c r="R220" s="9" t="n"/>
       <c r="S220" s="9" t="n"/>
@@ -6097,7 +6108,7 @@
       <c r="M221" s="9" t="n"/>
       <c r="N221" s="9" t="n"/>
       <c r="O221" s="9" t="n"/>
-      <c r="P221" s="9" t="n"/>
+      <c r="P221" s="17" t="n"/>
       <c r="Q221" s="9" t="n"/>
       <c r="R221" s="9" t="n"/>
       <c r="S221" s="9" t="n"/>
@@ -6118,7 +6129,7 @@
       <c r="M222" s="9" t="n"/>
       <c r="N222" s="9" t="n"/>
       <c r="O222" s="9" t="n"/>
-      <c r="P222" s="9" t="n"/>
+      <c r="P222" s="17" t="n"/>
       <c r="Q222" s="9" t="n"/>
       <c r="R222" s="9" t="n"/>
       <c r="S222" s="9" t="n"/>
@@ -6139,7 +6150,7 @@
       <c r="M223" s="9" t="n"/>
       <c r="N223" s="9" t="n"/>
       <c r="O223" s="9" t="n"/>
-      <c r="P223" s="9" t="n"/>
+      <c r="P223" s="17" t="n"/>
       <c r="Q223" s="9" t="n"/>
       <c r="R223" s="9" t="n"/>
       <c r="S223" s="9" t="n"/>
@@ -6160,7 +6171,7 @@
       <c r="M224" s="9" t="n"/>
       <c r="N224" s="9" t="n"/>
       <c r="O224" s="9" t="n"/>
-      <c r="P224" s="9" t="n"/>
+      <c r="P224" s="17" t="n"/>
       <c r="Q224" s="9" t="n"/>
       <c r="R224" s="9" t="n"/>
       <c r="S224" s="9" t="n"/>
@@ -6181,7 +6192,7 @@
       <c r="M225" s="9" t="n"/>
       <c r="N225" s="9" t="n"/>
       <c r="O225" s="9" t="n"/>
-      <c r="P225" s="9" t="n"/>
+      <c r="P225" s="17" t="n"/>
       <c r="Q225" s="9" t="n"/>
       <c r="R225" s="9" t="n"/>
       <c r="S225" s="9" t="n"/>
@@ -6202,7 +6213,7 @@
       <c r="M226" s="9" t="n"/>
       <c r="N226" s="9" t="n"/>
       <c r="O226" s="9" t="n"/>
-      <c r="P226" s="9" t="n"/>
+      <c r="P226" s="17" t="n"/>
       <c r="Q226" s="9" t="n"/>
       <c r="R226" s="9" t="n"/>
       <c r="S226" s="9" t="n"/>
@@ -6223,7 +6234,7 @@
       <c r="M227" s="9" t="n"/>
       <c r="N227" s="9" t="n"/>
       <c r="O227" s="9" t="n"/>
-      <c r="P227" s="9" t="n"/>
+      <c r="P227" s="17" t="n"/>
       <c r="Q227" s="9" t="n"/>
       <c r="R227" s="9" t="n"/>
       <c r="S227" s="9" t="n"/>
@@ -6244,7 +6255,7 @@
       <c r="M228" s="9" t="n"/>
       <c r="N228" s="9" t="n"/>
       <c r="O228" s="9" t="n"/>
-      <c r="P228" s="9" t="n"/>
+      <c r="P228" s="17" t="n"/>
       <c r="Q228" s="9" t="n"/>
       <c r="R228" s="9" t="n"/>
       <c r="S228" s="9" t="n"/>
@@ -6265,7 +6276,7 @@
       <c r="M229" s="9" t="n"/>
       <c r="N229" s="9" t="n"/>
       <c r="O229" s="9" t="n"/>
-      <c r="P229" s="9" t="n"/>
+      <c r="P229" s="17" t="n"/>
       <c r="Q229" s="9" t="n"/>
       <c r="R229" s="9" t="n"/>
       <c r="S229" s="9" t="n"/>
@@ -6286,7 +6297,7 @@
       <c r="M230" s="9" t="n"/>
       <c r="N230" s="9" t="n"/>
       <c r="O230" s="9" t="n"/>
-      <c r="P230" s="9" t="n"/>
+      <c r="P230" s="17" t="n"/>
       <c r="Q230" s="9" t="n"/>
       <c r="R230" s="9" t="n"/>
       <c r="S230" s="9" t="n"/>
@@ -6307,7 +6318,7 @@
       <c r="M231" s="9" t="n"/>
       <c r="N231" s="9" t="n"/>
       <c r="O231" s="9" t="n"/>
-      <c r="P231" s="9" t="n"/>
+      <c r="P231" s="17" t="n"/>
       <c r="Q231" s="9" t="n"/>
       <c r="R231" s="9" t="n"/>
       <c r="S231" s="9" t="n"/>
@@ -6328,7 +6339,7 @@
       <c r="M232" s="9" t="n"/>
       <c r="N232" s="9" t="n"/>
       <c r="O232" s="9" t="n"/>
-      <c r="P232" s="9" t="n"/>
+      <c r="P232" s="17" t="n"/>
       <c r="Q232" s="9" t="n"/>
       <c r="R232" s="9" t="n"/>
       <c r="S232" s="9" t="n"/>
@@ -6349,7 +6360,7 @@
       <c r="M233" s="9" t="n"/>
       <c r="N233" s="9" t="n"/>
       <c r="O233" s="9" t="n"/>
-      <c r="P233" s="9" t="n"/>
+      <c r="P233" s="17" t="n"/>
       <c r="Q233" s="9" t="n"/>
       <c r="R233" s="9" t="n"/>
       <c r="S233" s="9" t="n"/>
@@ -6370,7 +6381,7 @@
       <c r="M234" s="9" t="n"/>
       <c r="N234" s="9" t="n"/>
       <c r="O234" s="9" t="n"/>
-      <c r="P234" s="9" t="n"/>
+      <c r="P234" s="17" t="n"/>
       <c r="Q234" s="9" t="n"/>
       <c r="R234" s="9" t="n"/>
       <c r="S234" s="9" t="n"/>
@@ -6391,7 +6402,7 @@
       <c r="M235" s="9" t="n"/>
       <c r="N235" s="9" t="n"/>
       <c r="O235" s="9" t="n"/>
-      <c r="P235" s="9" t="n"/>
+      <c r="P235" s="17" t="n"/>
       <c r="Q235" s="9" t="n"/>
       <c r="R235" s="9" t="n"/>
       <c r="S235" s="9" t="n"/>
@@ -6412,7 +6423,7 @@
       <c r="M236" s="9" t="n"/>
       <c r="N236" s="9" t="n"/>
       <c r="O236" s="9" t="n"/>
-      <c r="P236" s="9" t="n"/>
+      <c r="P236" s="17" t="n"/>
       <c r="Q236" s="9" t="n"/>
       <c r="R236" s="9" t="n"/>
       <c r="S236" s="9" t="n"/>
@@ -6433,7 +6444,7 @@
       <c r="M237" s="9" t="n"/>
       <c r="N237" s="9" t="n"/>
       <c r="O237" s="9" t="n"/>
-      <c r="P237" s="9" t="n"/>
+      <c r="P237" s="17" t="n"/>
       <c r="Q237" s="9" t="n"/>
       <c r="R237" s="9" t="n"/>
       <c r="S237" s="9" t="n"/>
@@ -6454,7 +6465,7 @@
       <c r="M238" s="9" t="n"/>
       <c r="N238" s="9" t="n"/>
       <c r="O238" s="9" t="n"/>
-      <c r="P238" s="9" t="n"/>
+      <c r="P238" s="17" t="n"/>
       <c r="Q238" s="9" t="n"/>
       <c r="R238" s="9" t="n"/>
       <c r="S238" s="9" t="n"/>
@@ -6475,7 +6486,7 @@
       <c r="M239" s="9" t="n"/>
       <c r="N239" s="9" t="n"/>
       <c r="O239" s="9" t="n"/>
-      <c r="P239" s="9" t="n"/>
+      <c r="P239" s="17" t="n"/>
       <c r="Q239" s="9" t="n"/>
       <c r="R239" s="9" t="n"/>
       <c r="S239" s="9" t="n"/>
@@ -6496,7 +6507,7 @@
       <c r="M240" s="9" t="n"/>
       <c r="N240" s="9" t="n"/>
       <c r="O240" s="9" t="n"/>
-      <c r="P240" s="9" t="n"/>
+      <c r="P240" s="17" t="n"/>
       <c r="Q240" s="9" t="n"/>
       <c r="R240" s="9" t="n"/>
       <c r="S240" s="9" t="n"/>
@@ -6517,7 +6528,7 @@
       <c r="M241" s="9" t="n"/>
       <c r="N241" s="9" t="n"/>
       <c r="O241" s="9" t="n"/>
-      <c r="P241" s="9" t="n"/>
+      <c r="P241" s="17" t="n"/>
       <c r="Q241" s="9" t="n"/>
       <c r="R241" s="9" t="n"/>
       <c r="S241" s="9" t="n"/>
@@ -6538,7 +6549,7 @@
       <c r="M242" s="9" t="n"/>
       <c r="N242" s="9" t="n"/>
       <c r="O242" s="9" t="n"/>
-      <c r="P242" s="9" t="n"/>
+      <c r="P242" s="17" t="n"/>
       <c r="Q242" s="9" t="n"/>
       <c r="R242" s="9" t="n"/>
       <c r="S242" s="9" t="n"/>
@@ -6559,7 +6570,7 @@
       <c r="M243" s="9" t="n"/>
       <c r="N243" s="9" t="n"/>
       <c r="O243" s="9" t="n"/>
-      <c r="P243" s="9" t="n"/>
+      <c r="P243" s="17" t="n"/>
       <c r="Q243" s="9" t="n"/>
       <c r="R243" s="9" t="n"/>
       <c r="S243" s="9" t="n"/>
@@ -6580,7 +6591,7 @@
       <c r="M244" s="9" t="n"/>
       <c r="N244" s="9" t="n"/>
       <c r="O244" s="9" t="n"/>
-      <c r="P244" s="9" t="n"/>
+      <c r="P244" s="17" t="n"/>
       <c r="Q244" s="9" t="n"/>
       <c r="R244" s="9" t="n"/>
       <c r="S244" s="9" t="n"/>
@@ -6601,7 +6612,7 @@
       <c r="M245" s="9" t="n"/>
       <c r="N245" s="9" t="n"/>
       <c r="O245" s="9" t="n"/>
-      <c r="P245" s="9" t="n"/>
+      <c r="P245" s="17" t="n"/>
       <c r="Q245" s="9" t="n"/>
       <c r="R245" s="9" t="n"/>
       <c r="S245" s="9" t="n"/>
@@ -6622,7 +6633,7 @@
       <c r="M246" s="9" t="n"/>
       <c r="N246" s="9" t="n"/>
       <c r="O246" s="9" t="n"/>
-      <c r="P246" s="9" t="n"/>
+      <c r="P246" s="17" t="n"/>
       <c r="Q246" s="9" t="n"/>
       <c r="R246" s="9" t="n"/>
       <c r="S246" s="9" t="n"/>
@@ -6643,7 +6654,7 @@
       <c r="M247" s="9" t="n"/>
       <c r="N247" s="9" t="n"/>
       <c r="O247" s="9" t="n"/>
-      <c r="P247" s="9" t="n"/>
+      <c r="P247" s="17" t="n"/>
       <c r="Q247" s="9" t="n"/>
       <c r="R247" s="9" t="n"/>
       <c r="S247" s="9" t="n"/>
@@ -6664,7 +6675,7 @@
       <c r="M248" s="9" t="n"/>
       <c r="N248" s="9" t="n"/>
       <c r="O248" s="9" t="n"/>
-      <c r="P248" s="9" t="n"/>
+      <c r="P248" s="17" t="n"/>
       <c r="Q248" s="9" t="n"/>
       <c r="R248" s="9" t="n"/>
       <c r="S248" s="9" t="n"/>
@@ -6685,7 +6696,7 @@
       <c r="M249" s="9" t="n"/>
       <c r="N249" s="9" t="n"/>
       <c r="O249" s="9" t="n"/>
-      <c r="P249" s="9" t="n"/>
+      <c r="P249" s="17" t="n"/>
       <c r="Q249" s="9" t="n"/>
       <c r="R249" s="9" t="n"/>
       <c r="S249" s="9" t="n"/>
@@ -6706,7 +6717,7 @@
       <c r="M250" s="9" t="n"/>
       <c r="N250" s="9" t="n"/>
       <c r="O250" s="9" t="n"/>
-      <c r="P250" s="9" t="n"/>
+      <c r="P250" s="17" t="n"/>
       <c r="Q250" s="9" t="n"/>
       <c r="R250" s="9" t="n"/>
       <c r="S250" s="9" t="n"/>
@@ -6727,7 +6738,7 @@
       <c r="M251" s="9" t="n"/>
       <c r="N251" s="9" t="n"/>
       <c r="O251" s="9" t="n"/>
-      <c r="P251" s="9" t="n"/>
+      <c r="P251" s="17" t="n"/>
       <c r="Q251" s="9" t="n"/>
       <c r="R251" s="9" t="n"/>
       <c r="S251" s="9" t="n"/>
@@ -6748,7 +6759,7 @@
       <c r="M252" s="9" t="n"/>
       <c r="N252" s="9" t="n"/>
       <c r="O252" s="9" t="n"/>
-      <c r="P252" s="9" t="n"/>
+      <c r="P252" s="17" t="n"/>
       <c r="Q252" s="9" t="n"/>
       <c r="R252" s="9" t="n"/>
       <c r="S252" s="9" t="n"/>
@@ -6769,7 +6780,7 @@
       <c r="M253" s="9" t="n"/>
       <c r="N253" s="9" t="n"/>
       <c r="O253" s="9" t="n"/>
-      <c r="P253" s="9" t="n"/>
+      <c r="P253" s="17" t="n"/>
       <c r="Q253" s="9" t="n"/>
       <c r="R253" s="9" t="n"/>
       <c r="S253" s="9" t="n"/>
@@ -6790,7 +6801,7 @@
       <c r="M254" s="9" t="n"/>
       <c r="N254" s="9" t="n"/>
       <c r="O254" s="9" t="n"/>
-      <c r="P254" s="9" t="n"/>
+      <c r="P254" s="17" t="n"/>
       <c r="Q254" s="9" t="n"/>
       <c r="R254" s="9" t="n"/>
       <c r="S254" s="9" t="n"/>
@@ -6811,7 +6822,7 @@
       <c r="M255" s="9" t="n"/>
       <c r="N255" s="9" t="n"/>
       <c r="O255" s="9" t="n"/>
-      <c r="P255" s="9" t="n"/>
+      <c r="P255" s="17" t="n"/>
       <c r="Q255" s="9" t="n"/>
       <c r="R255" s="9" t="n"/>
       <c r="S255" s="9" t="n"/>
@@ -6832,7 +6843,7 @@
       <c r="M256" s="9" t="n"/>
       <c r="N256" s="9" t="n"/>
       <c r="O256" s="9" t="n"/>
-      <c r="P256" s="9" t="n"/>
+      <c r="P256" s="17" t="n"/>
       <c r="Q256" s="9" t="n"/>
       <c r="R256" s="9" t="n"/>
       <c r="S256" s="9" t="n"/>
@@ -6853,7 +6864,7 @@
       <c r="M257" s="9" t="n"/>
       <c r="N257" s="9" t="n"/>
       <c r="O257" s="9" t="n"/>
-      <c r="P257" s="9" t="n"/>
+      <c r="P257" s="17" t="n"/>
       <c r="Q257" s="9" t="n"/>
       <c r="R257" s="9" t="n"/>
       <c r="S257" s="9" t="n"/>
@@ -6874,7 +6885,7 @@
       <c r="M258" s="9" t="n"/>
       <c r="N258" s="9" t="n"/>
       <c r="O258" s="9" t="n"/>
-      <c r="P258" s="9" t="n"/>
+      <c r="P258" s="17" t="n"/>
       <c r="Q258" s="9" t="n"/>
       <c r="R258" s="9" t="n"/>
       <c r="S258" s="9" t="n"/>
@@ -6895,7 +6906,7 @@
       <c r="M259" s="9" t="n"/>
       <c r="N259" s="9" t="n"/>
       <c r="O259" s="9" t="n"/>
-      <c r="P259" s="9" t="n"/>
+      <c r="P259" s="17" t="n"/>
       <c r="Q259" s="9" t="n"/>
       <c r="R259" s="9" t="n"/>
       <c r="S259" s="9" t="n"/>
@@ -6916,7 +6927,7 @@
       <c r="M260" s="9" t="n"/>
       <c r="N260" s="9" t="n"/>
       <c r="O260" s="9" t="n"/>
-      <c r="P260" s="9" t="n"/>
+      <c r="P260" s="17" t="n"/>
       <c r="Q260" s="9" t="n"/>
       <c r="R260" s="9" t="n"/>
       <c r="S260" s="9" t="n"/>
@@ -6937,7 +6948,7 @@
       <c r="M261" s="9" t="n"/>
       <c r="N261" s="9" t="n"/>
       <c r="O261" s="9" t="n"/>
-      <c r="P261" s="9" t="n"/>
+      <c r="P261" s="17" t="n"/>
       <c r="Q261" s="9" t="n"/>
       <c r="R261" s="9" t="n"/>
       <c r="S261" s="9" t="n"/>
@@ -6958,7 +6969,7 @@
       <c r="M262" s="9" t="n"/>
       <c r="N262" s="9" t="n"/>
       <c r="O262" s="9" t="n"/>
-      <c r="P262" s="9" t="n"/>
+      <c r="P262" s="17" t="n"/>
       <c r="Q262" s="9" t="n"/>
       <c r="R262" s="9" t="n"/>
       <c r="S262" s="9" t="n"/>
@@ -6979,7 +6990,7 @@
       <c r="M263" s="9" t="n"/>
       <c r="N263" s="9" t="n"/>
       <c r="O263" s="9" t="n"/>
-      <c r="P263" s="9" t="n"/>
+      <c r="P263" s="17" t="n"/>
       <c r="Q263" s="9" t="n"/>
       <c r="R263" s="9" t="n"/>
       <c r="S263" s="9" t="n"/>
@@ -7000,7 +7011,7 @@
       <c r="M264" s="9" t="n"/>
       <c r="N264" s="9" t="n"/>
       <c r="O264" s="9" t="n"/>
-      <c r="P264" s="9" t="n"/>
+      <c r="P264" s="17" t="n"/>
       <c r="Q264" s="9" t="n"/>
       <c r="R264" s="9" t="n"/>
       <c r="S264" s="9" t="n"/>
@@ -7021,7 +7032,7 @@
       <c r="M265" s="9" t="n"/>
       <c r="N265" s="9" t="n"/>
       <c r="O265" s="9" t="n"/>
-      <c r="P265" s="9" t="n"/>
+      <c r="P265" s="17" t="n"/>
       <c r="Q265" s="9" t="n"/>
       <c r="R265" s="9" t="n"/>
       <c r="S265" s="9" t="n"/>
@@ -7042,7 +7053,7 @@
       <c r="M266" s="9" t="n"/>
       <c r="N266" s="9" t="n"/>
       <c r="O266" s="9" t="n"/>
-      <c r="P266" s="9" t="n"/>
+      <c r="P266" s="17" t="n"/>
       <c r="Q266" s="9" t="n"/>
       <c r="R266" s="9" t="n"/>
       <c r="S266" s="9" t="n"/>
@@ -7063,7 +7074,7 @@
       <c r="M267" s="9" t="n"/>
       <c r="N267" s="9" t="n"/>
       <c r="O267" s="9" t="n"/>
-      <c r="P267" s="9" t="n"/>
+      <c r="P267" s="17" t="n"/>
       <c r="Q267" s="9" t="n"/>
       <c r="R267" s="9" t="n"/>
       <c r="S267" s="9" t="n"/>
@@ -7084,7 +7095,7 @@
       <c r="M268" s="9" t="n"/>
       <c r="N268" s="9" t="n"/>
       <c r="O268" s="9" t="n"/>
-      <c r="P268" s="9" t="n"/>
+      <c r="P268" s="17" t="n"/>
       <c r="Q268" s="9" t="n"/>
       <c r="R268" s="9" t="n"/>
       <c r="S268" s="9" t="n"/>
@@ -7105,7 +7116,7 @@
       <c r="M269" s="9" t="n"/>
       <c r="N269" s="9" t="n"/>
       <c r="O269" s="9" t="n"/>
-      <c r="P269" s="9" t="n"/>
+      <c r="P269" s="17" t="n"/>
       <c r="Q269" s="9" t="n"/>
       <c r="R269" s="9" t="n"/>
       <c r="S269" s="9" t="n"/>
@@ -7126,7 +7137,7 @@
       <c r="M270" s="9" t="n"/>
       <c r="N270" s="9" t="n"/>
       <c r="O270" s="9" t="n"/>
-      <c r="P270" s="9" t="n"/>
+      <c r="P270" s="17" t="n"/>
       <c r="Q270" s="9" t="n"/>
       <c r="R270" s="9" t="n"/>
       <c r="S270" s="9" t="n"/>
@@ -7147,7 +7158,7 @@
       <c r="M271" s="9" t="n"/>
       <c r="N271" s="9" t="n"/>
       <c r="O271" s="9" t="n"/>
-      <c r="P271" s="9" t="n"/>
+      <c r="P271" s="17" t="n"/>
       <c r="Q271" s="9" t="n"/>
       <c r="R271" s="9" t="n"/>
       <c r="S271" s="9" t="n"/>
@@ -7168,7 +7179,7 @@
       <c r="M272" s="9" t="n"/>
       <c r="N272" s="9" t="n"/>
       <c r="O272" s="9" t="n"/>
-      <c r="P272" s="9" t="n"/>
+      <c r="P272" s="17" t="n"/>
       <c r="Q272" s="9" t="n"/>
       <c r="R272" s="9" t="n"/>
       <c r="S272" s="9" t="n"/>
@@ -7189,7 +7200,7 @@
       <c r="M273" s="9" t="n"/>
       <c r="N273" s="9" t="n"/>
       <c r="O273" s="9" t="n"/>
-      <c r="P273" s="9" t="n"/>
+      <c r="P273" s="17" t="n"/>
       <c r="Q273" s="9" t="n"/>
       <c r="R273" s="9" t="n"/>
       <c r="S273" s="9" t="n"/>
@@ -7210,7 +7221,7 @@
       <c r="M274" s="9" t="n"/>
       <c r="N274" s="9" t="n"/>
       <c r="O274" s="9" t="n"/>
-      <c r="P274" s="9" t="n"/>
+      <c r="P274" s="17" t="n"/>
       <c r="Q274" s="9" t="n"/>
       <c r="R274" s="9" t="n"/>
       <c r="S274" s="9" t="n"/>
@@ -7231,7 +7242,7 @@
       <c r="M275" s="9" t="n"/>
       <c r="N275" s="9" t="n"/>
       <c r="O275" s="9" t="n"/>
-      <c r="P275" s="9" t="n"/>
+      <c r="P275" s="17" t="n"/>
       <c r="Q275" s="9" t="n"/>
       <c r="R275" s="9" t="n"/>
       <c r="S275" s="9" t="n"/>
@@ -7252,7 +7263,7 @@
       <c r="M276" s="9" t="n"/>
       <c r="N276" s="9" t="n"/>
       <c r="O276" s="9" t="n"/>
-      <c r="P276" s="9" t="n"/>
+      <c r="P276" s="17" t="n"/>
       <c r="Q276" s="9" t="n"/>
       <c r="R276" s="9" t="n"/>
       <c r="S276" s="9" t="n"/>
@@ -7273,7 +7284,7 @@
       <c r="M277" s="9" t="n"/>
       <c r="N277" s="9" t="n"/>
       <c r="O277" s="9" t="n"/>
-      <c r="P277" s="9" t="n"/>
+      <c r="P277" s="17" t="n"/>
       <c r="Q277" s="9" t="n"/>
       <c r="R277" s="9" t="n"/>
       <c r="S277" s="9" t="n"/>
@@ -7294,7 +7305,7 @@
       <c r="M278" s="9" t="n"/>
       <c r="N278" s="9" t="n"/>
       <c r="O278" s="9" t="n"/>
-      <c r="P278" s="9" t="n"/>
+      <c r="P278" s="17" t="n"/>
       <c r="Q278" s="9" t="n"/>
       <c r="R278" s="9" t="n"/>
       <c r="S278" s="9" t="n"/>
@@ -7315,7 +7326,7 @@
       <c r="M279" s="9" t="n"/>
       <c r="N279" s="9" t="n"/>
       <c r="O279" s="9" t="n"/>
-      <c r="P279" s="9" t="n"/>
+      <c r="P279" s="17" t="n"/>
       <c r="Q279" s="9" t="n"/>
       <c r="R279" s="9" t="n"/>
       <c r="S279" s="9" t="n"/>
@@ -7336,7 +7347,7 @@
       <c r="M280" s="9" t="n"/>
       <c r="N280" s="9" t="n"/>
       <c r="O280" s="9" t="n"/>
-      <c r="P280" s="9" t="n"/>
+      <c r="P280" s="17" t="n"/>
       <c r="Q280" s="9" t="n"/>
       <c r="R280" s="9" t="n"/>
       <c r="S280" s="9" t="n"/>
@@ -7357,7 +7368,7 @@
       <c r="M281" s="9" t="n"/>
       <c r="N281" s="9" t="n"/>
       <c r="O281" s="9" t="n"/>
-      <c r="P281" s="9" t="n"/>
+      <c r="P281" s="17" t="n"/>
       <c r="Q281" s="9" t="n"/>
       <c r="R281" s="9" t="n"/>
       <c r="S281" s="9" t="n"/>
@@ -7378,7 +7389,7 @@
       <c r="M282" s="9" t="n"/>
       <c r="N282" s="9" t="n"/>
       <c r="O282" s="9" t="n"/>
-      <c r="P282" s="9" t="n"/>
+      <c r="P282" s="17" t="n"/>
       <c r="Q282" s="9" t="n"/>
       <c r="R282" s="9" t="n"/>
       <c r="S282" s="9" t="n"/>
@@ -7399,7 +7410,7 @@
       <c r="M283" s="9" t="n"/>
       <c r="N283" s="9" t="n"/>
       <c r="O283" s="9" t="n"/>
-      <c r="P283" s="9" t="n"/>
+      <c r="P283" s="17" t="n"/>
       <c r="Q283" s="9" t="n"/>
       <c r="R283" s="9" t="n"/>
       <c r="S283" s="9" t="n"/>
@@ -7420,7 +7431,7 @@
       <c r="M284" s="9" t="n"/>
       <c r="N284" s="9" t="n"/>
       <c r="O284" s="9" t="n"/>
-      <c r="P284" s="9" t="n"/>
+      <c r="P284" s="17" t="n"/>
       <c r="Q284" s="9" t="n"/>
       <c r="R284" s="9" t="n"/>
       <c r="S284" s="9" t="n"/>
@@ -7441,7 +7452,7 @@
       <c r="M285" s="9" t="n"/>
       <c r="N285" s="9" t="n"/>
       <c r="O285" s="9" t="n"/>
-      <c r="P285" s="9" t="n"/>
+      <c r="P285" s="17" t="n"/>
       <c r="Q285" s="9" t="n"/>
       <c r="R285" s="9" t="n"/>
       <c r="S285" s="9" t="n"/>
@@ -7462,7 +7473,7 @@
       <c r="M286" s="9" t="n"/>
       <c r="N286" s="9" t="n"/>
       <c r="O286" s="9" t="n"/>
-      <c r="P286" s="9" t="n"/>
+      <c r="P286" s="17" t="n"/>
       <c r="Q286" s="9" t="n"/>
       <c r="R286" s="9" t="n"/>
       <c r="S286" s="9" t="n"/>
@@ -7483,7 +7494,7 @@
       <c r="M287" s="9" t="n"/>
       <c r="N287" s="9" t="n"/>
       <c r="O287" s="9" t="n"/>
-      <c r="P287" s="9" t="n"/>
+      <c r="P287" s="17" t="n"/>
       <c r="Q287" s="9" t="n"/>
       <c r="R287" s="9" t="n"/>
       <c r="S287" s="9" t="n"/>
@@ -7504,7 +7515,7 @@
       <c r="M288" s="9" t="n"/>
       <c r="N288" s="9" t="n"/>
       <c r="O288" s="9" t="n"/>
-      <c r="P288" s="9" t="n"/>
+      <c r="P288" s="17" t="n"/>
       <c r="Q288" s="9" t="n"/>
       <c r="R288" s="9" t="n"/>
       <c r="S288" s="9" t="n"/>
@@ -7525,7 +7536,7 @@
       <c r="M289" s="9" t="n"/>
       <c r="N289" s="9" t="n"/>
       <c r="O289" s="9" t="n"/>
-      <c r="P289" s="9" t="n"/>
+      <c r="P289" s="17" t="n"/>
       <c r="Q289" s="9" t="n"/>
       <c r="R289" s="9" t="n"/>
       <c r="S289" s="9" t="n"/>
@@ -7546,7 +7557,7 @@
       <c r="M290" s="9" t="n"/>
       <c r="N290" s="9" t="n"/>
       <c r="O290" s="9" t="n"/>
-      <c r="P290" s="9" t="n"/>
+      <c r="P290" s="17" t="n"/>
       <c r="Q290" s="9" t="n"/>
       <c r="R290" s="9" t="n"/>
       <c r="S290" s="9" t="n"/>
@@ -7567,7 +7578,7 @@
       <c r="M291" s="9" t="n"/>
       <c r="N291" s="9" t="n"/>
       <c r="O291" s="9" t="n"/>
-      <c r="P291" s="9" t="n"/>
+      <c r="P291" s="17" t="n"/>
       <c r="Q291" s="9" t="n"/>
       <c r="R291" s="9" t="n"/>
       <c r="S291" s="9" t="n"/>
@@ -7588,7 +7599,7 @@
       <c r="M292" s="9" t="n"/>
       <c r="N292" s="9" t="n"/>
       <c r="O292" s="9" t="n"/>
-      <c r="P292" s="9" t="n"/>
+      <c r="P292" s="17" t="n"/>
       <c r="Q292" s="9" t="n"/>
       <c r="R292" s="9" t="n"/>
       <c r="S292" s="9" t="n"/>
@@ -7609,7 +7620,7 @@
       <c r="M293" s="9" t="n"/>
       <c r="N293" s="9" t="n"/>
       <c r="O293" s="9" t="n"/>
-      <c r="P293" s="9" t="n"/>
+      <c r="P293" s="17" t="n"/>
       <c r="Q293" s="9" t="n"/>
       <c r="R293" s="9" t="n"/>
       <c r="S293" s="9" t="n"/>
@@ -7630,7 +7641,7 @@
       <c r="M294" s="9" t="n"/>
       <c r="N294" s="9" t="n"/>
       <c r="O294" s="9" t="n"/>
-      <c r="P294" s="9" t="n"/>
+      <c r="P294" s="17" t="n"/>
       <c r="Q294" s="9" t="n"/>
       <c r="R294" s="9" t="n"/>
       <c r="S294" s="9" t="n"/>
@@ -7651,7 +7662,7 @@
       <c r="M295" s="9" t="n"/>
       <c r="N295" s="9" t="n"/>
       <c r="O295" s="9" t="n"/>
-      <c r="P295" s="9" t="n"/>
+      <c r="P295" s="17" t="n"/>
       <c r="Q295" s="9" t="n"/>
       <c r="R295" s="9" t="n"/>
       <c r="S295" s="9" t="n"/>
@@ -7672,7 +7683,7 @@
       <c r="M296" s="9" t="n"/>
       <c r="N296" s="9" t="n"/>
       <c r="O296" s="9" t="n"/>
-      <c r="P296" s="9" t="n"/>
+      <c r="P296" s="17" t="n"/>
       <c r="Q296" s="9" t="n"/>
       <c r="R296" s="9" t="n"/>
       <c r="S296" s="9" t="n"/>
@@ -7693,7 +7704,7 @@
       <c r="M297" s="9" t="n"/>
       <c r="N297" s="9" t="n"/>
       <c r="O297" s="9" t="n"/>
-      <c r="P297" s="9" t="n"/>
+      <c r="P297" s="17" t="n"/>
       <c r="Q297" s="9" t="n"/>
       <c r="R297" s="9" t="n"/>
       <c r="S297" s="9" t="n"/>
@@ -7714,7 +7725,7 @@
       <c r="M298" s="9" t="n"/>
       <c r="N298" s="9" t="n"/>
       <c r="O298" s="9" t="n"/>
-      <c r="P298" s="9" t="n"/>
+      <c r="P298" s="17" t="n"/>
       <c r="Q298" s="9" t="n"/>
       <c r="R298" s="9" t="n"/>
       <c r="S298" s="9" t="n"/>
@@ -7735,7 +7746,7 @@
       <c r="M299" s="9" t="n"/>
       <c r="N299" s="9" t="n"/>
       <c r="O299" s="9" t="n"/>
-      <c r="P299" s="9" t="n"/>
+      <c r="P299" s="17" t="n"/>
       <c r="Q299" s="9" t="n"/>
       <c r="R299" s="9" t="n"/>
       <c r="S299" s="9" t="n"/>
@@ -7756,7 +7767,7 @@
       <c r="M300" s="9" t="n"/>
       <c r="N300" s="9" t="n"/>
       <c r="O300" s="9" t="n"/>
-      <c r="P300" s="9" t="n"/>
+      <c r="P300" s="17" t="n"/>
       <c r="Q300" s="9" t="n"/>
       <c r="R300" s="9" t="n"/>
       <c r="S300" s="9" t="n"/>
@@ -7777,7 +7788,7 @@
       <c r="M301" s="9" t="n"/>
       <c r="N301" s="9" t="n"/>
       <c r="O301" s="9" t="n"/>
-      <c r="P301" s="9" t="n"/>
+      <c r="P301" s="17" t="n"/>
       <c r="Q301" s="9" t="n"/>
       <c r="R301" s="9" t="n"/>
       <c r="S301" s="9" t="n"/>
@@ -7798,7 +7809,7 @@
       <c r="M302" s="9" t="n"/>
       <c r="N302" s="9" t="n"/>
       <c r="O302" s="9" t="n"/>
-      <c r="P302" s="9" t="n"/>
+      <c r="P302" s="17" t="n"/>
       <c r="Q302" s="9" t="n"/>
       <c r="R302" s="9" t="n"/>
       <c r="S302" s="9" t="n"/>
@@ -7819,7 +7830,7 @@
       <c r="M303" s="9" t="n"/>
       <c r="N303" s="9" t="n"/>
       <c r="O303" s="9" t="n"/>
-      <c r="P303" s="9" t="n"/>
+      <c r="P303" s="17" t="n"/>
       <c r="Q303" s="9" t="n"/>
       <c r="R303" s="9" t="n"/>
       <c r="S303" s="9" t="n"/>
@@ -7840,7 +7851,7 @@
       <c r="M304" s="9" t="n"/>
       <c r="N304" s="9" t="n"/>
       <c r="O304" s="9" t="n"/>
-      <c r="P304" s="9" t="n"/>
+      <c r="P304" s="17" t="n"/>
       <c r="Q304" s="9" t="n"/>
       <c r="R304" s="9" t="n"/>
       <c r="S304" s="9" t="n"/>
@@ -7861,7 +7872,7 @@
       <c r="M305" s="9" t="n"/>
       <c r="N305" s="9" t="n"/>
       <c r="O305" s="9" t="n"/>
-      <c r="P305" s="9" t="n"/>
+      <c r="P305" s="17" t="n"/>
       <c r="Q305" s="9" t="n"/>
       <c r="R305" s="9" t="n"/>
       <c r="S305" s="9" t="n"/>
@@ -7882,7 +7893,7 @@
       <c r="M306" s="9" t="n"/>
       <c r="N306" s="9" t="n"/>
       <c r="O306" s="9" t="n"/>
-      <c r="P306" s="9" t="n"/>
+      <c r="P306" s="17" t="n"/>
       <c r="Q306" s="9" t="n"/>
       <c r="R306" s="9" t="n"/>
       <c r="S306" s="9" t="n"/>
@@ -7903,7 +7914,7 @@
       <c r="M307" s="9" t="n"/>
       <c r="N307" s="9" t="n"/>
       <c r="O307" s="9" t="n"/>
-      <c r="P307" s="9" t="n"/>
+      <c r="P307" s="17" t="n"/>
       <c r="Q307" s="9" t="n"/>
       <c r="R307" s="9" t="n"/>
       <c r="S307" s="9" t="n"/>
@@ -7924,7 +7935,7 @@
       <c r="M308" s="9" t="n"/>
       <c r="N308" s="9" t="n"/>
       <c r="O308" s="9" t="n"/>
-      <c r="P308" s="9" t="n"/>
+      <c r="P308" s="17" t="n"/>
       <c r="Q308" s="9" t="n"/>
       <c r="R308" s="9" t="n"/>
       <c r="S308" s="9" t="n"/>
@@ -7945,7 +7956,7 @@
       <c r="M309" s="9" t="n"/>
       <c r="N309" s="9" t="n"/>
       <c r="O309" s="9" t="n"/>
-      <c r="P309" s="9" t="n"/>
+      <c r="P309" s="17" t="n"/>
       <c r="Q309" s="9" t="n"/>
       <c r="R309" s="9" t="n"/>
       <c r="S309" s="9" t="n"/>
@@ -7966,7 +7977,7 @@
       <c r="M310" s="9" t="n"/>
       <c r="N310" s="9" t="n"/>
       <c r="O310" s="9" t="n"/>
-      <c r="P310" s="9" t="n"/>
+      <c r="P310" s="17" t="n"/>
       <c r="Q310" s="9" t="n"/>
       <c r="R310" s="9" t="n"/>
       <c r="S310" s="9" t="n"/>
@@ -7987,7 +7998,7 @@
       <c r="M311" s="9" t="n"/>
       <c r="N311" s="9" t="n"/>
       <c r="O311" s="9" t="n"/>
-      <c r="P311" s="9" t="n"/>
+      <c r="P311" s="17" t="n"/>
       <c r="Q311" s="9" t="n"/>
       <c r="R311" s="9" t="n"/>
       <c r="S311" s="9" t="n"/>
@@ -8008,7 +8019,7 @@
       <c r="M312" s="9" t="n"/>
       <c r="N312" s="9" t="n"/>
       <c r="O312" s="9" t="n"/>
-      <c r="P312" s="9" t="n"/>
+      <c r="P312" s="17" t="n"/>
       <c r="Q312" s="9" t="n"/>
       <c r="R312" s="9" t="n"/>
       <c r="S312" s="9" t="n"/>
@@ -8029,7 +8040,7 @@
       <c r="M313" s="9" t="n"/>
       <c r="N313" s="9" t="n"/>
       <c r="O313" s="9" t="n"/>
-      <c r="P313" s="9" t="n"/>
+      <c r="P313" s="17" t="n"/>
       <c r="Q313" s="9" t="n"/>
       <c r="R313" s="9" t="n"/>
       <c r="S313" s="9" t="n"/>
@@ -8050,7 +8061,7 @@
       <c r="M314" s="9" t="n"/>
       <c r="N314" s="9" t="n"/>
       <c r="O314" s="9" t="n"/>
-      <c r="P314" s="9" t="n"/>
+      <c r="P314" s="17" t="n"/>
       <c r="Q314" s="9" t="n"/>
       <c r="R314" s="9" t="n"/>
       <c r="S314" s="9" t="n"/>
@@ -8071,7 +8082,7 @@
       <c r="M315" s="9" t="n"/>
       <c r="N315" s="9" t="n"/>
       <c r="O315" s="9" t="n"/>
-      <c r="P315" s="9" t="n"/>
+      <c r="P315" s="17" t="n"/>
       <c r="Q315" s="9" t="n"/>
       <c r="R315" s="9" t="n"/>
       <c r="S315" s="9" t="n"/>
@@ -8092,7 +8103,7 @@
       <c r="M316" s="9" t="n"/>
       <c r="N316" s="9" t="n"/>
       <c r="O316" s="9" t="n"/>
-      <c r="P316" s="9" t="n"/>
+      <c r="P316" s="17" t="n"/>
       <c r="Q316" s="9" t="n"/>
       <c r="R316" s="9" t="n"/>
       <c r="S316" s="9" t="n"/>
@@ -8113,7 +8124,7 @@
       <c r="M317" s="9" t="n"/>
       <c r="N317" s="9" t="n"/>
       <c r="O317" s="9" t="n"/>
-      <c r="P317" s="9" t="n"/>
+      <c r="P317" s="17" t="n"/>
       <c r="Q317" s="9" t="n"/>
       <c r="R317" s="9" t="n"/>
       <c r="S317" s="9" t="n"/>
@@ -8134,7 +8145,7 @@
       <c r="M318" s="9" t="n"/>
       <c r="N318" s="9" t="n"/>
       <c r="O318" s="9" t="n"/>
-      <c r="P318" s="9" t="n"/>
+      <c r="P318" s="17" t="n"/>
       <c r="Q318" s="9" t="n"/>
       <c r="R318" s="9" t="n"/>
       <c r="S318" s="9" t="n"/>
@@ -8155,7 +8166,7 @@
       <c r="M319" s="9" t="n"/>
       <c r="N319" s="9" t="n"/>
       <c r="O319" s="9" t="n"/>
-      <c r="P319" s="9" t="n"/>
+      <c r="P319" s="17" t="n"/>
       <c r="Q319" s="9" t="n"/>
       <c r="R319" s="9" t="n"/>
       <c r="S319" s="9" t="n"/>
@@ -8176,7 +8187,7 @@
       <c r="M320" s="9" t="n"/>
       <c r="N320" s="9" t="n"/>
       <c r="O320" s="9" t="n"/>
-      <c r="P320" s="9" t="n"/>
+      <c r="P320" s="17" t="n"/>
       <c r="Q320" s="9" t="n"/>
       <c r="R320" s="9" t="n"/>
       <c r="S320" s="9" t="n"/>
@@ -8197,7 +8208,7 @@
       <c r="M321" s="9" t="n"/>
       <c r="N321" s="9" t="n"/>
       <c r="O321" s="9" t="n"/>
-      <c r="P321" s="9" t="n"/>
+      <c r="P321" s="17" t="n"/>
       <c r="Q321" s="9" t="n"/>
       <c r="R321" s="9" t="n"/>
       <c r="S321" s="9" t="n"/>
@@ -8218,7 +8229,7 @@
       <c r="M322" s="9" t="n"/>
       <c r="N322" s="9" t="n"/>
       <c r="O322" s="9" t="n"/>
-      <c r="P322" s="9" t="n"/>
+      <c r="P322" s="17" t="n"/>
       <c r="Q322" s="9" t="n"/>
       <c r="R322" s="9" t="n"/>
       <c r="S322" s="9" t="n"/>
@@ -8239,7 +8250,7 @@
       <c r="M323" s="9" t="n"/>
       <c r="N323" s="9" t="n"/>
       <c r="O323" s="9" t="n"/>
-      <c r="P323" s="9" t="n"/>
+      <c r="P323" s="17" t="n"/>
       <c r="Q323" s="9" t="n"/>
       <c r="R323" s="9" t="n"/>
       <c r="S323" s="9" t="n"/>
@@ -8260,7 +8271,7 @@
       <c r="M324" s="9" t="n"/>
       <c r="N324" s="9" t="n"/>
       <c r="O324" s="9" t="n"/>
-      <c r="P324" s="9" t="n"/>
+      <c r="P324" s="17" t="n"/>
       <c r="Q324" s="9" t="n"/>
       <c r="R324" s="9" t="n"/>
       <c r="S324" s="9" t="n"/>
@@ -8281,7 +8292,7 @@
       <c r="M325" s="9" t="n"/>
       <c r="N325" s="9" t="n"/>
       <c r="O325" s="9" t="n"/>
-      <c r="P325" s="9" t="n"/>
+      <c r="P325" s="17" t="n"/>
       <c r="Q325" s="9" t="n"/>
       <c r="R325" s="9" t="n"/>
       <c r="S325" s="9" t="n"/>
@@ -8302,7 +8313,7 @@
       <c r="M326" s="9" t="n"/>
       <c r="N326" s="9" t="n"/>
       <c r="O326" s="9" t="n"/>
-      <c r="P326" s="9" t="n"/>
+      <c r="P326" s="17" t="n"/>
       <c r="Q326" s="9" t="n"/>
       <c r="R326" s="9" t="n"/>
       <c r="S326" s="9" t="n"/>
@@ -8323,7 +8334,7 @@
       <c r="M327" s="9" t="n"/>
       <c r="N327" s="9" t="n"/>
       <c r="O327" s="9" t="n"/>
-      <c r="P327" s="9" t="n"/>
+      <c r="P327" s="17" t="n"/>
       <c r="Q327" s="9" t="n"/>
       <c r="R327" s="9" t="n"/>
       <c r="S327" s="9" t="n"/>
@@ -8344,7 +8355,7 @@
       <c r="M328" s="9" t="n"/>
       <c r="N328" s="9" t="n"/>
       <c r="O328" s="9" t="n"/>
-      <c r="P328" s="9" t="n"/>
+      <c r="P328" s="17" t="n"/>
       <c r="Q328" s="9" t="n"/>
       <c r="R328" s="9" t="n"/>
       <c r="S328" s="9" t="n"/>
@@ -8365,7 +8376,7 @@
       <c r="M329" s="9" t="n"/>
       <c r="N329" s="9" t="n"/>
       <c r="O329" s="9" t="n"/>
-      <c r="P329" s="9" t="n"/>
+      <c r="P329" s="17" t="n"/>
       <c r="Q329" s="9" t="n"/>
       <c r="R329" s="9" t="n"/>
       <c r="S329" s="9" t="n"/>
@@ -8386,7 +8397,7 @@
       <c r="M330" s="9" t="n"/>
       <c r="N330" s="9" t="n"/>
       <c r="O330" s="9" t="n"/>
-      <c r="P330" s="9" t="n"/>
+      <c r="P330" s="17" t="n"/>
       <c r="Q330" s="9" t="n"/>
       <c r="R330" s="9" t="n"/>
       <c r="S330" s="9" t="n"/>
@@ -8407,7 +8418,7 @@
       <c r="M331" s="9" t="n"/>
       <c r="N331" s="9" t="n"/>
       <c r="O331" s="9" t="n"/>
-      <c r="P331" s="9" t="n"/>
+      <c r="P331" s="17" t="n"/>
       <c r="Q331" s="9" t="n"/>
       <c r="R331" s="9" t="n"/>
       <c r="S331" s="9" t="n"/>
@@ -8428,7 +8439,7 @@
       <c r="M332" s="9" t="n"/>
       <c r="N332" s="9" t="n"/>
       <c r="O332" s="9" t="n"/>
-      <c r="P332" s="9" t="n"/>
+      <c r="P332" s="17" t="n"/>
       <c r="Q332" s="9" t="n"/>
       <c r="R332" s="9" t="n"/>
       <c r="S332" s="9" t="n"/>
@@ -8449,7 +8460,7 @@
       <c r="M333" s="9" t="n"/>
       <c r="N333" s="9" t="n"/>
       <c r="O333" s="9" t="n"/>
-      <c r="P333" s="9" t="n"/>
+      <c r="P333" s="17" t="n"/>
       <c r="Q333" s="9" t="n"/>
       <c r="R333" s="9" t="n"/>
       <c r="S333" s="9" t="n"/>
@@ -8470,7 +8481,7 @@
       <c r="M334" s="9" t="n"/>
       <c r="N334" s="9" t="n"/>
       <c r="O334" s="9" t="n"/>
-      <c r="P334" s="9" t="n"/>
+      <c r="P334" s="17" t="n"/>
       <c r="Q334" s="9" t="n"/>
       <c r="R334" s="9" t="n"/>
       <c r="S334" s="9" t="n"/>
@@ -8491,7 +8502,7 @@
       <c r="M335" s="9" t="n"/>
       <c r="N335" s="9" t="n"/>
       <c r="O335" s="9" t="n"/>
-      <c r="P335" s="9" t="n"/>
+      <c r="P335" s="17" t="n"/>
       <c r="Q335" s="9" t="n"/>
       <c r="R335" s="9" t="n"/>
       <c r="S335" s="9" t="n"/>
@@ -8512,7 +8523,7 @@
       <c r="M336" s="9" t="n"/>
       <c r="N336" s="9" t="n"/>
       <c r="O336" s="9" t="n"/>
-      <c r="P336" s="9" t="n"/>
+      <c r="P336" s="17" t="n"/>
       <c r="Q336" s="9" t="n"/>
       <c r="R336" s="9" t="n"/>
       <c r="S336" s="9" t="n"/>
@@ -8533,7 +8544,7 @@
       <c r="M337" s="9" t="n"/>
       <c r="N337" s="9" t="n"/>
       <c r="O337" s="9" t="n"/>
-      <c r="P337" s="9" t="n"/>
+      <c r="P337" s="17" t="n"/>
       <c r="Q337" s="9" t="n"/>
       <c r="R337" s="9" t="n"/>
       <c r="S337" s="9" t="n"/>
@@ -8554,7 +8565,7 @@
       <c r="M338" s="9" t="n"/>
       <c r="N338" s="9" t="n"/>
       <c r="O338" s="9" t="n"/>
-      <c r="P338" s="9" t="n"/>
+      <c r="P338" s="17" t="n"/>
       <c r="Q338" s="9" t="n"/>
       <c r="R338" s="9" t="n"/>
       <c r="S338" s="9" t="n"/>
@@ -8575,7 +8586,7 @@
       <c r="M339" s="9" t="n"/>
       <c r="N339" s="9" t="n"/>
       <c r="O339" s="9" t="n"/>
-      <c r="P339" s="9" t="n"/>
+      <c r="P339" s="17" t="n"/>
       <c r="Q339" s="9" t="n"/>
       <c r="R339" s="9" t="n"/>
       <c r="S339" s="9" t="n"/>
@@ -8596,7 +8607,7 @@
       <c r="M340" s="9" t="n"/>
       <c r="N340" s="9" t="n"/>
       <c r="O340" s="9" t="n"/>
-      <c r="P340" s="9" t="n"/>
+      <c r="P340" s="17" t="n"/>
       <c r="Q340" s="9" t="n"/>
       <c r="R340" s="9" t="n"/>
       <c r="S340" s="9" t="n"/>
@@ -8617,7 +8628,7 @@
       <c r="M341" s="9" t="n"/>
       <c r="N341" s="9" t="n"/>
       <c r="O341" s="9" t="n"/>
-      <c r="P341" s="9" t="n"/>
+      <c r="P341" s="17" t="n"/>
       <c r="Q341" s="9" t="n"/>
       <c r="R341" s="9" t="n"/>
       <c r="S341" s="9" t="n"/>
@@ -8638,7 +8649,7 @@
       <c r="M342" s="9" t="n"/>
       <c r="N342" s="9" t="n"/>
       <c r="O342" s="9" t="n"/>
-      <c r="P342" s="9" t="n"/>
+      <c r="P342" s="17" t="n"/>
       <c r="Q342" s="9" t="n"/>
       <c r="R342" s="9" t="n"/>
       <c r="S342" s="9" t="n"/>
@@ -8659,7 +8670,7 @@
       <c r="M343" s="9" t="n"/>
       <c r="N343" s="9" t="n"/>
       <c r="O343" s="9" t="n"/>
-      <c r="P343" s="9" t="n"/>
+      <c r="P343" s="17" t="n"/>
       <c r="Q343" s="9" t="n"/>
       <c r="R343" s="9" t="n"/>
       <c r="S343" s="9" t="n"/>
@@ -8680,7 +8691,7 @@
       <c r="M344" s="9" t="n"/>
       <c r="N344" s="9" t="n"/>
       <c r="O344" s="9" t="n"/>
-      <c r="P344" s="9" t="n"/>
+      <c r="P344" s="17" t="n"/>
       <c r="Q344" s="9" t="n"/>
       <c r="R344" s="9" t="n"/>
       <c r="S344" s="9" t="n"/>
@@ -8701,7 +8712,7 @@
       <c r="M345" s="9" t="n"/>
       <c r="N345" s="9" t="n"/>
       <c r="O345" s="9" t="n"/>
-      <c r="P345" s="9" t="n"/>
+      <c r="P345" s="17" t="n"/>
       <c r="Q345" s="9" t="n"/>
       <c r="R345" s="9" t="n"/>
       <c r="S345" s="9" t="n"/>
@@ -8722,7 +8733,7 @@
       <c r="M346" s="9" t="n"/>
       <c r="N346" s="9" t="n"/>
       <c r="O346" s="9" t="n"/>
-      <c r="P346" s="9" t="n"/>
+      <c r="P346" s="17" t="n"/>
       <c r="Q346" s="9" t="n"/>
       <c r="R346" s="9" t="n"/>
       <c r="S346" s="9" t="n"/>
@@ -8743,7 +8754,7 @@
       <c r="M347" s="9" t="n"/>
       <c r="N347" s="9" t="n"/>
       <c r="O347" s="9" t="n"/>
-      <c r="P347" s="9" t="n"/>
+      <c r="P347" s="17" t="n"/>
       <c r="Q347" s="9" t="n"/>
       <c r="R347" s="9" t="n"/>
       <c r="S347" s="9" t="n"/>
@@ -8764,7 +8775,7 @@
       <c r="M348" s="9" t="n"/>
       <c r="N348" s="9" t="n"/>
       <c r="O348" s="9" t="n"/>
-      <c r="P348" s="9" t="n"/>
+      <c r="P348" s="17" t="n"/>
       <c r="Q348" s="9" t="n"/>
       <c r="R348" s="9" t="n"/>
       <c r="S348" s="9" t="n"/>
@@ -8785,7 +8796,7 @@
       <c r="M349" s="9" t="n"/>
       <c r="N349" s="9" t="n"/>
       <c r="O349" s="9" t="n"/>
-      <c r="P349" s="9" t="n"/>
+      <c r="P349" s="17" t="n"/>
       <c r="Q349" s="9" t="n"/>
       <c r="R349" s="9" t="n"/>
       <c r="S349" s="9" t="n"/>
@@ -8806,7 +8817,7 @@
       <c r="M350" s="9" t="n"/>
       <c r="N350" s="9" t="n"/>
       <c r="O350" s="9" t="n"/>
-      <c r="P350" s="9" t="n"/>
+      <c r="P350" s="17" t="n"/>
       <c r="Q350" s="9" t="n"/>
       <c r="R350" s="9" t="n"/>
       <c r="S350" s="9" t="n"/>
@@ -8827,7 +8838,7 @@
       <c r="M351" s="9" t="n"/>
       <c r="N351" s="9" t="n"/>
       <c r="O351" s="9" t="n"/>
-      <c r="P351" s="9" t="n"/>
+      <c r="P351" s="17" t="n"/>
       <c r="Q351" s="9" t="n"/>
       <c r="R351" s="9" t="n"/>
       <c r="S351" s="9" t="n"/>
@@ -8848,7 +8859,7 @@
       <c r="M352" s="9" t="n"/>
       <c r="N352" s="9" t="n"/>
       <c r="O352" s="9" t="n"/>
-      <c r="P352" s="9" t="n"/>
+      <c r="P352" s="17" t="n"/>
       <c r="Q352" s="9" t="n"/>
       <c r="R352" s="9" t="n"/>
       <c r="S352" s="9" t="n"/>
@@ -8869,7 +8880,7 @@
       <c r="M353" s="9" t="n"/>
       <c r="N353" s="9" t="n"/>
       <c r="O353" s="9" t="n"/>
-      <c r="P353" s="9" t="n"/>
+      <c r="P353" s="17" t="n"/>
       <c r="Q353" s="9" t="n"/>
       <c r="R353" s="9" t="n"/>
       <c r="S353" s="9" t="n"/>
@@ -8890,7 +8901,7 @@
       <c r="M354" s="9" t="n"/>
       <c r="N354" s="9" t="n"/>
       <c r="O354" s="9" t="n"/>
-      <c r="P354" s="9" t="n"/>
+      <c r="P354" s="17" t="n"/>
       <c r="Q354" s="9" t="n"/>
       <c r="R354" s="9" t="n"/>
       <c r="S354" s="9" t="n"/>
@@ -8911,7 +8922,7 @@
       <c r="M355" s="9" t="n"/>
       <c r="N355" s="9" t="n"/>
       <c r="O355" s="9" t="n"/>
-      <c r="P355" s="9" t="n"/>
+      <c r="P355" s="17" t="n"/>
       <c r="Q355" s="9" t="n"/>
       <c r="R355" s="9" t="n"/>
       <c r="S355" s="9" t="n"/>
@@ -8932,7 +8943,7 @@
       <c r="M356" s="9" t="n"/>
       <c r="N356" s="9" t="n"/>
       <c r="O356" s="9" t="n"/>
-      <c r="P356" s="9" t="n"/>
+      <c r="P356" s="17" t="n"/>
       <c r="Q356" s="9" t="n"/>
       <c r="R356" s="9" t="n"/>
       <c r="S356" s="9" t="n"/>
@@ -8953,7 +8964,7 @@
       <c r="M357" s="9" t="n"/>
       <c r="N357" s="9" t="n"/>
       <c r="O357" s="9" t="n"/>
-      <c r="P357" s="9" t="n"/>
+      <c r="P357" s="17" t="n"/>
       <c r="Q357" s="9" t="n"/>
       <c r="R357" s="9" t="n"/>
       <c r="S357" s="9" t="n"/>
@@ -8974,7 +8985,7 @@
       <c r="M358" s="9" t="n"/>
       <c r="N358" s="9" t="n"/>
       <c r="O358" s="9" t="n"/>
-      <c r="P358" s="9" t="n"/>
+      <c r="P358" s="17" t="n"/>
       <c r="Q358" s="9" t="n"/>
       <c r="R358" s="9" t="n"/>
       <c r="S358" s="9" t="n"/>
@@ -8995,7 +9006,7 @@
       <c r="M359" s="9" t="n"/>
       <c r="N359" s="9" t="n"/>
       <c r="O359" s="9" t="n"/>
-      <c r="P359" s="9" t="n"/>
+      <c r="P359" s="17" t="n"/>
       <c r="Q359" s="9" t="n"/>
       <c r="R359" s="9" t="n"/>
       <c r="S359" s="9" t="n"/>
@@ -9016,7 +9027,7 @@
       <c r="M360" s="9" t="n"/>
       <c r="N360" s="9" t="n"/>
       <c r="O360" s="9" t="n"/>
-      <c r="P360" s="9" t="n"/>
+      <c r="P360" s="17" t="n"/>
       <c r="Q360" s="9" t="n"/>
       <c r="R360" s="9" t="n"/>
       <c r="S360" s="9" t="n"/>
@@ -9037,7 +9048,7 @@
       <c r="M361" s="9" t="n"/>
       <c r="N361" s="9" t="n"/>
       <c r="O361" s="9" t="n"/>
-      <c r="P361" s="9" t="n"/>
+      <c r="P361" s="17" t="n"/>
       <c r="Q361" s="9" t="n"/>
       <c r="R361" s="9" t="n"/>
       <c r="S361" s="9" t="n"/>
@@ -9058,7 +9069,7 @@
       <c r="M362" s="9" t="n"/>
       <c r="N362" s="9" t="n"/>
       <c r="O362" s="9" t="n"/>
-      <c r="P362" s="9" t="n"/>
+      <c r="P362" s="17" t="n"/>
       <c r="Q362" s="9" t="n"/>
       <c r="R362" s="9" t="n"/>
       <c r="S362" s="9" t="n"/>
@@ -9079,7 +9090,7 @@
       <c r="M363" s="9" t="n"/>
       <c r="N363" s="9" t="n"/>
       <c r="O363" s="9" t="n"/>
-      <c r="P363" s="9" t="n"/>
+      <c r="P363" s="17" t="n"/>
       <c r="Q363" s="9" t="n"/>
       <c r="R363" s="9" t="n"/>
       <c r="S363" s="9" t="n"/>
@@ -9100,7 +9111,7 @@
       <c r="M364" s="9" t="n"/>
       <c r="N364" s="9" t="n"/>
       <c r="O364" s="9" t="n"/>
-      <c r="P364" s="9" t="n"/>
+      <c r="P364" s="17" t="n"/>
       <c r="Q364" s="9" t="n"/>
       <c r="R364" s="9" t="n"/>
       <c r="S364" s="9" t="n"/>
@@ -9121,7 +9132,7 @@
       <c r="M365" s="9" t="n"/>
       <c r="N365" s="9" t="n"/>
       <c r="O365" s="9" t="n"/>
-      <c r="P365" s="9" t="n"/>
+      <c r="P365" s="17" t="n"/>
       <c r="Q365" s="9" t="n"/>
       <c r="R365" s="9" t="n"/>
       <c r="S365" s="9" t="n"/>
@@ -9142,7 +9153,7 @@
       <c r="M366" s="9" t="n"/>
       <c r="N366" s="9" t="n"/>
       <c r="O366" s="9" t="n"/>
-      <c r="P366" s="9" t="n"/>
+      <c r="P366" s="17" t="n"/>
       <c r="Q366" s="9" t="n"/>
       <c r="R366" s="9" t="n"/>
       <c r="S366" s="9" t="n"/>
@@ -9163,7 +9174,7 @@
       <c r="M367" s="9" t="n"/>
       <c r="N367" s="9" t="n"/>
       <c r="O367" s="9" t="n"/>
-      <c r="P367" s="9" t="n"/>
+      <c r="P367" s="17" t="n"/>
       <c r="Q367" s="9" t="n"/>
       <c r="R367" s="9" t="n"/>
       <c r="S367" s="9" t="n"/>
@@ -9184,7 +9195,7 @@
       <c r="M368" s="9" t="n"/>
       <c r="N368" s="9" t="n"/>
       <c r="O368" s="9" t="n"/>
-      <c r="P368" s="9" t="n"/>
+      <c r="P368" s="17" t="n"/>
       <c r="Q368" s="9" t="n"/>
       <c r="R368" s="9" t="n"/>
       <c r="S368" s="9" t="n"/>
@@ -9205,7 +9216,7 @@
       <c r="M369" s="9" t="n"/>
       <c r="N369" s="9" t="n"/>
       <c r="O369" s="9" t="n"/>
-      <c r="P369" s="9" t="n"/>
+      <c r="P369" s="17" t="n"/>
       <c r="Q369" s="9" t="n"/>
       <c r="R369" s="9" t="n"/>
       <c r="S369" s="9" t="n"/>
@@ -9226,7 +9237,7 @@
       <c r="M370" s="9" t="n"/>
       <c r="N370" s="9" t="n"/>
       <c r="O370" s="9" t="n"/>
-      <c r="P370" s="9" t="n"/>
+      <c r="P370" s="17" t="n"/>
       <c r="Q370" s="9" t="n"/>
       <c r="R370" s="9" t="n"/>
       <c r="S370" s="9" t="n"/>
@@ -9247,7 +9258,7 @@
       <c r="M371" s="9" t="n"/>
       <c r="N371" s="9" t="n"/>
       <c r="O371" s="9" t="n"/>
-      <c r="P371" s="9" t="n"/>
+      <c r="P371" s="17" t="n"/>
       <c r="Q371" s="9" t="n"/>
       <c r="R371" s="9" t="n"/>
       <c r="S371" s="9" t="n"/>
@@ -9268,7 +9279,7 @@
       <c r="M372" s="9" t="n"/>
       <c r="N372" s="9" t="n"/>
       <c r="O372" s="9" t="n"/>
-      <c r="P372" s="9" t="n"/>
+      <c r="P372" s="17" t="n"/>
       <c r="Q372" s="9" t="n"/>
       <c r="R372" s="9" t="n"/>
       <c r="S372" s="9" t="n"/>
@@ -9289,7 +9300,7 @@
       <c r="M373" s="9" t="n"/>
       <c r="N373" s="9" t="n"/>
       <c r="O373" s="9" t="n"/>
-      <c r="P373" s="9" t="n"/>
+      <c r="P373" s="17" t="n"/>
       <c r="Q373" s="9" t="n"/>
       <c r="R373" s="9" t="n"/>
       <c r="S373" s="9" t="n"/>
@@ -9310,7 +9321,7 @@
       <c r="M374" s="9" t="n"/>
       <c r="N374" s="9" t="n"/>
       <c r="O374" s="9" t="n"/>
-      <c r="P374" s="9" t="n"/>
+      <c r="P374" s="17" t="n"/>
       <c r="Q374" s="9" t="n"/>
       <c r="R374" s="9" t="n"/>
       <c r="S374" s="9" t="n"/>
@@ -9331,7 +9342,7 @@
       <c r="M375" s="9" t="n"/>
       <c r="N375" s="9" t="n"/>
       <c r="O375" s="9" t="n"/>
-      <c r="P375" s="9" t="n"/>
+      <c r="P375" s="17" t="n"/>
       <c r="Q375" s="9" t="n"/>
       <c r="R375" s="9" t="n"/>
       <c r="S375" s="9" t="n"/>
@@ -9352,7 +9363,7 @@
       <c r="M376" s="9" t="n"/>
       <c r="N376" s="9" t="n"/>
       <c r="O376" s="9" t="n"/>
-      <c r="P376" s="9" t="n"/>
+      <c r="P376" s="17" t="n"/>
       <c r="Q376" s="9" t="n"/>
       <c r="R376" s="9" t="n"/>
       <c r="S376" s="9" t="n"/>
@@ -9373,7 +9384,7 @@
       <c r="M377" s="9" t="n"/>
       <c r="N377" s="9" t="n"/>
       <c r="O377" s="9" t="n"/>
-      <c r="P377" s="9" t="n"/>
+      <c r="P377" s="17" t="n"/>
       <c r="Q377" s="9" t="n"/>
       <c r="R377" s="9" t="n"/>
       <c r="S377" s="9" t="n"/>
@@ -9394,7 +9405,7 @@
       <c r="M378" s="9" t="n"/>
       <c r="N378" s="9" t="n"/>
       <c r="O378" s="9" t="n"/>
-      <c r="P378" s="9" t="n"/>
+      <c r="P378" s="17" t="n"/>
       <c r="Q378" s="9" t="n"/>
       <c r="R378" s="9" t="n"/>
       <c r="S378" s="9" t="n"/>
@@ -9415,7 +9426,7 @@
       <c r="M379" s="9" t="n"/>
       <c r="N379" s="9" t="n"/>
       <c r="O379" s="9" t="n"/>
-      <c r="P379" s="9" t="n"/>
+      <c r="P379" s="17" t="n"/>
       <c r="Q379" s="9" t="n"/>
       <c r="R379" s="9" t="n"/>
       <c r="S379" s="9" t="n"/>
@@ -9436,7 +9447,7 @@
       <c r="M380" s="9" t="n"/>
       <c r="N380" s="9" t="n"/>
       <c r="O380" s="9" t="n"/>
-      <c r="P380" s="9" t="n"/>
+      <c r="P380" s="17" t="n"/>
       <c r="Q380" s="9" t="n"/>
       <c r="R380" s="9" t="n"/>
       <c r="S380" s="9" t="n"/>
@@ -9457,7 +9468,7 @@
       <c r="M381" s="9" t="n"/>
       <c r="N381" s="9" t="n"/>
       <c r="O381" s="9" t="n"/>
-      <c r="P381" s="9" t="n"/>
+      <c r="P381" s="17" t="n"/>
       <c r="Q381" s="9" t="n"/>
       <c r="R381" s="9" t="n"/>
       <c r="S381" s="9" t="n"/>
@@ -9478,7 +9489,7 @@
       <c r="M382" s="9" t="n"/>
       <c r="N382" s="9" t="n"/>
       <c r="O382" s="9" t="n"/>
-      <c r="P382" s="9" t="n"/>
+      <c r="P382" s="17" t="n"/>
       <c r="Q382" s="9" t="n"/>
       <c r="R382" s="9" t="n"/>
       <c r="S382" s="9" t="n"/>
@@ -9499,7 +9510,7 @@
       <c r="M383" s="9" t="n"/>
       <c r="N383" s="9" t="n"/>
       <c r="O383" s="9" t="n"/>
-      <c r="P383" s="9" t="n"/>
+      <c r="P383" s="17" t="n"/>
       <c r="Q383" s="9" t="n"/>
       <c r="R383" s="9" t="n"/>
       <c r="S383" s="9" t="n"/>
@@ -9520,7 +9531,7 @@
       <c r="M384" s="9" t="n"/>
       <c r="N384" s="9" t="n"/>
       <c r="O384" s="9" t="n"/>
-      <c r="P384" s="9" t="n"/>
+      <c r="P384" s="17" t="n"/>
       <c r="Q384" s="9" t="n"/>
       <c r="R384" s="9" t="n"/>
       <c r="S384" s="9" t="n"/>
@@ -9541,7 +9552,7 @@
       <c r="M385" s="9" t="n"/>
       <c r="N385" s="9" t="n"/>
       <c r="O385" s="9" t="n"/>
-      <c r="P385" s="9" t="n"/>
+      <c r="P385" s="17" t="n"/>
       <c r="Q385" s="9" t="n"/>
       <c r="R385" s="9" t="n"/>
       <c r="S385" s="9" t="n"/>
@@ -9562,7 +9573,7 @@
       <c r="M386" s="9" t="n"/>
       <c r="N386" s="9" t="n"/>
       <c r="O386" s="9" t="n"/>
-      <c r="P386" s="9" t="n"/>
+      <c r="P386" s="17" t="n"/>
       <c r="Q386" s="9" t="n"/>
       <c r="R386" s="9" t="n"/>
       <c r="S386" s="9" t="n"/>
@@ -9583,7 +9594,7 @@
       <c r="M387" s="9" t="n"/>
       <c r="N387" s="9" t="n"/>
       <c r="O387" s="9" t="n"/>
-      <c r="P387" s="9" t="n"/>
+      <c r="P387" s="17" t="n"/>
       <c r="Q387" s="9" t="n"/>
       <c r="R387" s="9" t="n"/>
       <c r="S387" s="9" t="n"/>
@@ -9604,7 +9615,7 @@
       <c r="M388" s="9" t="n"/>
       <c r="N388" s="9" t="n"/>
       <c r="O388" s="9" t="n"/>
-      <c r="P388" s="9" t="n"/>
+      <c r="P388" s="17" t="n"/>
       <c r="Q388" s="9" t="n"/>
       <c r="R388" s="9" t="n"/>
       <c r="S388" s="9" t="n"/>
@@ -9625,7 +9636,7 @@
       <c r="M389" s="9" t="n"/>
       <c r="N389" s="9" t="n"/>
       <c r="O389" s="9" t="n"/>
-      <c r="P389" s="9" t="n"/>
+      <c r="P389" s="17" t="n"/>
       <c r="Q389" s="9" t="n"/>
       <c r="R389" s="9" t="n"/>
       <c r="S389" s="9" t="n"/>
@@ -9646,7 +9657,7 @@
       <c r="M390" s="9" t="n"/>
       <c r="N390" s="9" t="n"/>
       <c r="O390" s="9" t="n"/>
-      <c r="P390" s="9" t="n"/>
+      <c r="P390" s="17" t="n"/>
       <c r="Q390" s="9" t="n"/>
       <c r="R390" s="9" t="n"/>
       <c r="S390" s="9" t="n"/>
@@ -9667,7 +9678,7 @@
       <c r="M391" s="9" t="n"/>
       <c r="N391" s="9" t="n"/>
       <c r="O391" s="9" t="n"/>
-      <c r="P391" s="9" t="n"/>
+      <c r="P391" s="17" t="n"/>
       <c r="Q391" s="9" t="n"/>
       <c r="R391" s="9" t="n"/>
       <c r="S391" s="9" t="n"/>
@@ -9688,7 +9699,7 @@
       <c r="M392" s="9" t="n"/>
       <c r="N392" s="9" t="n"/>
       <c r="O392" s="9" t="n"/>
-      <c r="P392" s="9" t="n"/>
+      <c r="P392" s="17" t="n"/>
       <c r="Q392" s="9" t="n"/>
       <c r="R392" s="9" t="n"/>
       <c r="S392" s="9" t="n"/>
@@ -9709,7 +9720,7 @@
       <c r="M393" s="9" t="n"/>
       <c r="N393" s="9" t="n"/>
       <c r="O393" s="9" t="n"/>
-      <c r="P393" s="9" t="n"/>
+      <c r="P393" s="17" t="n"/>
       <c r="Q393" s="9" t="n"/>
       <c r="R393" s="9" t="n"/>
       <c r="S393" s="9" t="n"/>
@@ -9730,7 +9741,7 @@
       <c r="M394" s="9" t="n"/>
       <c r="N394" s="9" t="n"/>
       <c r="O394" s="9" t="n"/>
-      <c r="P394" s="9" t="n"/>
+      <c r="P394" s="17" t="n"/>
       <c r="Q394" s="9" t="n"/>
       <c r="R394" s="9" t="n"/>
       <c r="S394" s="9" t="n"/>
@@ -9751,7 +9762,7 @@
       <c r="M395" s="9" t="n"/>
       <c r="N395" s="9" t="n"/>
       <c r="O395" s="9" t="n"/>
-      <c r="P395" s="9" t="n"/>
+      <c r="P395" s="17" t="n"/>
       <c r="Q395" s="9" t="n"/>
       <c r="R395" s="9" t="n"/>
       <c r="S395" s="9" t="n"/>
@@ -9772,7 +9783,7 @@
       <c r="M396" s="9" t="n"/>
       <c r="N396" s="9" t="n"/>
       <c r="O396" s="9" t="n"/>
-      <c r="P396" s="9" t="n"/>
+      <c r="P396" s="17" t="n"/>
       <c r="Q396" s="9" t="n"/>
       <c r="R396" s="9" t="n"/>
       <c r="S396" s="9" t="n"/>
@@ -9793,7 +9804,7 @@
       <c r="M397" s="9" t="n"/>
       <c r="N397" s="9" t="n"/>
       <c r="O397" s="9" t="n"/>
-      <c r="P397" s="9" t="n"/>
+      <c r="P397" s="17" t="n"/>
       <c r="Q397" s="9" t="n"/>
       <c r="R397" s="9" t="n"/>
       <c r="S397" s="9" t="n"/>
@@ -9814,7 +9825,7 @@
       <c r="M398" s="9" t="n"/>
       <c r="N398" s="9" t="n"/>
       <c r="O398" s="9" t="n"/>
-      <c r="P398" s="9" t="n"/>
+      <c r="P398" s="17" t="n"/>
       <c r="Q398" s="9" t="n"/>
       <c r="R398" s="9" t="n"/>
       <c r="S398" s="9" t="n"/>
@@ -9835,7 +9846,7 @@
       <c r="M399" s="9" t="n"/>
       <c r="N399" s="9" t="n"/>
       <c r="O399" s="9" t="n"/>
-      <c r="P399" s="9" t="n"/>
+      <c r="P399" s="17" t="n"/>
       <c r="Q399" s="9" t="n"/>
       <c r="R399" s="9" t="n"/>
       <c r="S399" s="9" t="n"/>
@@ -9856,7 +9867,7 @@
       <c r="M400" s="9" t="n"/>
       <c r="N400" s="9" t="n"/>
       <c r="O400" s="9" t="n"/>
-      <c r="P400" s="9" t="n"/>
+      <c r="P400" s="17" t="n"/>
       <c r="Q400" s="9" t="n"/>
       <c r="R400" s="9" t="n"/>
       <c r="S400" s="9" t="n"/>
@@ -9877,7 +9888,7 @@
       <c r="M401" s="9" t="n"/>
       <c r="N401" s="9" t="n"/>
       <c r="O401" s="9" t="n"/>
-      <c r="P401" s="9" t="n"/>
+      <c r="P401" s="17" t="n"/>
       <c r="Q401" s="9" t="n"/>
       <c r="R401" s="9" t="n"/>
       <c r="S401" s="9" t="n"/>
@@ -9898,7 +9909,7 @@
       <c r="M402" s="9" t="n"/>
       <c r="N402" s="9" t="n"/>
       <c r="O402" s="9" t="n"/>
-      <c r="P402" s="9" t="n"/>
+      <c r="P402" s="17" t="n"/>
       <c r="Q402" s="9" t="n"/>
       <c r="R402" s="9" t="n"/>
       <c r="S402" s="9" t="n"/>
@@ -9919,7 +9930,7 @@
       <c r="M403" s="9" t="n"/>
       <c r="N403" s="9" t="n"/>
       <c r="O403" s="9" t="n"/>
-      <c r="P403" s="9" t="n"/>
+      <c r="P403" s="17" t="n"/>
       <c r="Q403" s="9" t="n"/>
       <c r="R403" s="9" t="n"/>
       <c r="S403" s="9" t="n"/>
@@ -9940,7 +9951,7 @@
       <c r="M404" s="9" t="n"/>
       <c r="N404" s="9" t="n"/>
       <c r="O404" s="9" t="n"/>
-      <c r="P404" s="9" t="n"/>
+      <c r="P404" s="17" t="n"/>
       <c r="Q404" s="9" t="n"/>
       <c r="R404" s="9" t="n"/>
       <c r="S404" s="9" t="n"/>
@@ -9961,7 +9972,7 @@
       <c r="M405" s="9" t="n"/>
       <c r="N405" s="9" t="n"/>
       <c r="O405" s="9" t="n"/>
-      <c r="P405" s="9" t="n"/>
+      <c r="P405" s="17" t="n"/>
       <c r="Q405" s="9" t="n"/>
       <c r="R405" s="9" t="n"/>
       <c r="S405" s="9" t="n"/>
@@ -9982,7 +9993,7 @@
       <c r="M406" s="9" t="n"/>
       <c r="N406" s="9" t="n"/>
       <c r="O406" s="9" t="n"/>
-      <c r="P406" s="9" t="n"/>
+      <c r="P406" s="17" t="n"/>
       <c r="Q406" s="9" t="n"/>
       <c r="R406" s="9" t="n"/>
       <c r="S406" s="9" t="n"/>
@@ -10003,7 +10014,7 @@
       <c r="M407" s="9" t="n"/>
       <c r="N407" s="9" t="n"/>
       <c r="O407" s="9" t="n"/>
-      <c r="P407" s="9" t="n"/>
+      <c r="P407" s="17" t="n"/>
       <c r="Q407" s="9" t="n"/>
       <c r="R407" s="9" t="n"/>
       <c r="S407" s="9" t="n"/>
@@ -10024,7 +10035,7 @@
       <c r="M408" s="9" t="n"/>
       <c r="N408" s="9" t="n"/>
       <c r="O408" s="9" t="n"/>
-      <c r="P408" s="9" t="n"/>
+      <c r="P408" s="17" t="n"/>
       <c r="Q408" s="9" t="n"/>
       <c r="R408" s="9" t="n"/>
       <c r="S408" s="9" t="n"/>
@@ -10045,7 +10056,7 @@
       <c r="M409" s="9" t="n"/>
       <c r="N409" s="9" t="n"/>
       <c r="O409" s="9" t="n"/>
-      <c r="P409" s="9" t="n"/>
+      <c r="P409" s="17" t="n"/>
       <c r="Q409" s="9" t="n"/>
       <c r="R409" s="9" t="n"/>
       <c r="S409" s="9" t="n"/>
@@ -10066,7 +10077,7 @@
       <c r="M410" s="9" t="n"/>
       <c r="N410" s="9" t="n"/>
       <c r="O410" s="9" t="n"/>
-      <c r="P410" s="9" t="n"/>
+      <c r="P410" s="17" t="n"/>
       <c r="Q410" s="9" t="n"/>
       <c r="R410" s="9" t="n"/>
       <c r="S410" s="9" t="n"/>
@@ -10087,7 +10098,7 @@
       <c r="M411" s="9" t="n"/>
       <c r="N411" s="9" t="n"/>
       <c r="O411" s="9" t="n"/>
-      <c r="P411" s="9" t="n"/>
+      <c r="P411" s="17" t="n"/>
       <c r="Q411" s="9" t="n"/>
       <c r="R411" s="9" t="n"/>
       <c r="S411" s="9" t="n"/>
@@ -10108,7 +10119,7 @@
       <c r="M412" s="9" t="n"/>
       <c r="N412" s="9" t="n"/>
       <c r="O412" s="9" t="n"/>
-      <c r="P412" s="9" t="n"/>
+      <c r="P412" s="17" t="n"/>
       <c r="Q412" s="9" t="n"/>
       <c r="R412" s="9" t="n"/>
       <c r="S412" s="9" t="n"/>
@@ -10129,7 +10140,7 @@
       <c r="M413" s="9" t="n"/>
       <c r="N413" s="9" t="n"/>
       <c r="O413" s="9" t="n"/>
-      <c r="P413" s="9" t="n"/>
+      <c r="P413" s="17" t="n"/>
       <c r="Q413" s="9" t="n"/>
       <c r="R413" s="9" t="n"/>
       <c r="S413" s="9" t="n"/>
@@ -10150,7 +10161,7 @@
       <c r="M414" s="9" t="n"/>
       <c r="N414" s="9" t="n"/>
       <c r="O414" s="9" t="n"/>
-      <c r="P414" s="9" t="n"/>
+      <c r="P414" s="17" t="n"/>
       <c r="Q414" s="9" t="n"/>
       <c r="R414" s="9" t="n"/>
       <c r="S414" s="9" t="n"/>
@@ -10171,7 +10182,7 @@
       <c r="M415" s="9" t="n"/>
       <c r="N415" s="9" t="n"/>
       <c r="O415" s="9" t="n"/>
-      <c r="P415" s="9" t="n"/>
+      <c r="P415" s="17" t="n"/>
       <c r="Q415" s="9" t="n"/>
       <c r="R415" s="9" t="n"/>
       <c r="S415" s="9" t="n"/>
@@ -10192,7 +10203,7 @@
       <c r="M416" s="9" t="n"/>
       <c r="N416" s="9" t="n"/>
       <c r="O416" s="9" t="n"/>
-      <c r="P416" s="9" t="n"/>
+      <c r="P416" s="17" t="n"/>
       <c r="Q416" s="9" t="n"/>
       <c r="R416" s="9" t="n"/>
       <c r="S416" s="9" t="n"/>
@@ -10213,7 +10224,7 @@
       <c r="M417" s="9" t="n"/>
       <c r="N417" s="9" t="n"/>
       <c r="O417" s="9" t="n"/>
-      <c r="P417" s="9" t="n"/>
+      <c r="P417" s="17" t="n"/>
       <c r="Q417" s="9" t="n"/>
       <c r="R417" s="9" t="n"/>
       <c r="S417" s="9" t="n"/>
@@ -10234,7 +10245,7 @@
       <c r="M418" s="9" t="n"/>
       <c r="N418" s="9" t="n"/>
       <c r="O418" s="9" t="n"/>
-      <c r="P418" s="9" t="n"/>
+      <c r="P418" s="17" t="n"/>
       <c r="Q418" s="9" t="n"/>
       <c r="R418" s="9" t="n"/>
       <c r="S418" s="9" t="n"/>
@@ -10255,7 +10266,7 @@
       <c r="M419" s="9" t="n"/>
       <c r="N419" s="9" t="n"/>
       <c r="O419" s="9" t="n"/>
-      <c r="P419" s="9" t="n"/>
+      <c r="P419" s="17" t="n"/>
       <c r="Q419" s="9" t="n"/>
       <c r="R419" s="9" t="n"/>
       <c r="S419" s="9" t="n"/>
@@ -10276,7 +10287,7 @@
       <c r="M420" s="9" t="n"/>
       <c r="N420" s="9" t="n"/>
       <c r="O420" s="9" t="n"/>
-      <c r="P420" s="9" t="n"/>
+      <c r="P420" s="17" t="n"/>
       <c r="Q420" s="9" t="n"/>
       <c r="R420" s="9" t="n"/>
       <c r="S420" s="9" t="n"/>
@@ -10297,7 +10308,7 @@
       <c r="M421" s="9" t="n"/>
       <c r="N421" s="9" t="n"/>
       <c r="O421" s="9" t="n"/>
-      <c r="P421" s="9" t="n"/>
+      <c r="P421" s="17" t="n"/>
       <c r="Q421" s="9" t="n"/>
       <c r="R421" s="9" t="n"/>
       <c r="S421" s="9" t="n"/>
@@ -10318,7 +10329,7 @@
       <c r="M422" s="9" t="n"/>
       <c r="N422" s="9" t="n"/>
       <c r="O422" s="9" t="n"/>
-      <c r="P422" s="9" t="n"/>
+      <c r="P422" s="17" t="n"/>
       <c r="Q422" s="9" t="n"/>
       <c r="R422" s="9" t="n"/>
       <c r="S422" s="9" t="n"/>
@@ -10339,7 +10350,7 @@
       <c r="M423" s="9" t="n"/>
       <c r="N423" s="9" t="n"/>
       <c r="O423" s="9" t="n"/>
-      <c r="P423" s="9" t="n"/>
+      <c r="P423" s="17" t="n"/>
       <c r="Q423" s="9" t="n"/>
       <c r="R423" s="9" t="n"/>
       <c r="S423" s="9" t="n"/>
@@ -10360,7 +10371,7 @@
       <c r="M424" s="9" t="n"/>
       <c r="N424" s="9" t="n"/>
       <c r="O424" s="9" t="n"/>
-      <c r="P424" s="9" t="n"/>
+      <c r="P424" s="17" t="n"/>
       <c r="Q424" s="9" t="n"/>
       <c r="R424" s="9" t="n"/>
       <c r="S424" s="9" t="n"/>
@@ -10381,7 +10392,7 @@
       <c r="M425" s="9" t="n"/>
       <c r="N425" s="9" t="n"/>
       <c r="O425" s="9" t="n"/>
-      <c r="P425" s="9" t="n"/>
+      <c r="P425" s="17" t="n"/>
       <c r="Q425" s="9" t="n"/>
       <c r="R425" s="9" t="n"/>
       <c r="S425" s="9" t="n"/>
@@ -10402,7 +10413,7 @@
       <c r="M426" s="9" t="n"/>
       <c r="N426" s="9" t="n"/>
       <c r="O426" s="9" t="n"/>
-      <c r="P426" s="9" t="n"/>
+      <c r="P426" s="17" t="n"/>
       <c r="Q426" s="9" t="n"/>
       <c r="R426" s="9" t="n"/>
       <c r="S426" s="9" t="n"/>
@@ -10423,7 +10434,7 @@
       <c r="M427" s="9" t="n"/>
       <c r="N427" s="9" t="n"/>
       <c r="O427" s="9" t="n"/>
-      <c r="P427" s="9" t="n"/>
+      <c r="P427" s="17" t="n"/>
       <c r="Q427" s="9" t="n"/>
       <c r="R427" s="9" t="n"/>
       <c r="S427" s="9" t="n"/>
@@ -10444,7 +10455,7 @@
       <c r="M428" s="9" t="n"/>
       <c r="N428" s="9" t="n"/>
       <c r="O428" s="9" t="n"/>
-      <c r="P428" s="9" t="n"/>
+      <c r="P428" s="17" t="n"/>
       <c r="Q428" s="9" t="n"/>
       <c r="R428" s="9" t="n"/>
       <c r="S428" s="9" t="n"/>
@@ -10465,7 +10476,7 @@
       <c r="M429" s="9" t="n"/>
       <c r="N429" s="9" t="n"/>
       <c r="O429" s="9" t="n"/>
-      <c r="P429" s="9" t="n"/>
+      <c r="P429" s="17" t="n"/>
       <c r="Q429" s="9" t="n"/>
       <c r="R429" s="9" t="n"/>
       <c r="S429" s="9" t="n"/>
@@ -10486,7 +10497,7 @@
       <c r="M430" s="9" t="n"/>
       <c r="N430" s="9" t="n"/>
       <c r="O430" s="9" t="n"/>
-      <c r="P430" s="9" t="n"/>
+      <c r="P430" s="17" t="n"/>
       <c r="Q430" s="9" t="n"/>
       <c r="R430" s="9" t="n"/>
       <c r="S430" s="9" t="n"/>
@@ -10507,7 +10518,7 @@
       <c r="M431" s="9" t="n"/>
       <c r="N431" s="9" t="n"/>
       <c r="O431" s="9" t="n"/>
-      <c r="P431" s="9" t="n"/>
+      <c r="P431" s="17" t="n"/>
       <c r="Q431" s="9" t="n"/>
       <c r="R431" s="9" t="n"/>
       <c r="S431" s="9" t="n"/>
@@ -10528,7 +10539,7 @@
       <c r="M432" s="9" t="n"/>
       <c r="N432" s="9" t="n"/>
       <c r="O432" s="9" t="n"/>
-      <c r="P432" s="9" t="n"/>
+      <c r="P432" s="17" t="n"/>
       <c r="Q432" s="9" t="n"/>
       <c r="R432" s="9" t="n"/>
       <c r="S432" s="9" t="n"/>
@@ -10549,7 +10560,7 @@
       <c r="M433" s="9" t="n"/>
       <c r="N433" s="9" t="n"/>
       <c r="O433" s="9" t="n"/>
-      <c r="P433" s="9" t="n"/>
+      <c r="P433" s="17" t="n"/>
       <c r="Q433" s="9" t="n"/>
       <c r="R433" s="9" t="n"/>
       <c r="S433" s="9" t="n"/>
@@ -10570,7 +10581,7 @@
       <c r="M434" s="9" t="n"/>
       <c r="N434" s="9" t="n"/>
       <c r="O434" s="9" t="n"/>
-      <c r="P434" s="9" t="n"/>
+      <c r="P434" s="17" t="n"/>
       <c r="Q434" s="9" t="n"/>
       <c r="R434" s="9" t="n"/>
       <c r="S434" s="9" t="n"/>
@@ -10591,7 +10602,7 @@
       <c r="M435" s="9" t="n"/>
       <c r="N435" s="9" t="n"/>
       <c r="O435" s="9" t="n"/>
-      <c r="P435" s="9" t="n"/>
+      <c r="P435" s="17" t="n"/>
       <c r="Q435" s="9" t="n"/>
       <c r="R435" s="9" t="n"/>
       <c r="S435" s="9" t="n"/>
@@ -10612,7 +10623,7 @@
       <c r="M436" s="9" t="n"/>
       <c r="N436" s="9" t="n"/>
       <c r="O436" s="9" t="n"/>
-      <c r="P436" s="9" t="n"/>
+      <c r="P436" s="17" t="n"/>
       <c r="Q436" s="9" t="n"/>
       <c r="R436" s="9" t="n"/>
       <c r="S436" s="9" t="n"/>
@@ -10633,7 +10644,7 @@
       <c r="M437" s="9" t="n"/>
       <c r="N437" s="9" t="n"/>
       <c r="O437" s="9" t="n"/>
-      <c r="P437" s="9" t="n"/>
+      <c r="P437" s="17" t="n"/>
       <c r="Q437" s="9" t="n"/>
       <c r="R437" s="9" t="n"/>
       <c r="S437" s="9" t="n"/>
@@ -10654,7 +10665,7 @@
       <c r="M438" s="9" t="n"/>
       <c r="N438" s="9" t="n"/>
       <c r="O438" s="9" t="n"/>
-      <c r="P438" s="9" t="n"/>
+      <c r="P438" s="17" t="n"/>
       <c r="Q438" s="9" t="n"/>
       <c r="R438" s="9" t="n"/>
       <c r="S438" s="9" t="n"/>
@@ -10675,7 +10686,7 @@
       <c r="M439" s="9" t="n"/>
       <c r="N439" s="9" t="n"/>
       <c r="O439" s="9" t="n"/>
-      <c r="P439" s="9" t="n"/>
+      <c r="P439" s="17" t="n"/>
       <c r="Q439" s="9" t="n"/>
       <c r="R439" s="9" t="n"/>
       <c r="S439" s="9" t="n"/>
@@ -10696,7 +10707,7 @@
       <c r="M440" s="9" t="n"/>
       <c r="N440" s="9" t="n"/>
       <c r="O440" s="9" t="n"/>
-      <c r="P440" s="9" t="n"/>
+      <c r="P440" s="17" t="n"/>
       <c r="Q440" s="9" t="n"/>
       <c r="R440" s="9" t="n"/>
       <c r="S440" s="9" t="n"/>
@@ -10717,7 +10728,7 @@
       <c r="M441" s="9" t="n"/>
       <c r="N441" s="9" t="n"/>
       <c r="O441" s="9" t="n"/>
-      <c r="P441" s="9" t="n"/>
+      <c r="P441" s="17" t="n"/>
       <c r="Q441" s="9" t="n"/>
       <c r="R441" s="9" t="n"/>
       <c r="S441" s="9" t="n"/>
@@ -10738,7 +10749,7 @@
       <c r="M442" s="9" t="n"/>
       <c r="N442" s="9" t="n"/>
       <c r="O442" s="9" t="n"/>
-      <c r="P442" s="9" t="n"/>
+      <c r="P442" s="17" t="n"/>
       <c r="Q442" s="9" t="n"/>
       <c r="R442" s="9" t="n"/>
       <c r="S442" s="9" t="n"/>
@@ -10759,7 +10770,7 @@
       <c r="M443" s="9" t="n"/>
       <c r="N443" s="9" t="n"/>
       <c r="O443" s="9" t="n"/>
-      <c r="P443" s="9" t="n"/>
+      <c r="P443" s="17" t="n"/>
       <c r="Q443" s="9" t="n"/>
       <c r="R443" s="9" t="n"/>
       <c r="S443" s="9" t="n"/>
@@ -10780,7 +10791,7 @@
       <c r="M444" s="9" t="n"/>
       <c r="N444" s="9" t="n"/>
       <c r="O444" s="9" t="n"/>
-      <c r="P444" s="9" t="n"/>
+      <c r="P444" s="17" t="n"/>
       <c r="Q444" s="9" t="n"/>
       <c r="R444" s="9" t="n"/>
       <c r="S444" s="9" t="n"/>
@@ -10801,7 +10812,7 @@
       <c r="M445" s="9" t="n"/>
       <c r="N445" s="9" t="n"/>
       <c r="O445" s="9" t="n"/>
-      <c r="P445" s="9" t="n"/>
+      <c r="P445" s="17" t="n"/>
       <c r="Q445" s="9" t="n"/>
       <c r="R445" s="9" t="n"/>
       <c r="S445" s="9" t="n"/>
@@ -10822,7 +10833,7 @@
       <c r="M446" s="9" t="n"/>
       <c r="N446" s="9" t="n"/>
       <c r="O446" s="9" t="n"/>
-      <c r="P446" s="9" t="n"/>
+      <c r="P446" s="17" t="n"/>
       <c r="Q446" s="9" t="n"/>
       <c r="R446" s="9" t="n"/>
       <c r="S446" s="9" t="n"/>
@@ -10843,7 +10854,7 @@
       <c r="M447" s="9" t="n"/>
       <c r="N447" s="9" t="n"/>
       <c r="O447" s="9" t="n"/>
-      <c r="P447" s="9" t="n"/>
+      <c r="P447" s="17" t="n"/>
       <c r="Q447" s="9" t="n"/>
       <c r="R447" s="9" t="n"/>
       <c r="S447" s="9" t="n"/>
@@ -10864,7 +10875,7 @@
       <c r="M448" s="9" t="n"/>
       <c r="N448" s="9" t="n"/>
       <c r="O448" s="9" t="n"/>
-      <c r="P448" s="9" t="n"/>
+      <c r="P448" s="17" t="n"/>
       <c r="Q448" s="9" t="n"/>
       <c r="R448" s="9" t="n"/>
       <c r="S448" s="9" t="n"/>
@@ -10885,7 +10896,7 @@
       <c r="M449" s="9" t="n"/>
       <c r="N449" s="9" t="n"/>
       <c r="O449" s="9" t="n"/>
-      <c r="P449" s="9" t="n"/>
+      <c r="P449" s="17" t="n"/>
       <c r="Q449" s="9" t="n"/>
       <c r="R449" s="9" t="n"/>
       <c r="S449" s="9" t="n"/>
@@ -10906,7 +10917,7 @@
       <c r="M450" s="9" t="n"/>
       <c r="N450" s="9" t="n"/>
       <c r="O450" s="9" t="n"/>
-      <c r="P450" s="9" t="n"/>
+      <c r="P450" s="17" t="n"/>
       <c r="Q450" s="9" t="n"/>
       <c r="R450" s="9" t="n"/>
       <c r="S450" s="9" t="n"/>
@@ -10927,7 +10938,7 @@
       <c r="M451" s="9" t="n"/>
       <c r="N451" s="9" t="n"/>
       <c r="O451" s="9" t="n"/>
-      <c r="P451" s="9" t="n"/>
+      <c r="P451" s="17" t="n"/>
       <c r="Q451" s="9" t="n"/>
       <c r="R451" s="9" t="n"/>
       <c r="S451" s="9" t="n"/>
@@ -10948,7 +10959,7 @@
       <c r="M452" s="9" t="n"/>
       <c r="N452" s="9" t="n"/>
       <c r="O452" s="9" t="n"/>
-      <c r="P452" s="9" t="n"/>
+      <c r="P452" s="17" t="n"/>
       <c r="Q452" s="9" t="n"/>
       <c r="R452" s="9" t="n"/>
       <c r="S452" s="9" t="n"/>
@@ -10969,7 +10980,7 @@
       <c r="M453" s="9" t="n"/>
       <c r="N453" s="9" t="n"/>
       <c r="O453" s="9" t="n"/>
-      <c r="P453" s="9" t="n"/>
+      <c r="P453" s="17" t="n"/>
       <c r="Q453" s="9" t="n"/>
       <c r="R453" s="9" t="n"/>
       <c r="S453" s="9" t="n"/>
@@ -10990,7 +11001,7 @@
       <c r="M454" s="9" t="n"/>
       <c r="N454" s="9" t="n"/>
       <c r="O454" s="9" t="n"/>
-      <c r="P454" s="9" t="n"/>
+      <c r="P454" s="17" t="n"/>
       <c r="Q454" s="9" t="n"/>
       <c r="R454" s="9" t="n"/>
       <c r="S454" s="9" t="n"/>
@@ -11011,7 +11022,7 @@
       <c r="M455" s="9" t="n"/>
       <c r="N455" s="9" t="n"/>
       <c r="O455" s="9" t="n"/>
-      <c r="P455" s="9" t="n"/>
+      <c r="P455" s="17" t="n"/>
       <c r="Q455" s="9" t="n"/>
       <c r="R455" s="9" t="n"/>
       <c r="S455" s="9" t="n"/>
@@ -11032,7 +11043,7 @@
       <c r="M456" s="9" t="n"/>
       <c r="N456" s="9" t="n"/>
       <c r="O456" s="9" t="n"/>
-      <c r="P456" s="9" t="n"/>
+      <c r="P456" s="17" t="n"/>
       <c r="Q456" s="9" t="n"/>
       <c r="R456" s="9" t="n"/>
       <c r="S456" s="9" t="n"/>
@@ -11053,7 +11064,7 @@
       <c r="M457" s="9" t="n"/>
       <c r="N457" s="9" t="n"/>
       <c r="O457" s="9" t="n"/>
-      <c r="P457" s="9" t="n"/>
+      <c r="P457" s="17" t="n"/>
       <c r="Q457" s="9" t="n"/>
       <c r="R457" s="9" t="n"/>
       <c r="S457" s="9" t="n"/>
@@ -11074,7 +11085,7 @@
       <c r="M458" s="9" t="n"/>
       <c r="N458" s="9" t="n"/>
       <c r="O458" s="9" t="n"/>
-      <c r="P458" s="9" t="n"/>
+      <c r="P458" s="17" t="n"/>
       <c r="Q458" s="9" t="n"/>
       <c r="R458" s="9" t="n"/>
       <c r="S458" s="9" t="n"/>
@@ -11095,7 +11106,7 @@
       <c r="M459" s="9" t="n"/>
       <c r="N459" s="9" t="n"/>
       <c r="O459" s="9" t="n"/>
-      <c r="P459" s="9" t="n"/>
+      <c r="P459" s="17" t="n"/>
       <c r="Q459" s="9" t="n"/>
       <c r="R459" s="9" t="n"/>
       <c r="S459" s="9" t="n"/>
@@ -11116,7 +11127,7 @@
       <c r="M460" s="9" t="n"/>
       <c r="N460" s="9" t="n"/>
       <c r="O460" s="9" t="n"/>
-      <c r="P460" s="9" t="n"/>
+      <c r="P460" s="17" t="n"/>
       <c r="Q460" s="9" t="n"/>
       <c r="R460" s="9" t="n"/>
       <c r="S460" s="9" t="n"/>
@@ -11137,7 +11148,7 @@
       <c r="M461" s="9" t="n"/>
       <c r="N461" s="9" t="n"/>
       <c r="O461" s="9" t="n"/>
-      <c r="P461" s="9" t="n"/>
+      <c r="P461" s="17" t="n"/>
       <c r="Q461" s="9" t="n"/>
       <c r="R461" s="9" t="n"/>
       <c r="S461" s="9" t="n"/>
@@ -11158,7 +11169,7 @@
       <c r="M462" s="9" t="n"/>
       <c r="N462" s="9" t="n"/>
       <c r="O462" s="9" t="n"/>
-      <c r="P462" s="9" t="n"/>
+      <c r="P462" s="17" t="n"/>
       <c r="Q462" s="9" t="n"/>
       <c r="R462" s="9" t="n"/>
       <c r="S462" s="9" t="n"/>
@@ -11179,7 +11190,7 @@
       <c r="M463" s="9" t="n"/>
       <c r="N463" s="9" t="n"/>
       <c r="O463" s="9" t="n"/>
-      <c r="P463" s="9" t="n"/>
+      <c r="P463" s="17" t="n"/>
       <c r="Q463" s="9" t="n"/>
       <c r="R463" s="9" t="n"/>
       <c r="S463" s="9" t="n"/>
@@ -11200,7 +11211,7 @@
       <c r="M464" s="9" t="n"/>
       <c r="N464" s="9" t="n"/>
       <c r="O464" s="9" t="n"/>
-      <c r="P464" s="9" t="n"/>
+      <c r="P464" s="17" t="n"/>
       <c r="Q464" s="9" t="n"/>
       <c r="R464" s="9" t="n"/>
       <c r="S464" s="9" t="n"/>
@@ -11221,7 +11232,7 @@
       <c r="M465" s="9" t="n"/>
       <c r="N465" s="9" t="n"/>
       <c r="O465" s="9" t="n"/>
-      <c r="P465" s="9" t="n"/>
+      <c r="P465" s="17" t="n"/>
       <c r="Q465" s="9" t="n"/>
       <c r="R465" s="9" t="n"/>
       <c r="S465" s="9" t="n"/>
@@ -11242,7 +11253,7 @@
       <c r="M466" s="9" t="n"/>
       <c r="N466" s="9" t="n"/>
       <c r="O466" s="9" t="n"/>
-      <c r="P466" s="9" t="n"/>
+      <c r="P466" s="17" t="n"/>
       <c r="Q466" s="9" t="n"/>
       <c r="R466" s="9" t="n"/>
       <c r="S466" s="9" t="n"/>
@@ -11263,7 +11274,7 @@
       <c r="M467" s="9" t="n"/>
       <c r="N467" s="9" t="n"/>
       <c r="O467" s="9" t="n"/>
-      <c r="P467" s="9" t="n"/>
+      <c r="P467" s="17" t="n"/>
       <c r="Q467" s="9" t="n"/>
       <c r="R467" s="9" t="n"/>
       <c r="S467" s="9" t="n"/>
@@ -11284,7 +11295,7 @@
       <c r="M468" s="9" t="n"/>
       <c r="N468" s="9" t="n"/>
       <c r="O468" s="9" t="n"/>
-      <c r="P468" s="9" t="n"/>
+      <c r="P468" s="17" t="n"/>
       <c r="Q468" s="9" t="n"/>
       <c r="R468" s="9" t="n"/>
       <c r="S468" s="9" t="n"/>
@@ -11305,7 +11316,7 @@
       <c r="M469" s="9" t="n"/>
       <c r="N469" s="9" t="n"/>
       <c r="O469" s="9" t="n"/>
-      <c r="P469" s="9" t="n"/>
+      <c r="P469" s="17" t="n"/>
       <c r="Q469" s="9" t="n"/>
       <c r="R469" s="9" t="n"/>
       <c r="S469" s="9" t="n"/>
@@ -11326,7 +11337,7 @@
       <c r="M470" s="9" t="n"/>
       <c r="N470" s="9" t="n"/>
       <c r="O470" s="9" t="n"/>
-      <c r="P470" s="9" t="n"/>
+      <c r="P470" s="17" t="n"/>
       <c r="Q470" s="9" t="n"/>
       <c r="R470" s="9" t="n"/>
       <c r="S470" s="9" t="n"/>
@@ -11347,7 +11358,7 @@
       <c r="M471" s="9" t="n"/>
       <c r="N471" s="9" t="n"/>
       <c r="O471" s="9" t="n"/>
-      <c r="P471" s="9" t="n"/>
+      <c r="P471" s="17" t="n"/>
       <c r="Q471" s="9" t="n"/>
       <c r="R471" s="9" t="n"/>
       <c r="S471" s="9" t="n"/>
@@ -11368,7 +11379,7 @@
       <c r="M472" s="9" t="n"/>
       <c r="N472" s="9" t="n"/>
       <c r="O472" s="9" t="n"/>
-      <c r="P472" s="9" t="n"/>
+      <c r="P472" s="17" t="n"/>
       <c r="Q472" s="9" t="n"/>
       <c r="R472" s="9" t="n"/>
       <c r="S472" s="9" t="n"/>
@@ -11389,7 +11400,7 @@
       <c r="M473" s="9" t="n"/>
       <c r="N473" s="9" t="n"/>
       <c r="O473" s="9" t="n"/>
-      <c r="P473" s="9" t="n"/>
+      <c r="P473" s="17" t="n"/>
       <c r="Q473" s="9" t="n"/>
       <c r="R473" s="9" t="n"/>
       <c r="S473" s="9" t="n"/>
@@ -11410,7 +11421,7 @@
       <c r="M474" s="9" t="n"/>
       <c r="N474" s="9" t="n"/>
       <c r="O474" s="9" t="n"/>
-      <c r="P474" s="9" t="n"/>
+      <c r="P474" s="17" t="n"/>
       <c r="Q474" s="9" t="n"/>
       <c r="R474" s="9" t="n"/>
       <c r="S474" s="9" t="n"/>
@@ -11431,7 +11442,7 @@
       <c r="M475" s="9" t="n"/>
       <c r="N475" s="9" t="n"/>
       <c r="O475" s="9" t="n"/>
-      <c r="P475" s="9" t="n"/>
+      <c r="P475" s="17" t="n"/>
       <c r="Q475" s="9" t="n"/>
       <c r="R475" s="9" t="n"/>
       <c r="S475" s="9" t="n"/>
@@ -11452,7 +11463,7 @@
       <c r="M476" s="9" t="n"/>
       <c r="N476" s="9" t="n"/>
       <c r="O476" s="9" t="n"/>
-      <c r="P476" s="9" t="n"/>
+      <c r="P476" s="17" t="n"/>
       <c r="Q476" s="9" t="n"/>
       <c r="R476" s="9" t="n"/>
       <c r="S476" s="9" t="n"/>
@@ -11473,7 +11484,7 @@
       <c r="M477" s="9" t="n"/>
       <c r="N477" s="9" t="n"/>
       <c r="O477" s="9" t="n"/>
-      <c r="P477" s="9" t="n"/>
+      <c r="P477" s="17" t="n"/>
       <c r="Q477" s="9" t="n"/>
       <c r="R477" s="9" t="n"/>
       <c r="S477" s="9" t="n"/>
@@ -11494,7 +11505,7 @@
       <c r="M478" s="9" t="n"/>
       <c r="N478" s="9" t="n"/>
       <c r="O478" s="9" t="n"/>
-      <c r="P478" s="9" t="n"/>
+      <c r="P478" s="17" t="n"/>
       <c r="Q478" s="9" t="n"/>
       <c r="R478" s="9" t="n"/>
       <c r="S478" s="9" t="n"/>
@@ -11515,7 +11526,7 @@
       <c r="M479" s="9" t="n"/>
       <c r="N479" s="9" t="n"/>
       <c r="O479" s="9" t="n"/>
-      <c r="P479" s="9" t="n"/>
+      <c r="P479" s="17" t="n"/>
       <c r="Q479" s="9" t="n"/>
       <c r="R479" s="9" t="n"/>
       <c r="S479" s="9" t="n"/>
@@ -11536,7 +11547,7 @@
       <c r="M480" s="9" t="n"/>
       <c r="N480" s="9" t="n"/>
       <c r="O480" s="9" t="n"/>
-      <c r="P480" s="9" t="n"/>
+      <c r="P480" s="17" t="n"/>
       <c r="Q480" s="9" t="n"/>
       <c r="R480" s="9" t="n"/>
       <c r="S480" s="9" t="n"/>
@@ -11557,7 +11568,7 @@
       <c r="M481" s="9" t="n"/>
       <c r="N481" s="9" t="n"/>
       <c r="O481" s="9" t="n"/>
-      <c r="P481" s="9" t="n"/>
+      <c r="P481" s="17" t="n"/>
       <c r="Q481" s="9" t="n"/>
       <c r="R481" s="9" t="n"/>
       <c r="S481" s="9" t="n"/>
@@ -11578,7 +11589,7 @@
       <c r="M482" s="9" t="n"/>
       <c r="N482" s="9" t="n"/>
       <c r="O482" s="9" t="n"/>
-      <c r="P482" s="9" t="n"/>
+      <c r="P482" s="17" t="n"/>
       <c r="Q482" s="9" t="n"/>
       <c r="R482" s="9" t="n"/>
       <c r="S482" s="9" t="n"/>
@@ -11599,7 +11610,7 @@
       <c r="M483" s="9" t="n"/>
       <c r="N483" s="9" t="n"/>
       <c r="O483" s="9" t="n"/>
-      <c r="P483" s="9" t="n"/>
+      <c r="P483" s="17" t="n"/>
       <c r="Q483" s="9" t="n"/>
       <c r="R483" s="9" t="n"/>
       <c r="S483" s="9" t="n"/>
@@ -11620,7 +11631,7 @@
       <c r="M484" s="9" t="n"/>
       <c r="N484" s="9" t="n"/>
       <c r="O484" s="9" t="n"/>
-      <c r="P484" s="9" t="n"/>
+      <c r="P484" s="17" t="n"/>
       <c r="Q484" s="9" t="n"/>
       <c r="R484" s="9" t="n"/>
       <c r="S484" s="9" t="n"/>
@@ -11641,7 +11652,7 @@
       <c r="M485" s="9" t="n"/>
       <c r="N485" s="9" t="n"/>
       <c r="O485" s="9" t="n"/>
-      <c r="P485" s="9" t="n"/>
+      <c r="P485" s="17" t="n"/>
       <c r="Q485" s="9" t="n"/>
       <c r="R485" s="9" t="n"/>
       <c r="S485" s="9" t="n"/>
@@ -11662,7 +11673,7 @@
       <c r="M486" s="9" t="n"/>
       <c r="N486" s="9" t="n"/>
       <c r="O486" s="9" t="n"/>
-      <c r="P486" s="9" t="n"/>
+      <c r="P486" s="17" t="n"/>
       <c r="Q486" s="9" t="n"/>
       <c r="R486" s="9" t="n"/>
       <c r="S486" s="9" t="n"/>
@@ -11683,7 +11694,7 @@
       <c r="M487" s="9" t="n"/>
       <c r="N487" s="9" t="n"/>
       <c r="O487" s="9" t="n"/>
-      <c r="P487" s="9" t="n"/>
+      <c r="P487" s="17" t="n"/>
       <c r="Q487" s="9" t="n"/>
       <c r="R487" s="9" t="n"/>
       <c r="S487" s="9" t="n"/>
@@ -11704,7 +11715,7 @@
       <c r="M488" s="9" t="n"/>
       <c r="N488" s="9" t="n"/>
       <c r="O488" s="9" t="n"/>
-      <c r="P488" s="9" t="n"/>
+      <c r="P488" s="17" t="n"/>
       <c r="Q488" s="9" t="n"/>
       <c r="R488" s="9" t="n"/>
       <c r="S488" s="9" t="n"/>
@@ -11725,7 +11736,7 @@
       <c r="M489" s="9" t="n"/>
       <c r="N489" s="9" t="n"/>
       <c r="O489" s="9" t="n"/>
-      <c r="P489" s="9" t="n"/>
+      <c r="P489" s="17" t="n"/>
       <c r="Q489" s="9" t="n"/>
       <c r="R489" s="9" t="n"/>
       <c r="S489" s="9" t="n"/>
@@ -11746,7 +11757,7 @@
       <c r="M490" s="9" t="n"/>
       <c r="N490" s="9" t="n"/>
       <c r="O490" s="9" t="n"/>
-      <c r="P490" s="9" t="n"/>
+      <c r="P490" s="17" t="n"/>
       <c r="Q490" s="9" t="n"/>
       <c r="R490" s="9" t="n"/>
       <c r="S490" s="9" t="n"/>
@@ -11767,7 +11778,7 @@
       <c r="M491" s="9" t="n"/>
       <c r="N491" s="9" t="n"/>
       <c r="O491" s="9" t="n"/>
-      <c r="P491" s="9" t="n"/>
+      <c r="P491" s="17" t="n"/>
       <c r="Q491" s="9" t="n"/>
       <c r="R491" s="9" t="n"/>
       <c r="S491" s="9" t="n"/>
@@ -11788,7 +11799,7 @@
       <c r="M492" s="9" t="n"/>
       <c r="N492" s="9" t="n"/>
       <c r="O492" s="9" t="n"/>
-      <c r="P492" s="9" t="n"/>
+      <c r="P492" s="17" t="n"/>
       <c r="Q492" s="9" t="n"/>
       <c r="R492" s="9" t="n"/>
       <c r="S492" s="9" t="n"/>
@@ -11809,7 +11820,7 @@
       <c r="M493" s="9" t="n"/>
       <c r="N493" s="9" t="n"/>
       <c r="O493" s="9" t="n"/>
-      <c r="P493" s="9" t="n"/>
+      <c r="P493" s="17" t="n"/>
       <c r="Q493" s="9" t="n"/>
       <c r="R493" s="9" t="n"/>
       <c r="S493" s="9" t="n"/>
@@ -11830,7 +11841,7 @@
       <c r="M494" s="9" t="n"/>
       <c r="N494" s="9" t="n"/>
       <c r="O494" s="9" t="n"/>
-      <c r="P494" s="9" t="n"/>
+      <c r="P494" s="17" t="n"/>
       <c r="Q494" s="9" t="n"/>
       <c r="R494" s="9" t="n"/>
       <c r="S494" s="9" t="n"/>
@@ -11851,7 +11862,7 @@
       <c r="M495" s="9" t="n"/>
       <c r="N495" s="9" t="n"/>
       <c r="O495" s="9" t="n"/>
-      <c r="P495" s="9" t="n"/>
+      <c r="P495" s="17" t="n"/>
       <c r="Q495" s="9" t="n"/>
       <c r="R495" s="9" t="n"/>
       <c r="S495" s="9" t="n"/>
@@ -11872,7 +11883,7 @@
       <c r="M496" s="9" t="n"/>
       <c r="N496" s="9" t="n"/>
       <c r="O496" s="9" t="n"/>
-      <c r="P496" s="9" t="n"/>
+      <c r="P496" s="17" t="n"/>
       <c r="Q496" s="9" t="n"/>
       <c r="R496" s="9" t="n"/>
       <c r="S496" s="9" t="n"/>
@@ -11893,7 +11904,7 @@
       <c r="M497" s="9" t="n"/>
       <c r="N497" s="9" t="n"/>
       <c r="O497" s="9" t="n"/>
-      <c r="P497" s="9" t="n"/>
+      <c r="P497" s="17" t="n"/>
       <c r="Q497" s="9" t="n"/>
       <c r="R497" s="9" t="n"/>
       <c r="S497" s="9" t="n"/>
@@ -11914,7 +11925,7 @@
       <c r="M498" s="9" t="n"/>
       <c r="N498" s="9" t="n"/>
       <c r="O498" s="9" t="n"/>
-      <c r="P498" s="9" t="n"/>
+      <c r="P498" s="17" t="n"/>
       <c r="Q498" s="9" t="n"/>
       <c r="R498" s="9" t="n"/>
       <c r="S498" s="9" t="n"/>
@@ -11935,7 +11946,7 @@
       <c r="M499" s="9" t="n"/>
       <c r="N499" s="9" t="n"/>
       <c r="O499" s="9" t="n"/>
-      <c r="P499" s="9" t="n"/>
+      <c r="P499" s="17" t="n"/>
       <c r="Q499" s="9" t="n"/>
       <c r="R499" s="9" t="n"/>
       <c r="S499" s="9" t="n"/>
@@ -11956,7 +11967,7 @@
       <c r="M500" s="9" t="n"/>
       <c r="N500" s="9" t="n"/>
       <c r="O500" s="9" t="n"/>
-      <c r="P500" s="9" t="n"/>
+      <c r="P500" s="17" t="n"/>
       <c r="Q500" s="9" t="n"/>
       <c r="R500" s="9" t="n"/>
       <c r="S500" s="9" t="n"/>
@@ -11977,13 +11988,13 @@
       <c r="M501" s="9" t="n"/>
       <c r="N501" s="9" t="n"/>
       <c r="O501" s="9" t="n"/>
-      <c r="P501" s="9" t="n"/>
+      <c r="P501" s="17" t="n"/>
       <c r="Q501" s="9" t="n"/>
       <c r="R501" s="9" t="n"/>
       <c r="S501" s="9" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="9">
     <dataValidation sqref="I2:I501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Codebook value" error="Pick a value from the list." type="list">
       <formula1>'Error codebook'!$A$2:$A$10</formula1>
     </dataValidation>
@@ -12007,6 +12018,9 @@
     </dataValidation>
     <dataValidation sqref="P2:P501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Codebook value" error="Pick a value from the list." type="list">
       <formula1>"yes,no,n/a"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1,2,3,4,5,6,7,8,5',6',7',8',pilot"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: log bugs, pre-code stuck events for verification
D74. Until the standard harness is frozen, issues from live runs go in
docs/bugs.md (seeded with B1-B5 from today) and their stuck events are
coded in the workbook's Annotations sheet, marked pre-freeze. In grid
runs Claude pre-codes every stuck event as a draft and the research lead
verifies it: annotations gain a verified_by field (workbook column T),
and export/validate report rows awaiting verification. The stopped
cell-5 run's six stuck events are drafted (E08 for the FLE lab bug; E09
where the backstop fired with nothing wrong).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/codebook-v0.xlsx
+++ b/docs/codebook-v0.xlsx
@@ -628,7 +628,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>1) Open the run's trajectory; list its intervention records (each is one stuck event). 2) Read the ~5 steps before the event: the policy code, execution errors and verifier reasons. 3) Pick ONE primary error code (the root cause) and optionally one secondary. 4) If a human answered, code the guidance the same way (the text itself is copied from the trajectory on export). 5) Leave 'unstuck' blank - it is computed on export (rule below). 6) Record codebook version and your initials. 7) Export and validate: python -m factorio_maxxing.annotations export</t>
+          <t>1) Open the run's trajectory; list its intervention records (each is one stuck event). 2) Read the ~5 steps before the event: the policy code, execution errors and verifier reasons. 3) Pick ONE primary error code (the root cause) and optionally one secondary. 4) If a human answered, code the guidance the same way (the text itself is copied from the trajectory on export). 5) Leave 'unstuck' blank - it is computed on export (rule below). 6) Record codebook version and annotator. 7) Export and validate: python -m factorio_maxxing.annotations export. From the grid runs on (D74), Claude pre-codes every stuck event as 'Claude (draft)' and the research lead verifies each row: correct it if needed, then put your initials in 'verified by'. Only verified rows are the catalogue.</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Yellow cells are the ones you fill in (Annotations sheet, and k above). Grey column P is computed on export. Columns C, G, H and N are for reading only: export copies policy model, intervention_index, stuck_reason and guidance text verbatim from the trajectory. The 'Worked examples' sheet shows the expected format with real stuck events from the goal-5 rescue run.</t>
+          <t>Yellow cells are the ones you fill in (Annotations sheet, and k above). Grey column P is computed on export. Columns C, G, H and N are for reading only: export copies policy model, intervention_index, stuck_reason and guidance text verbatim from the trajectory. 'verified by' (column T) holds the initials of whoever checked a draft row. Rows whose notes say 'pre-freeze' come from runs before the standard harness was frozen and are excluded from grid analysis. The 'Worked examples' sheet shows the expected format with real stuck events from the goal-5 rescue run.</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S501"/>
+  <dimension ref="A1:T501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1394,6 +1394,7 @@
     <col width="9" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
     <col width="28" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1492,132 +1493,435 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="T1" s="5" t="inlineStr">
+        <is>
+          <t>verified by</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="n"/>
-      <c r="B2" s="8" t="n"/>
-      <c r="C2" s="8" t="n"/>
-      <c r="D2" s="8" t="n"/>
-      <c r="E2" s="8" t="n"/>
-      <c r="F2" s="8" t="n"/>
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>20261021T162318-3e77267c</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="n">
+        <v>19</v>
+      </c>
       <c r="G2" s="8" t="n"/>
-      <c r="H2" s="8" t="n"/>
-      <c r="I2" s="8" t="n"/>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>E09</t>
+        </is>
+      </c>
       <c r="J2" s="8" t="n"/>
-      <c r="K2" s="8" t="n"/>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>No error found: steps 15-19 the agent was building copper/iron drills and furnaces and collecting plates normally. The 20-step backstop fired (D67) without the agent being stuck - candidate for a v1 'false alarm' code.</t>
+        </is>
+      </c>
       <c r="L2" s="8" t="n"/>
       <c r="M2" s="8" t="n"/>
       <c r="N2" s="8" t="n"/>
       <c r="O2" s="8" t="n"/>
       <c r="P2" s="16" t="n"/>
-      <c r="Q2" s="8" t="n"/>
-      <c r="R2" s="8" t="n"/>
-      <c r="S2" s="8" t="n"/>
+      <c r="Q2" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R2" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S2" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze pilot run (harness a5c45df, stopped at step 137); exclude from grid analysis.</t>
+        </is>
+      </c>
+      <c r="T2" s="8" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="n"/>
-      <c r="B3" s="8" t="n"/>
-      <c r="C3" s="8" t="n"/>
-      <c r="D3" s="8" t="n"/>
-      <c r="E3" s="8" t="n"/>
-      <c r="F3" s="8" t="n"/>
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>20261021T162318-3e77267c</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>39</v>
+      </c>
       <c r="G3" s="8" t="n"/>
-      <c r="H3" s="8" t="n"/>
-      <c r="I3" s="8" t="n"/>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>E09</t>
+        </is>
+      </c>
       <c r="J3" s="8" t="n"/>
-      <c r="K3" s="8" t="n"/>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>No clear error: steps 35-39 normal progress (automation researched at step 33, logistics research running, assemblers crafted); coal ran out (coal=0) at step 39. Backstop fired (D67) - candidate for a v1 'false alarm' code.</t>
+        </is>
+      </c>
       <c r="L3" s="8" t="n"/>
       <c r="M3" s="8" t="n"/>
       <c r="N3" s="8" t="n"/>
       <c r="O3" s="8" t="n"/>
       <c r="P3" s="16" t="n"/>
-      <c r="Q3" s="8" t="n"/>
-      <c r="R3" s="8" t="n"/>
-      <c r="S3" s="8" t="n"/>
+      <c r="Q3" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R3" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S3" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze pilot run (harness a5c45df, stopped at step 137); exclude from grid analysis.</t>
+        </is>
+      </c>
+      <c r="T3" s="8" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="n"/>
-      <c r="B4" s="8" t="n"/>
-      <c r="C4" s="8" t="n"/>
-      <c r="D4" s="8" t="n"/>
-      <c r="E4" s="8" t="n"/>
-      <c r="F4" s="8" t="n"/>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>20261021T162318-3e77267c</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>59</v>
+      </c>
       <c r="G4" s="8" t="n"/>
-      <c r="H4" s="8" t="n"/>
-      <c r="I4" s="8" t="n"/>
-      <c r="J4" s="8" t="n"/>
-      <c r="K4" s="8" t="n"/>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>E08</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>E06</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>FLE bug B1 (D73): research set to logistic-science-pack at step 45, after which FLE drops every lab from get_entities/get_entity/place_entity read-back. Steps 55-59: place_entity reports 'Could not place lab' though the lab leaves inventory; get_entities returns no labs; the agent re-crafts and re-places.</t>
+        </is>
+      </c>
       <c r="L4" s="8" t="n"/>
       <c r="M4" s="8" t="n"/>
       <c r="N4" s="8" t="n"/>
       <c r="O4" s="8" t="n"/>
       <c r="P4" s="16" t="n"/>
-      <c r="Q4" s="8" t="n"/>
-      <c r="R4" s="8" t="n"/>
-      <c r="S4" s="8" t="n"/>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R4" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S4" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze pilot run (harness a5c45df, stopped at step 137); exclude from grid analysis. Environment attribution.</t>
+        </is>
+      </c>
+      <c r="T4" s="8" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n"/>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="8" t="n"/>
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>20261021T162318-3e77267c</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>79</v>
+      </c>
       <c r="G5" s="8" t="n"/>
-      <c r="H5" s="8" t="n"/>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="8" t="n"/>
-      <c r="K5" s="8" t="n"/>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>E08</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>E06</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>FLE bug B1 (D73) continuing: steps 76-79 craft lab, placement 'fails', get_entities finds no labs anywhere ('Labs in world: []').</t>
+        </is>
+      </c>
       <c r="L5" s="8" t="n"/>
       <c r="M5" s="8" t="n"/>
       <c r="N5" s="8" t="n"/>
       <c r="O5" s="8" t="n"/>
       <c r="P5" s="16" t="n"/>
-      <c r="Q5" s="8" t="n"/>
-      <c r="R5" s="8" t="n"/>
-      <c r="S5" s="8" t="n"/>
+      <c r="Q5" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R5" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S5" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze pilot run (harness a5c45df, stopped at step 137); exclude from grid analysis. Environment attribution.</t>
+        </is>
+      </c>
+      <c r="T5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="n"/>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="8" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="8" t="n"/>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>20261021T162318-3e77267c</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>99</v>
+      </c>
       <c r="G6" s="8" t="n"/>
-      <c r="H6" s="8" t="n"/>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="8" t="n"/>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>E08</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>E06</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>FLE bug B1 (D73) continuing: steps 95-99 inspects the 'failed' spot (empty to it), crafts another lab, places again. 20+ invisible unpowered labs on the map.</t>
+        </is>
+      </c>
       <c r="L6" s="8" t="n"/>
       <c r="M6" s="8" t="n"/>
       <c r="N6" s="8" t="n"/>
       <c r="O6" s="8" t="n"/>
       <c r="P6" s="16" t="n"/>
-      <c r="Q6" s="8" t="n"/>
-      <c r="R6" s="8" t="n"/>
-      <c r="S6" s="8" t="n"/>
+      <c r="Q6" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R6" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S6" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze pilot run (harness a5c45df, stopped at step 137); exclude from grid analysis. Environment attribution.</t>
+        </is>
+      </c>
+      <c r="T6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n"/>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>20261021T162318-3e77267c</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>119</v>
+      </c>
       <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8" t="n"/>
-      <c r="K7" s="8" t="n"/>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>E08</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>E06</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>FLE bug B1 (D73) continuing: steps 115-119 refuels drills, crafts gears and yet another lab. 28 invisible labs on the map by the end of the run.</t>
+        </is>
+      </c>
       <c r="L7" s="8" t="n"/>
       <c r="M7" s="8" t="n"/>
       <c r="N7" s="8" t="n"/>
       <c r="O7" s="8" t="n"/>
       <c r="P7" s="16" t="n"/>
-      <c r="Q7" s="8" t="n"/>
-      <c r="R7" s="8" t="n"/>
-      <c r="S7" s="8" t="n"/>
+      <c r="Q7" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R7" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S7" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze pilot run (harness a5c45df, stopped at step 137); exclude from grid analysis. Environment attribution.</t>
+        </is>
+      </c>
+      <c r="T7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n"/>
@@ -1639,6 +1943,7 @@
       <c r="Q8" s="8" t="n"/>
       <c r="R8" s="8" t="n"/>
       <c r="S8" s="8" t="n"/>
+      <c r="T8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n"/>
@@ -1660,6 +1965,7 @@
       <c r="Q9" s="8" t="n"/>
       <c r="R9" s="8" t="n"/>
       <c r="S9" s="8" t="n"/>
+      <c r="T9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n"/>
@@ -1681,6 +1987,7 @@
       <c r="Q10" s="8" t="n"/>
       <c r="R10" s="8" t="n"/>
       <c r="S10" s="8" t="n"/>
+      <c r="T10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n"/>
@@ -1702,6 +2009,7 @@
       <c r="Q11" s="8" t="n"/>
       <c r="R11" s="8" t="n"/>
       <c r="S11" s="8" t="n"/>
+      <c r="T11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n"/>
@@ -1723,6 +2031,7 @@
       <c r="Q12" s="8" t="n"/>
       <c r="R12" s="8" t="n"/>
       <c r="S12" s="8" t="n"/>
+      <c r="T12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n"/>
@@ -1744,6 +2053,7 @@
       <c r="Q13" s="8" t="n"/>
       <c r="R13" s="8" t="n"/>
       <c r="S13" s="8" t="n"/>
+      <c r="T13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n"/>
@@ -1765,6 +2075,7 @@
       <c r="Q14" s="8" t="n"/>
       <c r="R14" s="8" t="n"/>
       <c r="S14" s="8" t="n"/>
+      <c r="T14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n"/>
@@ -1786,6 +2097,7 @@
       <c r="Q15" s="8" t="n"/>
       <c r="R15" s="8" t="n"/>
       <c r="S15" s="8" t="n"/>
+      <c r="T15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n"/>
@@ -1807,6 +2119,7 @@
       <c r="Q16" s="8" t="n"/>
       <c r="R16" s="8" t="n"/>
       <c r="S16" s="8" t="n"/>
+      <c r="T16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n"/>
@@ -1828,6 +2141,7 @@
       <c r="Q17" s="8" t="n"/>
       <c r="R17" s="8" t="n"/>
       <c r="S17" s="8" t="n"/>
+      <c r="T17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n"/>
@@ -1849,6 +2163,7 @@
       <c r="Q18" s="8" t="n"/>
       <c r="R18" s="8" t="n"/>
       <c r="S18" s="8" t="n"/>
+      <c r="T18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n"/>
@@ -1870,6 +2185,7 @@
       <c r="Q19" s="8" t="n"/>
       <c r="R19" s="8" t="n"/>
       <c r="S19" s="8" t="n"/>
+      <c r="T19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n"/>
@@ -1891,6 +2207,7 @@
       <c r="Q20" s="8" t="n"/>
       <c r="R20" s="8" t="n"/>
       <c r="S20" s="8" t="n"/>
+      <c r="T20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n"/>
@@ -1912,6 +2229,7 @@
       <c r="Q21" s="8" t="n"/>
       <c r="R21" s="8" t="n"/>
       <c r="S21" s="8" t="n"/>
+      <c r="T21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="n"/>
@@ -1933,6 +2251,7 @@
       <c r="Q22" s="9" t="n"/>
       <c r="R22" s="9" t="n"/>
       <c r="S22" s="9" t="n"/>
+      <c r="T22" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="n"/>
@@ -1954,6 +2273,7 @@
       <c r="Q23" s="9" t="n"/>
       <c r="R23" s="9" t="n"/>
       <c r="S23" s="9" t="n"/>
+      <c r="T23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="n"/>
@@ -1975,6 +2295,7 @@
       <c r="Q24" s="9" t="n"/>
       <c r="R24" s="9" t="n"/>
       <c r="S24" s="9" t="n"/>
+      <c r="T24" s="9" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n"/>
@@ -1996,6 +2317,7 @@
       <c r="Q25" s="9" t="n"/>
       <c r="R25" s="9" t="n"/>
       <c r="S25" s="9" t="n"/>
+      <c r="T25" s="9" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n"/>
@@ -2017,6 +2339,7 @@
       <c r="Q26" s="9" t="n"/>
       <c r="R26" s="9" t="n"/>
       <c r="S26" s="9" t="n"/>
+      <c r="T26" s="9" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n"/>
@@ -2038,6 +2361,7 @@
       <c r="Q27" s="9" t="n"/>
       <c r="R27" s="9" t="n"/>
       <c r="S27" s="9" t="n"/>
+      <c r="T27" s="9" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="9" t="n"/>
@@ -2059,6 +2383,7 @@
       <c r="Q28" s="9" t="n"/>
       <c r="R28" s="9" t="n"/>
       <c r="S28" s="9" t="n"/>
+      <c r="T28" s="9" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n"/>
@@ -2080,6 +2405,7 @@
       <c r="Q29" s="9" t="n"/>
       <c r="R29" s="9" t="n"/>
       <c r="S29" s="9" t="n"/>
+      <c r="T29" s="9" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="9" t="n"/>
@@ -2101,6 +2427,7 @@
       <c r="Q30" s="9" t="n"/>
       <c r="R30" s="9" t="n"/>
       <c r="S30" s="9" t="n"/>
+      <c r="T30" s="9" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n"/>
@@ -2122,6 +2449,7 @@
       <c r="Q31" s="9" t="n"/>
       <c r="R31" s="9" t="n"/>
       <c r="S31" s="9" t="n"/>
+      <c r="T31" s="9" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="9" t="n"/>
@@ -2143,6 +2471,7 @@
       <c r="Q32" s="9" t="n"/>
       <c r="R32" s="9" t="n"/>
       <c r="S32" s="9" t="n"/>
+      <c r="T32" s="9" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="9" t="n"/>
@@ -2164,6 +2493,7 @@
       <c r="Q33" s="9" t="n"/>
       <c r="R33" s="9" t="n"/>
       <c r="S33" s="9" t="n"/>
+      <c r="T33" s="9" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="9" t="n"/>
@@ -2185,6 +2515,7 @@
       <c r="Q34" s="9" t="n"/>
       <c r="R34" s="9" t="n"/>
       <c r="S34" s="9" t="n"/>
+      <c r="T34" s="9" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="9" t="n"/>
@@ -2206,6 +2537,7 @@
       <c r="Q35" s="9" t="n"/>
       <c r="R35" s="9" t="n"/>
       <c r="S35" s="9" t="n"/>
+      <c r="T35" s="9" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="9" t="n"/>
@@ -2227,6 +2559,7 @@
       <c r="Q36" s="9" t="n"/>
       <c r="R36" s="9" t="n"/>
       <c r="S36" s="9" t="n"/>
+      <c r="T36" s="9" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="9" t="n"/>
@@ -2248,6 +2581,7 @@
       <c r="Q37" s="9" t="n"/>
       <c r="R37" s="9" t="n"/>
       <c r="S37" s="9" t="n"/>
+      <c r="T37" s="9" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="9" t="n"/>
@@ -2269,6 +2603,7 @@
       <c r="Q38" s="9" t="n"/>
       <c r="R38" s="9" t="n"/>
       <c r="S38" s="9" t="n"/>
+      <c r="T38" s="9" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="9" t="n"/>
@@ -2290,6 +2625,7 @@
       <c r="Q39" s="9" t="n"/>
       <c r="R39" s="9" t="n"/>
       <c r="S39" s="9" t="n"/>
+      <c r="T39" s="9" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="9" t="n"/>
@@ -2311,6 +2647,7 @@
       <c r="Q40" s="9" t="n"/>
       <c r="R40" s="9" t="n"/>
       <c r="S40" s="9" t="n"/>
+      <c r="T40" s="9" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="9" t="n"/>
@@ -2332,6 +2669,7 @@
       <c r="Q41" s="9" t="n"/>
       <c r="R41" s="9" t="n"/>
       <c r="S41" s="9" t="n"/>
+      <c r="T41" s="9" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="9" t="n"/>
@@ -2353,6 +2691,7 @@
       <c r="Q42" s="9" t="n"/>
       <c r="R42" s="9" t="n"/>
       <c r="S42" s="9" t="n"/>
+      <c r="T42" s="9" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="9" t="n"/>
@@ -2374,6 +2713,7 @@
       <c r="Q43" s="9" t="n"/>
       <c r="R43" s="9" t="n"/>
       <c r="S43" s="9" t="n"/>
+      <c r="T43" s="9" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="9" t="n"/>
@@ -2395,6 +2735,7 @@
       <c r="Q44" s="9" t="n"/>
       <c r="R44" s="9" t="n"/>
       <c r="S44" s="9" t="n"/>
+      <c r="T44" s="9" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="9" t="n"/>
@@ -2416,6 +2757,7 @@
       <c r="Q45" s="9" t="n"/>
       <c r="R45" s="9" t="n"/>
       <c r="S45" s="9" t="n"/>
+      <c r="T45" s="9" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="9" t="n"/>
@@ -2437,6 +2779,7 @@
       <c r="Q46" s="9" t="n"/>
       <c r="R46" s="9" t="n"/>
       <c r="S46" s="9" t="n"/>
+      <c r="T46" s="9" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="9" t="n"/>
@@ -2458,6 +2801,7 @@
       <c r="Q47" s="9" t="n"/>
       <c r="R47" s="9" t="n"/>
       <c r="S47" s="9" t="n"/>
+      <c r="T47" s="9" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="9" t="n"/>
@@ -2479,6 +2823,7 @@
       <c r="Q48" s="9" t="n"/>
       <c r="R48" s="9" t="n"/>
       <c r="S48" s="9" t="n"/>
+      <c r="T48" s="9" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="9" t="n"/>
@@ -2500,6 +2845,7 @@
       <c r="Q49" s="9" t="n"/>
       <c r="R49" s="9" t="n"/>
       <c r="S49" s="9" t="n"/>
+      <c r="T49" s="9" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="9" t="n"/>
@@ -2521,6 +2867,7 @@
       <c r="Q50" s="9" t="n"/>
       <c r="R50" s="9" t="n"/>
       <c r="S50" s="9" t="n"/>
+      <c r="T50" s="9" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="9" t="n"/>
@@ -2542,6 +2889,7 @@
       <c r="Q51" s="9" t="n"/>
       <c r="R51" s="9" t="n"/>
       <c r="S51" s="9" t="n"/>
+      <c r="T51" s="9" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="9" t="n"/>
@@ -2563,6 +2911,7 @@
       <c r="Q52" s="9" t="n"/>
       <c r="R52" s="9" t="n"/>
       <c r="S52" s="9" t="n"/>
+      <c r="T52" s="9" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="9" t="n"/>
@@ -2584,6 +2933,7 @@
       <c r="Q53" s="9" t="n"/>
       <c r="R53" s="9" t="n"/>
       <c r="S53" s="9" t="n"/>
+      <c r="T53" s="9" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="9" t="n"/>
@@ -2605,6 +2955,7 @@
       <c r="Q54" s="9" t="n"/>
       <c r="R54" s="9" t="n"/>
       <c r="S54" s="9" t="n"/>
+      <c r="T54" s="9" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n"/>
@@ -2626,6 +2977,7 @@
       <c r="Q55" s="9" t="n"/>
       <c r="R55" s="9" t="n"/>
       <c r="S55" s="9" t="n"/>
+      <c r="T55" s="9" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="9" t="n"/>
@@ -2647,6 +2999,7 @@
       <c r="Q56" s="9" t="n"/>
       <c r="R56" s="9" t="n"/>
       <c r="S56" s="9" t="n"/>
+      <c r="T56" s="9" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="9" t="n"/>
@@ -2668,6 +3021,7 @@
       <c r="Q57" s="9" t="n"/>
       <c r="R57" s="9" t="n"/>
       <c r="S57" s="9" t="n"/>
+      <c r="T57" s="9" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="9" t="n"/>
@@ -2689,6 +3043,7 @@
       <c r="Q58" s="9" t="n"/>
       <c r="R58" s="9" t="n"/>
       <c r="S58" s="9" t="n"/>
+      <c r="T58" s="9" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="9" t="n"/>
@@ -2710,6 +3065,7 @@
       <c r="Q59" s="9" t="n"/>
       <c r="R59" s="9" t="n"/>
       <c r="S59" s="9" t="n"/>
+      <c r="T59" s="9" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="9" t="n"/>
@@ -2731,6 +3087,7 @@
       <c r="Q60" s="9" t="n"/>
       <c r="R60" s="9" t="n"/>
       <c r="S60" s="9" t="n"/>
+      <c r="T60" s="9" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n"/>
@@ -2752,6 +3109,7 @@
       <c r="Q61" s="9" t="n"/>
       <c r="R61" s="9" t="n"/>
       <c r="S61" s="9" t="n"/>
+      <c r="T61" s="9" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="9" t="n"/>
@@ -2773,6 +3131,7 @@
       <c r="Q62" s="9" t="n"/>
       <c r="R62" s="9" t="n"/>
       <c r="S62" s="9" t="n"/>
+      <c r="T62" s="9" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="9" t="n"/>
@@ -2794,6 +3153,7 @@
       <c r="Q63" s="9" t="n"/>
       <c r="R63" s="9" t="n"/>
       <c r="S63" s="9" t="n"/>
+      <c r="T63" s="9" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="9" t="n"/>
@@ -2815,6 +3175,7 @@
       <c r="Q64" s="9" t="n"/>
       <c r="R64" s="9" t="n"/>
       <c r="S64" s="9" t="n"/>
+      <c r="T64" s="9" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="9" t="n"/>
@@ -2836,6 +3197,7 @@
       <c r="Q65" s="9" t="n"/>
       <c r="R65" s="9" t="n"/>
       <c r="S65" s="9" t="n"/>
+      <c r="T65" s="9" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="9" t="n"/>
@@ -2857,6 +3219,7 @@
       <c r="Q66" s="9" t="n"/>
       <c r="R66" s="9" t="n"/>
       <c r="S66" s="9" t="n"/>
+      <c r="T66" s="9" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="9" t="n"/>
@@ -2878,6 +3241,7 @@
       <c r="Q67" s="9" t="n"/>
       <c r="R67" s="9" t="n"/>
       <c r="S67" s="9" t="n"/>
+      <c r="T67" s="9" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="9" t="n"/>
@@ -2899,6 +3263,7 @@
       <c r="Q68" s="9" t="n"/>
       <c r="R68" s="9" t="n"/>
       <c r="S68" s="9" t="n"/>
+      <c r="T68" s="9" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="9" t="n"/>
@@ -2920,6 +3285,7 @@
       <c r="Q69" s="9" t="n"/>
       <c r="R69" s="9" t="n"/>
       <c r="S69" s="9" t="n"/>
+      <c r="T69" s="9" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="9" t="n"/>
@@ -2941,6 +3307,7 @@
       <c r="Q70" s="9" t="n"/>
       <c r="R70" s="9" t="n"/>
       <c r="S70" s="9" t="n"/>
+      <c r="T70" s="9" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="9" t="n"/>
@@ -2962,6 +3329,7 @@
       <c r="Q71" s="9" t="n"/>
       <c r="R71" s="9" t="n"/>
       <c r="S71" s="9" t="n"/>
+      <c r="T71" s="9" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="9" t="n"/>
@@ -2983,6 +3351,7 @@
       <c r="Q72" s="9" t="n"/>
       <c r="R72" s="9" t="n"/>
       <c r="S72" s="9" t="n"/>
+      <c r="T72" s="9" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="9" t="n"/>
@@ -3004,6 +3373,7 @@
       <c r="Q73" s="9" t="n"/>
       <c r="R73" s="9" t="n"/>
       <c r="S73" s="9" t="n"/>
+      <c r="T73" s="9" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="n"/>
@@ -3025,6 +3395,7 @@
       <c r="Q74" s="9" t="n"/>
       <c r="R74" s="9" t="n"/>
       <c r="S74" s="9" t="n"/>
+      <c r="T74" s="9" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="9" t="n"/>
@@ -3046,6 +3417,7 @@
       <c r="Q75" s="9" t="n"/>
       <c r="R75" s="9" t="n"/>
       <c r="S75" s="9" t="n"/>
+      <c r="T75" s="9" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="9" t="n"/>
@@ -3067,6 +3439,7 @@
       <c r="Q76" s="9" t="n"/>
       <c r="R76" s="9" t="n"/>
       <c r="S76" s="9" t="n"/>
+      <c r="T76" s="9" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="9" t="n"/>
@@ -3088,6 +3461,7 @@
       <c r="Q77" s="9" t="n"/>
       <c r="R77" s="9" t="n"/>
       <c r="S77" s="9" t="n"/>
+      <c r="T77" s="9" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="9" t="n"/>
@@ -3109,6 +3483,7 @@
       <c r="Q78" s="9" t="n"/>
       <c r="R78" s="9" t="n"/>
       <c r="S78" s="9" t="n"/>
+      <c r="T78" s="9" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="9" t="n"/>
@@ -3130,6 +3505,7 @@
       <c r="Q79" s="9" t="n"/>
       <c r="R79" s="9" t="n"/>
       <c r="S79" s="9" t="n"/>
+      <c r="T79" s="9" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="9" t="n"/>
@@ -3151,6 +3527,7 @@
       <c r="Q80" s="9" t="n"/>
       <c r="R80" s="9" t="n"/>
       <c r="S80" s="9" t="n"/>
+      <c r="T80" s="9" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="9" t="n"/>
@@ -3172,6 +3549,7 @@
       <c r="Q81" s="9" t="n"/>
       <c r="R81" s="9" t="n"/>
       <c r="S81" s="9" t="n"/>
+      <c r="T81" s="9" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="9" t="n"/>
@@ -3193,6 +3571,7 @@
       <c r="Q82" s="9" t="n"/>
       <c r="R82" s="9" t="n"/>
       <c r="S82" s="9" t="n"/>
+      <c r="T82" s="9" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="9" t="n"/>
@@ -3214,6 +3593,7 @@
       <c r="Q83" s="9" t="n"/>
       <c r="R83" s="9" t="n"/>
       <c r="S83" s="9" t="n"/>
+      <c r="T83" s="9" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="9" t="n"/>
@@ -3235,6 +3615,7 @@
       <c r="Q84" s="9" t="n"/>
       <c r="R84" s="9" t="n"/>
       <c r="S84" s="9" t="n"/>
+      <c r="T84" s="9" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="9" t="n"/>
@@ -3256,6 +3637,7 @@
       <c r="Q85" s="9" t="n"/>
       <c r="R85" s="9" t="n"/>
       <c r="S85" s="9" t="n"/>
+      <c r="T85" s="9" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="9" t="n"/>
@@ -3277,6 +3659,7 @@
       <c r="Q86" s="9" t="n"/>
       <c r="R86" s="9" t="n"/>
       <c r="S86" s="9" t="n"/>
+      <c r="T86" s="9" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="9" t="n"/>
@@ -3298,6 +3681,7 @@
       <c r="Q87" s="9" t="n"/>
       <c r="R87" s="9" t="n"/>
       <c r="S87" s="9" t="n"/>
+      <c r="T87" s="9" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="9" t="n"/>
@@ -3319,6 +3703,7 @@
       <c r="Q88" s="9" t="n"/>
       <c r="R88" s="9" t="n"/>
       <c r="S88" s="9" t="n"/>
+      <c r="T88" s="9" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="9" t="n"/>
@@ -3340,6 +3725,7 @@
       <c r="Q89" s="9" t="n"/>
       <c r="R89" s="9" t="n"/>
       <c r="S89" s="9" t="n"/>
+      <c r="T89" s="9" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="9" t="n"/>
@@ -3361,6 +3747,7 @@
       <c r="Q90" s="9" t="n"/>
       <c r="R90" s="9" t="n"/>
       <c r="S90" s="9" t="n"/>
+      <c r="T90" s="9" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="9" t="n"/>
@@ -3382,6 +3769,7 @@
       <c r="Q91" s="9" t="n"/>
       <c r="R91" s="9" t="n"/>
       <c r="S91" s="9" t="n"/>
+      <c r="T91" s="9" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="9" t="n"/>
@@ -3403,6 +3791,7 @@
       <c r="Q92" s="9" t="n"/>
       <c r="R92" s="9" t="n"/>
       <c r="S92" s="9" t="n"/>
+      <c r="T92" s="9" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="9" t="n"/>
@@ -3424,6 +3813,7 @@
       <c r="Q93" s="9" t="n"/>
       <c r="R93" s="9" t="n"/>
       <c r="S93" s="9" t="n"/>
+      <c r="T93" s="9" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="9" t="n"/>
@@ -3445,6 +3835,7 @@
       <c r="Q94" s="9" t="n"/>
       <c r="R94" s="9" t="n"/>
       <c r="S94" s="9" t="n"/>
+      <c r="T94" s="9" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="9" t="n"/>
@@ -3466,6 +3857,7 @@
       <c r="Q95" s="9" t="n"/>
       <c r="R95" s="9" t="n"/>
       <c r="S95" s="9" t="n"/>
+      <c r="T95" s="9" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="9" t="n"/>
@@ -3487,6 +3879,7 @@
       <c r="Q96" s="9" t="n"/>
       <c r="R96" s="9" t="n"/>
       <c r="S96" s="9" t="n"/>
+      <c r="T96" s="9" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="9" t="n"/>
@@ -3508,6 +3901,7 @@
       <c r="Q97" s="9" t="n"/>
       <c r="R97" s="9" t="n"/>
       <c r="S97" s="9" t="n"/>
+      <c r="T97" s="9" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="9" t="n"/>
@@ -3529,6 +3923,7 @@
       <c r="Q98" s="9" t="n"/>
       <c r="R98" s="9" t="n"/>
       <c r="S98" s="9" t="n"/>
+      <c r="T98" s="9" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="9" t="n"/>
@@ -3550,6 +3945,7 @@
       <c r="Q99" s="9" t="n"/>
       <c r="R99" s="9" t="n"/>
       <c r="S99" s="9" t="n"/>
+      <c r="T99" s="9" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="9" t="n"/>
@@ -3571,6 +3967,7 @@
       <c r="Q100" s="9" t="n"/>
       <c r="R100" s="9" t="n"/>
       <c r="S100" s="9" t="n"/>
+      <c r="T100" s="9" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="9" t="n"/>
@@ -3592,6 +3989,7 @@
       <c r="Q101" s="9" t="n"/>
       <c r="R101" s="9" t="n"/>
       <c r="S101" s="9" t="n"/>
+      <c r="T101" s="9" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="9" t="n"/>
@@ -3613,6 +4011,7 @@
       <c r="Q102" s="9" t="n"/>
       <c r="R102" s="9" t="n"/>
       <c r="S102" s="9" t="n"/>
+      <c r="T102" s="9" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="9" t="n"/>
@@ -3634,6 +4033,7 @@
       <c r="Q103" s="9" t="n"/>
       <c r="R103" s="9" t="n"/>
       <c r="S103" s="9" t="n"/>
+      <c r="T103" s="9" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="9" t="n"/>
@@ -3655,6 +4055,7 @@
       <c r="Q104" s="9" t="n"/>
       <c r="R104" s="9" t="n"/>
       <c r="S104" s="9" t="n"/>
+      <c r="T104" s="9" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="9" t="n"/>
@@ -3676,6 +4077,7 @@
       <c r="Q105" s="9" t="n"/>
       <c r="R105" s="9" t="n"/>
       <c r="S105" s="9" t="n"/>
+      <c r="T105" s="9" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="9" t="n"/>
@@ -3697,6 +4099,7 @@
       <c r="Q106" s="9" t="n"/>
       <c r="R106" s="9" t="n"/>
       <c r="S106" s="9" t="n"/>
+      <c r="T106" s="9" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="9" t="n"/>
@@ -3718,6 +4121,7 @@
       <c r="Q107" s="9" t="n"/>
       <c r="R107" s="9" t="n"/>
       <c r="S107" s="9" t="n"/>
+      <c r="T107" s="9" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="9" t="n"/>
@@ -3739,6 +4143,7 @@
       <c r="Q108" s="9" t="n"/>
       <c r="R108" s="9" t="n"/>
       <c r="S108" s="9" t="n"/>
+      <c r="T108" s="9" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="9" t="n"/>
@@ -3760,6 +4165,7 @@
       <c r="Q109" s="9" t="n"/>
       <c r="R109" s="9" t="n"/>
       <c r="S109" s="9" t="n"/>
+      <c r="T109" s="9" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="9" t="n"/>
@@ -3781,6 +4187,7 @@
       <c r="Q110" s="9" t="n"/>
       <c r="R110" s="9" t="n"/>
       <c r="S110" s="9" t="n"/>
+      <c r="T110" s="9" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="9" t="n"/>
@@ -3802,6 +4209,7 @@
       <c r="Q111" s="9" t="n"/>
       <c r="R111" s="9" t="n"/>
       <c r="S111" s="9" t="n"/>
+      <c r="T111" s="9" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="9" t="n"/>
@@ -3823,6 +4231,7 @@
       <c r="Q112" s="9" t="n"/>
       <c r="R112" s="9" t="n"/>
       <c r="S112" s="9" t="n"/>
+      <c r="T112" s="9" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="9" t="n"/>
@@ -3844,6 +4253,7 @@
       <c r="Q113" s="9" t="n"/>
       <c r="R113" s="9" t="n"/>
       <c r="S113" s="9" t="n"/>
+      <c r="T113" s="9" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="9" t="n"/>
@@ -3865,6 +4275,7 @@
       <c r="Q114" s="9" t="n"/>
       <c r="R114" s="9" t="n"/>
       <c r="S114" s="9" t="n"/>
+      <c r="T114" s="9" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="9" t="n"/>
@@ -3886,6 +4297,7 @@
       <c r="Q115" s="9" t="n"/>
       <c r="R115" s="9" t="n"/>
       <c r="S115" s="9" t="n"/>
+      <c r="T115" s="9" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="9" t="n"/>
@@ -3907,6 +4319,7 @@
       <c r="Q116" s="9" t="n"/>
       <c r="R116" s="9" t="n"/>
       <c r="S116" s="9" t="n"/>
+      <c r="T116" s="9" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="9" t="n"/>
@@ -3928,6 +4341,7 @@
       <c r="Q117" s="9" t="n"/>
       <c r="R117" s="9" t="n"/>
       <c r="S117" s="9" t="n"/>
+      <c r="T117" s="9" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="9" t="n"/>
@@ -3949,6 +4363,7 @@
       <c r="Q118" s="9" t="n"/>
       <c r="R118" s="9" t="n"/>
       <c r="S118" s="9" t="n"/>
+      <c r="T118" s="9" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="9" t="n"/>
@@ -3970,6 +4385,7 @@
       <c r="Q119" s="9" t="n"/>
       <c r="R119" s="9" t="n"/>
       <c r="S119" s="9" t="n"/>
+      <c r="T119" s="9" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="9" t="n"/>
@@ -3991,6 +4407,7 @@
       <c r="Q120" s="9" t="n"/>
       <c r="R120" s="9" t="n"/>
       <c r="S120" s="9" t="n"/>
+      <c r="T120" s="9" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="9" t="n"/>
@@ -4012,6 +4429,7 @@
       <c r="Q121" s="9" t="n"/>
       <c r="R121" s="9" t="n"/>
       <c r="S121" s="9" t="n"/>
+      <c r="T121" s="9" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="9" t="n"/>
@@ -4033,6 +4451,7 @@
       <c r="Q122" s="9" t="n"/>
       <c r="R122" s="9" t="n"/>
       <c r="S122" s="9" t="n"/>
+      <c r="T122" s="9" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="9" t="n"/>
@@ -4054,6 +4473,7 @@
       <c r="Q123" s="9" t="n"/>
       <c r="R123" s="9" t="n"/>
       <c r="S123" s="9" t="n"/>
+      <c r="T123" s="9" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="9" t="n"/>
@@ -4075,6 +4495,7 @@
       <c r="Q124" s="9" t="n"/>
       <c r="R124" s="9" t="n"/>
       <c r="S124" s="9" t="n"/>
+      <c r="T124" s="9" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="9" t="n"/>
@@ -4096,6 +4517,7 @@
       <c r="Q125" s="9" t="n"/>
       <c r="R125" s="9" t="n"/>
       <c r="S125" s="9" t="n"/>
+      <c r="T125" s="9" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="9" t="n"/>
@@ -4117,6 +4539,7 @@
       <c r="Q126" s="9" t="n"/>
       <c r="R126" s="9" t="n"/>
       <c r="S126" s="9" t="n"/>
+      <c r="T126" s="9" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="9" t="n"/>
@@ -4138,6 +4561,7 @@
       <c r="Q127" s="9" t="n"/>
       <c r="R127" s="9" t="n"/>
       <c r="S127" s="9" t="n"/>
+      <c r="T127" s="9" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="9" t="n"/>
@@ -4159,6 +4583,7 @@
       <c r="Q128" s="9" t="n"/>
       <c r="R128" s="9" t="n"/>
       <c r="S128" s="9" t="n"/>
+      <c r="T128" s="9" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="9" t="n"/>
@@ -4180,6 +4605,7 @@
       <c r="Q129" s="9" t="n"/>
       <c r="R129" s="9" t="n"/>
       <c r="S129" s="9" t="n"/>
+      <c r="T129" s="9" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="9" t="n"/>
@@ -4201,6 +4627,7 @@
       <c r="Q130" s="9" t="n"/>
       <c r="R130" s="9" t="n"/>
       <c r="S130" s="9" t="n"/>
+      <c r="T130" s="9" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="9" t="n"/>
@@ -4222,6 +4649,7 @@
       <c r="Q131" s="9" t="n"/>
       <c r="R131" s="9" t="n"/>
       <c r="S131" s="9" t="n"/>
+      <c r="T131" s="9" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="9" t="n"/>
@@ -4243,6 +4671,7 @@
       <c r="Q132" s="9" t="n"/>
       <c r="R132" s="9" t="n"/>
       <c r="S132" s="9" t="n"/>
+      <c r="T132" s="9" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="9" t="n"/>
@@ -4264,6 +4693,7 @@
       <c r="Q133" s="9" t="n"/>
       <c r="R133" s="9" t="n"/>
       <c r="S133" s="9" t="n"/>
+      <c r="T133" s="9" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="9" t="n"/>
@@ -4285,6 +4715,7 @@
       <c r="Q134" s="9" t="n"/>
       <c r="R134" s="9" t="n"/>
       <c r="S134" s="9" t="n"/>
+      <c r="T134" s="9" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="9" t="n"/>
@@ -4306,6 +4737,7 @@
       <c r="Q135" s="9" t="n"/>
       <c r="R135" s="9" t="n"/>
       <c r="S135" s="9" t="n"/>
+      <c r="T135" s="9" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="9" t="n"/>
@@ -4327,6 +4759,7 @@
       <c r="Q136" s="9" t="n"/>
       <c r="R136" s="9" t="n"/>
       <c r="S136" s="9" t="n"/>
+      <c r="T136" s="9" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="9" t="n"/>
@@ -4348,6 +4781,7 @@
       <c r="Q137" s="9" t="n"/>
       <c r="R137" s="9" t="n"/>
       <c r="S137" s="9" t="n"/>
+      <c r="T137" s="9" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="9" t="n"/>
@@ -4369,6 +4803,7 @@
       <c r="Q138" s="9" t="n"/>
       <c r="R138" s="9" t="n"/>
       <c r="S138" s="9" t="n"/>
+      <c r="T138" s="9" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="9" t="n"/>
@@ -4390,6 +4825,7 @@
       <c r="Q139" s="9" t="n"/>
       <c r="R139" s="9" t="n"/>
       <c r="S139" s="9" t="n"/>
+      <c r="T139" s="9" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="9" t="n"/>
@@ -4411,6 +4847,7 @@
       <c r="Q140" s="9" t="n"/>
       <c r="R140" s="9" t="n"/>
       <c r="S140" s="9" t="n"/>
+      <c r="T140" s="9" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="9" t="n"/>
@@ -4432,6 +4869,7 @@
       <c r="Q141" s="9" t="n"/>
       <c r="R141" s="9" t="n"/>
       <c r="S141" s="9" t="n"/>
+      <c r="T141" s="9" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="9" t="n"/>
@@ -4453,6 +4891,7 @@
       <c r="Q142" s="9" t="n"/>
       <c r="R142" s="9" t="n"/>
       <c r="S142" s="9" t="n"/>
+      <c r="T142" s="9" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="9" t="n"/>
@@ -4474,6 +4913,7 @@
       <c r="Q143" s="9" t="n"/>
       <c r="R143" s="9" t="n"/>
       <c r="S143" s="9" t="n"/>
+      <c r="T143" s="9" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="9" t="n"/>
@@ -4495,6 +4935,7 @@
       <c r="Q144" s="9" t="n"/>
       <c r="R144" s="9" t="n"/>
       <c r="S144" s="9" t="n"/>
+      <c r="T144" s="9" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="9" t="n"/>
@@ -4516,6 +4957,7 @@
       <c r="Q145" s="9" t="n"/>
       <c r="R145" s="9" t="n"/>
       <c r="S145" s="9" t="n"/>
+      <c r="T145" s="9" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="9" t="n"/>
@@ -4537,6 +4979,7 @@
       <c r="Q146" s="9" t="n"/>
       <c r="R146" s="9" t="n"/>
       <c r="S146" s="9" t="n"/>
+      <c r="T146" s="9" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="9" t="n"/>
@@ -4558,6 +5001,7 @@
       <c r="Q147" s="9" t="n"/>
       <c r="R147" s="9" t="n"/>
       <c r="S147" s="9" t="n"/>
+      <c r="T147" s="9" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="9" t="n"/>
@@ -4579,6 +5023,7 @@
       <c r="Q148" s="9" t="n"/>
       <c r="R148" s="9" t="n"/>
       <c r="S148" s="9" t="n"/>
+      <c r="T148" s="9" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="9" t="n"/>
@@ -4600,6 +5045,7 @@
       <c r="Q149" s="9" t="n"/>
       <c r="R149" s="9" t="n"/>
       <c r="S149" s="9" t="n"/>
+      <c r="T149" s="9" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="9" t="n"/>
@@ -4621,6 +5067,7 @@
       <c r="Q150" s="9" t="n"/>
       <c r="R150" s="9" t="n"/>
       <c r="S150" s="9" t="n"/>
+      <c r="T150" s="9" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="9" t="n"/>
@@ -4642,6 +5089,7 @@
       <c r="Q151" s="9" t="n"/>
       <c r="R151" s="9" t="n"/>
       <c r="S151" s="9" t="n"/>
+      <c r="T151" s="9" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="9" t="n"/>
@@ -4663,6 +5111,7 @@
       <c r="Q152" s="9" t="n"/>
       <c r="R152" s="9" t="n"/>
       <c r="S152" s="9" t="n"/>
+      <c r="T152" s="9" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="9" t="n"/>
@@ -4684,6 +5133,7 @@
       <c r="Q153" s="9" t="n"/>
       <c r="R153" s="9" t="n"/>
       <c r="S153" s="9" t="n"/>
+      <c r="T153" s="9" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="9" t="n"/>
@@ -4705,6 +5155,7 @@
       <c r="Q154" s="9" t="n"/>
       <c r="R154" s="9" t="n"/>
       <c r="S154" s="9" t="n"/>
+      <c r="T154" s="9" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="9" t="n"/>
@@ -4726,6 +5177,7 @@
       <c r="Q155" s="9" t="n"/>
       <c r="R155" s="9" t="n"/>
       <c r="S155" s="9" t="n"/>
+      <c r="T155" s="9" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="9" t="n"/>
@@ -4747,6 +5199,7 @@
       <c r="Q156" s="9" t="n"/>
       <c r="R156" s="9" t="n"/>
       <c r="S156" s="9" t="n"/>
+      <c r="T156" s="9" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="9" t="n"/>
@@ -4768,6 +5221,7 @@
       <c r="Q157" s="9" t="n"/>
       <c r="R157" s="9" t="n"/>
       <c r="S157" s="9" t="n"/>
+      <c r="T157" s="9" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="9" t="n"/>
@@ -4789,6 +5243,7 @@
       <c r="Q158" s="9" t="n"/>
       <c r="R158" s="9" t="n"/>
       <c r="S158" s="9" t="n"/>
+      <c r="T158" s="9" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="9" t="n"/>
@@ -4810,6 +5265,7 @@
       <c r="Q159" s="9" t="n"/>
       <c r="R159" s="9" t="n"/>
       <c r="S159" s="9" t="n"/>
+      <c r="T159" s="9" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="9" t="n"/>
@@ -4831,6 +5287,7 @@
       <c r="Q160" s="9" t="n"/>
       <c r="R160" s="9" t="n"/>
       <c r="S160" s="9" t="n"/>
+      <c r="T160" s="9" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="9" t="n"/>
@@ -4852,6 +5309,7 @@
       <c r="Q161" s="9" t="n"/>
       <c r="R161" s="9" t="n"/>
       <c r="S161" s="9" t="n"/>
+      <c r="T161" s="9" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="9" t="n"/>
@@ -4873,6 +5331,7 @@
       <c r="Q162" s="9" t="n"/>
       <c r="R162" s="9" t="n"/>
       <c r="S162" s="9" t="n"/>
+      <c r="T162" s="9" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="9" t="n"/>
@@ -4894,6 +5353,7 @@
       <c r="Q163" s="9" t="n"/>
       <c r="R163" s="9" t="n"/>
       <c r="S163" s="9" t="n"/>
+      <c r="T163" s="9" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="9" t="n"/>
@@ -4915,6 +5375,7 @@
       <c r="Q164" s="9" t="n"/>
       <c r="R164" s="9" t="n"/>
       <c r="S164" s="9" t="n"/>
+      <c r="T164" s="9" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="9" t="n"/>
@@ -4936,6 +5397,7 @@
       <c r="Q165" s="9" t="n"/>
       <c r="R165" s="9" t="n"/>
       <c r="S165" s="9" t="n"/>
+      <c r="T165" s="9" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="9" t="n"/>
@@ -4957,6 +5419,7 @@
       <c r="Q166" s="9" t="n"/>
       <c r="R166" s="9" t="n"/>
       <c r="S166" s="9" t="n"/>
+      <c r="T166" s="9" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="9" t="n"/>
@@ -4978,6 +5441,7 @@
       <c r="Q167" s="9" t="n"/>
       <c r="R167" s="9" t="n"/>
       <c r="S167" s="9" t="n"/>
+      <c r="T167" s="9" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="9" t="n"/>
@@ -4999,6 +5463,7 @@
       <c r="Q168" s="9" t="n"/>
       <c r="R168" s="9" t="n"/>
       <c r="S168" s="9" t="n"/>
+      <c r="T168" s="9" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="9" t="n"/>
@@ -5020,6 +5485,7 @@
       <c r="Q169" s="9" t="n"/>
       <c r="R169" s="9" t="n"/>
       <c r="S169" s="9" t="n"/>
+      <c r="T169" s="9" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="9" t="n"/>
@@ -5041,6 +5507,7 @@
       <c r="Q170" s="9" t="n"/>
       <c r="R170" s="9" t="n"/>
       <c r="S170" s="9" t="n"/>
+      <c r="T170" s="9" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="9" t="n"/>
@@ -5062,6 +5529,7 @@
       <c r="Q171" s="9" t="n"/>
       <c r="R171" s="9" t="n"/>
       <c r="S171" s="9" t="n"/>
+      <c r="T171" s="9" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="9" t="n"/>
@@ -5083,6 +5551,7 @@
       <c r="Q172" s="9" t="n"/>
       <c r="R172" s="9" t="n"/>
       <c r="S172" s="9" t="n"/>
+      <c r="T172" s="9" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="9" t="n"/>
@@ -5104,6 +5573,7 @@
       <c r="Q173" s="9" t="n"/>
       <c r="R173" s="9" t="n"/>
       <c r="S173" s="9" t="n"/>
+      <c r="T173" s="9" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="9" t="n"/>
@@ -5125,6 +5595,7 @@
       <c r="Q174" s="9" t="n"/>
       <c r="R174" s="9" t="n"/>
       <c r="S174" s="9" t="n"/>
+      <c r="T174" s="9" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="9" t="n"/>
@@ -5146,6 +5617,7 @@
       <c r="Q175" s="9" t="n"/>
       <c r="R175" s="9" t="n"/>
       <c r="S175" s="9" t="n"/>
+      <c r="T175" s="9" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="9" t="n"/>
@@ -5167,6 +5639,7 @@
       <c r="Q176" s="9" t="n"/>
       <c r="R176" s="9" t="n"/>
       <c r="S176" s="9" t="n"/>
+      <c r="T176" s="9" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="9" t="n"/>
@@ -5188,6 +5661,7 @@
       <c r="Q177" s="9" t="n"/>
       <c r="R177" s="9" t="n"/>
       <c r="S177" s="9" t="n"/>
+      <c r="T177" s="9" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="9" t="n"/>
@@ -5209,6 +5683,7 @@
       <c r="Q178" s="9" t="n"/>
       <c r="R178" s="9" t="n"/>
       <c r="S178" s="9" t="n"/>
+      <c r="T178" s="9" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="9" t="n"/>
@@ -5230,6 +5705,7 @@
       <c r="Q179" s="9" t="n"/>
       <c r="R179" s="9" t="n"/>
       <c r="S179" s="9" t="n"/>
+      <c r="T179" s="9" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="9" t="n"/>
@@ -5251,6 +5727,7 @@
       <c r="Q180" s="9" t="n"/>
       <c r="R180" s="9" t="n"/>
       <c r="S180" s="9" t="n"/>
+      <c r="T180" s="9" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="9" t="n"/>
@@ -5272,6 +5749,7 @@
       <c r="Q181" s="9" t="n"/>
       <c r="R181" s="9" t="n"/>
       <c r="S181" s="9" t="n"/>
+      <c r="T181" s="9" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="9" t="n"/>
@@ -5293,6 +5771,7 @@
       <c r="Q182" s="9" t="n"/>
       <c r="R182" s="9" t="n"/>
       <c r="S182" s="9" t="n"/>
+      <c r="T182" s="9" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="9" t="n"/>
@@ -5314,6 +5793,7 @@
       <c r="Q183" s="9" t="n"/>
       <c r="R183" s="9" t="n"/>
       <c r="S183" s="9" t="n"/>
+      <c r="T183" s="9" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="9" t="n"/>
@@ -5335,6 +5815,7 @@
       <c r="Q184" s="9" t="n"/>
       <c r="R184" s="9" t="n"/>
       <c r="S184" s="9" t="n"/>
+      <c r="T184" s="9" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="9" t="n"/>
@@ -5356,6 +5837,7 @@
       <c r="Q185" s="9" t="n"/>
       <c r="R185" s="9" t="n"/>
       <c r="S185" s="9" t="n"/>
+      <c r="T185" s="9" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="9" t="n"/>
@@ -5377,6 +5859,7 @@
       <c r="Q186" s="9" t="n"/>
       <c r="R186" s="9" t="n"/>
       <c r="S186" s="9" t="n"/>
+      <c r="T186" s="9" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="9" t="n"/>
@@ -5398,6 +5881,7 @@
       <c r="Q187" s="9" t="n"/>
       <c r="R187" s="9" t="n"/>
       <c r="S187" s="9" t="n"/>
+      <c r="T187" s="9" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="9" t="n"/>
@@ -5419,6 +5903,7 @@
       <c r="Q188" s="9" t="n"/>
       <c r="R188" s="9" t="n"/>
       <c r="S188" s="9" t="n"/>
+      <c r="T188" s="9" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="9" t="n"/>
@@ -5440,6 +5925,7 @@
       <c r="Q189" s="9" t="n"/>
       <c r="R189" s="9" t="n"/>
       <c r="S189" s="9" t="n"/>
+      <c r="T189" s="9" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="9" t="n"/>
@@ -5461,6 +5947,7 @@
       <c r="Q190" s="9" t="n"/>
       <c r="R190" s="9" t="n"/>
       <c r="S190" s="9" t="n"/>
+      <c r="T190" s="9" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="9" t="n"/>
@@ -5482,6 +5969,7 @@
       <c r="Q191" s="9" t="n"/>
       <c r="R191" s="9" t="n"/>
       <c r="S191" s="9" t="n"/>
+      <c r="T191" s="9" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="9" t="n"/>
@@ -5503,6 +5991,7 @@
       <c r="Q192" s="9" t="n"/>
       <c r="R192" s="9" t="n"/>
       <c r="S192" s="9" t="n"/>
+      <c r="T192" s="9" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="9" t="n"/>
@@ -5524,6 +6013,7 @@
       <c r="Q193" s="9" t="n"/>
       <c r="R193" s="9" t="n"/>
       <c r="S193" s="9" t="n"/>
+      <c r="T193" s="9" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="9" t="n"/>
@@ -5545,6 +6035,7 @@
       <c r="Q194" s="9" t="n"/>
       <c r="R194" s="9" t="n"/>
       <c r="S194" s="9" t="n"/>
+      <c r="T194" s="9" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="9" t="n"/>
@@ -5566,6 +6057,7 @@
       <c r="Q195" s="9" t="n"/>
       <c r="R195" s="9" t="n"/>
       <c r="S195" s="9" t="n"/>
+      <c r="T195" s="9" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="9" t="n"/>
@@ -5587,6 +6079,7 @@
       <c r="Q196" s="9" t="n"/>
       <c r="R196" s="9" t="n"/>
       <c r="S196" s="9" t="n"/>
+      <c r="T196" s="9" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="9" t="n"/>
@@ -5608,6 +6101,7 @@
       <c r="Q197" s="9" t="n"/>
       <c r="R197" s="9" t="n"/>
       <c r="S197" s="9" t="n"/>
+      <c r="T197" s="9" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="9" t="n"/>
@@ -5629,6 +6123,7 @@
       <c r="Q198" s="9" t="n"/>
       <c r="R198" s="9" t="n"/>
       <c r="S198" s="9" t="n"/>
+      <c r="T198" s="9" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="9" t="n"/>
@@ -5650,6 +6145,7 @@
       <c r="Q199" s="9" t="n"/>
       <c r="R199" s="9" t="n"/>
       <c r="S199" s="9" t="n"/>
+      <c r="T199" s="9" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="9" t="n"/>
@@ -5671,6 +6167,7 @@
       <c r="Q200" s="9" t="n"/>
       <c r="R200" s="9" t="n"/>
       <c r="S200" s="9" t="n"/>
+      <c r="T200" s="9" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="9" t="n"/>
@@ -5692,6 +6189,7 @@
       <c r="Q201" s="9" t="n"/>
       <c r="R201" s="9" t="n"/>
       <c r="S201" s="9" t="n"/>
+      <c r="T201" s="9" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="9" t="n"/>
@@ -5713,6 +6211,7 @@
       <c r="Q202" s="9" t="n"/>
       <c r="R202" s="9" t="n"/>
       <c r="S202" s="9" t="n"/>
+      <c r="T202" s="9" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="9" t="n"/>
@@ -5734,6 +6233,7 @@
       <c r="Q203" s="9" t="n"/>
       <c r="R203" s="9" t="n"/>
       <c r="S203" s="9" t="n"/>
+      <c r="T203" s="9" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="9" t="n"/>
@@ -5755,6 +6255,7 @@
       <c r="Q204" s="9" t="n"/>
       <c r="R204" s="9" t="n"/>
       <c r="S204" s="9" t="n"/>
+      <c r="T204" s="9" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="9" t="n"/>
@@ -5776,6 +6277,7 @@
       <c r="Q205" s="9" t="n"/>
       <c r="R205" s="9" t="n"/>
       <c r="S205" s="9" t="n"/>
+      <c r="T205" s="9" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="9" t="n"/>
@@ -5797,6 +6299,7 @@
       <c r="Q206" s="9" t="n"/>
       <c r="R206" s="9" t="n"/>
       <c r="S206" s="9" t="n"/>
+      <c r="T206" s="9" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="9" t="n"/>
@@ -5818,6 +6321,7 @@
       <c r="Q207" s="9" t="n"/>
       <c r="R207" s="9" t="n"/>
       <c r="S207" s="9" t="n"/>
+      <c r="T207" s="9" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="9" t="n"/>
@@ -5839,6 +6343,7 @@
       <c r="Q208" s="9" t="n"/>
       <c r="R208" s="9" t="n"/>
       <c r="S208" s="9" t="n"/>
+      <c r="T208" s="9" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="9" t="n"/>
@@ -5860,6 +6365,7 @@
       <c r="Q209" s="9" t="n"/>
       <c r="R209" s="9" t="n"/>
       <c r="S209" s="9" t="n"/>
+      <c r="T209" s="9" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="9" t="n"/>
@@ -5881,6 +6387,7 @@
       <c r="Q210" s="9" t="n"/>
       <c r="R210" s="9" t="n"/>
       <c r="S210" s="9" t="n"/>
+      <c r="T210" s="9" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="9" t="n"/>
@@ -5902,6 +6409,7 @@
       <c r="Q211" s="9" t="n"/>
       <c r="R211" s="9" t="n"/>
       <c r="S211" s="9" t="n"/>
+      <c r="T211" s="9" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="9" t="n"/>
@@ -5923,6 +6431,7 @@
       <c r="Q212" s="9" t="n"/>
       <c r="R212" s="9" t="n"/>
       <c r="S212" s="9" t="n"/>
+      <c r="T212" s="9" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="9" t="n"/>
@@ -5944,6 +6453,7 @@
       <c r="Q213" s="9" t="n"/>
       <c r="R213" s="9" t="n"/>
       <c r="S213" s="9" t="n"/>
+      <c r="T213" s="9" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="9" t="n"/>
@@ -5965,6 +6475,7 @@
       <c r="Q214" s="9" t="n"/>
       <c r="R214" s="9" t="n"/>
       <c r="S214" s="9" t="n"/>
+      <c r="T214" s="9" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="9" t="n"/>
@@ -5986,6 +6497,7 @@
       <c r="Q215" s="9" t="n"/>
       <c r="R215" s="9" t="n"/>
       <c r="S215" s="9" t="n"/>
+      <c r="T215" s="9" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="9" t="n"/>
@@ -6007,6 +6519,7 @@
       <c r="Q216" s="9" t="n"/>
       <c r="R216" s="9" t="n"/>
       <c r="S216" s="9" t="n"/>
+      <c r="T216" s="9" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="9" t="n"/>
@@ -6028,6 +6541,7 @@
       <c r="Q217" s="9" t="n"/>
       <c r="R217" s="9" t="n"/>
       <c r="S217" s="9" t="n"/>
+      <c r="T217" s="9" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="9" t="n"/>
@@ -6049,6 +6563,7 @@
       <c r="Q218" s="9" t="n"/>
       <c r="R218" s="9" t="n"/>
       <c r="S218" s="9" t="n"/>
+      <c r="T218" s="9" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="9" t="n"/>
@@ -6070,6 +6585,7 @@
       <c r="Q219" s="9" t="n"/>
       <c r="R219" s="9" t="n"/>
       <c r="S219" s="9" t="n"/>
+      <c r="T219" s="9" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="9" t="n"/>
@@ -6091,6 +6607,7 @@
       <c r="Q220" s="9" t="n"/>
       <c r="R220" s="9" t="n"/>
       <c r="S220" s="9" t="n"/>
+      <c r="T220" s="9" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="9" t="n"/>
@@ -6112,6 +6629,7 @@
       <c r="Q221" s="9" t="n"/>
       <c r="R221" s="9" t="n"/>
       <c r="S221" s="9" t="n"/>
+      <c r="T221" s="9" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="9" t="n"/>
@@ -6133,6 +6651,7 @@
       <c r="Q222" s="9" t="n"/>
       <c r="R222" s="9" t="n"/>
       <c r="S222" s="9" t="n"/>
+      <c r="T222" s="9" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="9" t="n"/>
@@ -6154,6 +6673,7 @@
       <c r="Q223" s="9" t="n"/>
       <c r="R223" s="9" t="n"/>
       <c r="S223" s="9" t="n"/>
+      <c r="T223" s="9" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="9" t="n"/>
@@ -6175,6 +6695,7 @@
       <c r="Q224" s="9" t="n"/>
       <c r="R224" s="9" t="n"/>
       <c r="S224" s="9" t="n"/>
+      <c r="T224" s="9" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="9" t="n"/>
@@ -6196,6 +6717,7 @@
       <c r="Q225" s="9" t="n"/>
       <c r="R225" s="9" t="n"/>
       <c r="S225" s="9" t="n"/>
+      <c r="T225" s="9" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="9" t="n"/>
@@ -6217,6 +6739,7 @@
       <c r="Q226" s="9" t="n"/>
       <c r="R226" s="9" t="n"/>
       <c r="S226" s="9" t="n"/>
+      <c r="T226" s="9" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="9" t="n"/>
@@ -6238,6 +6761,7 @@
       <c r="Q227" s="9" t="n"/>
       <c r="R227" s="9" t="n"/>
       <c r="S227" s="9" t="n"/>
+      <c r="T227" s="9" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="9" t="n"/>
@@ -6259,6 +6783,7 @@
       <c r="Q228" s="9" t="n"/>
       <c r="R228" s="9" t="n"/>
       <c r="S228" s="9" t="n"/>
+      <c r="T228" s="9" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="9" t="n"/>
@@ -6280,6 +6805,7 @@
       <c r="Q229" s="9" t="n"/>
       <c r="R229" s="9" t="n"/>
       <c r="S229" s="9" t="n"/>
+      <c r="T229" s="9" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="9" t="n"/>
@@ -6301,6 +6827,7 @@
       <c r="Q230" s="9" t="n"/>
       <c r="R230" s="9" t="n"/>
       <c r="S230" s="9" t="n"/>
+      <c r="T230" s="9" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="9" t="n"/>
@@ -6322,6 +6849,7 @@
       <c r="Q231" s="9" t="n"/>
       <c r="R231" s="9" t="n"/>
       <c r="S231" s="9" t="n"/>
+      <c r="T231" s="9" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="9" t="n"/>
@@ -6343,6 +6871,7 @@
       <c r="Q232" s="9" t="n"/>
       <c r="R232" s="9" t="n"/>
       <c r="S232" s="9" t="n"/>
+      <c r="T232" s="9" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="9" t="n"/>
@@ -6364,6 +6893,7 @@
       <c r="Q233" s="9" t="n"/>
       <c r="R233" s="9" t="n"/>
       <c r="S233" s="9" t="n"/>
+      <c r="T233" s="9" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="9" t="n"/>
@@ -6385,6 +6915,7 @@
       <c r="Q234" s="9" t="n"/>
       <c r="R234" s="9" t="n"/>
       <c r="S234" s="9" t="n"/>
+      <c r="T234" s="9" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="9" t="n"/>
@@ -6406,6 +6937,7 @@
       <c r="Q235" s="9" t="n"/>
       <c r="R235" s="9" t="n"/>
       <c r="S235" s="9" t="n"/>
+      <c r="T235" s="9" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="9" t="n"/>
@@ -6427,6 +6959,7 @@
       <c r="Q236" s="9" t="n"/>
       <c r="R236" s="9" t="n"/>
       <c r="S236" s="9" t="n"/>
+      <c r="T236" s="9" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="9" t="n"/>
@@ -6448,6 +6981,7 @@
       <c r="Q237" s="9" t="n"/>
       <c r="R237" s="9" t="n"/>
       <c r="S237" s="9" t="n"/>
+      <c r="T237" s="9" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="9" t="n"/>
@@ -6469,6 +7003,7 @@
       <c r="Q238" s="9" t="n"/>
       <c r="R238" s="9" t="n"/>
       <c r="S238" s="9" t="n"/>
+      <c r="T238" s="9" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="9" t="n"/>
@@ -6490,6 +7025,7 @@
       <c r="Q239" s="9" t="n"/>
       <c r="R239" s="9" t="n"/>
       <c r="S239" s="9" t="n"/>
+      <c r="T239" s="9" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="9" t="n"/>
@@ -6511,6 +7047,7 @@
       <c r="Q240" s="9" t="n"/>
       <c r="R240" s="9" t="n"/>
       <c r="S240" s="9" t="n"/>
+      <c r="T240" s="9" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="9" t="n"/>
@@ -6532,6 +7069,7 @@
       <c r="Q241" s="9" t="n"/>
       <c r="R241" s="9" t="n"/>
       <c r="S241" s="9" t="n"/>
+      <c r="T241" s="9" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="9" t="n"/>
@@ -6553,6 +7091,7 @@
       <c r="Q242" s="9" t="n"/>
       <c r="R242" s="9" t="n"/>
       <c r="S242" s="9" t="n"/>
+      <c r="T242" s="9" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="9" t="n"/>
@@ -6574,6 +7113,7 @@
       <c r="Q243" s="9" t="n"/>
       <c r="R243" s="9" t="n"/>
       <c r="S243" s="9" t="n"/>
+      <c r="T243" s="9" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="9" t="n"/>
@@ -6595,6 +7135,7 @@
       <c r="Q244" s="9" t="n"/>
       <c r="R244" s="9" t="n"/>
       <c r="S244" s="9" t="n"/>
+      <c r="T244" s="9" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="9" t="n"/>
@@ -6616,6 +7157,7 @@
       <c r="Q245" s="9" t="n"/>
       <c r="R245" s="9" t="n"/>
       <c r="S245" s="9" t="n"/>
+      <c r="T245" s="9" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="9" t="n"/>
@@ -6637,6 +7179,7 @@
       <c r="Q246" s="9" t="n"/>
       <c r="R246" s="9" t="n"/>
       <c r="S246" s="9" t="n"/>
+      <c r="T246" s="9" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="9" t="n"/>
@@ -6658,6 +7201,7 @@
       <c r="Q247" s="9" t="n"/>
       <c r="R247" s="9" t="n"/>
       <c r="S247" s="9" t="n"/>
+      <c r="T247" s="9" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="9" t="n"/>
@@ -6679,6 +7223,7 @@
       <c r="Q248" s="9" t="n"/>
       <c r="R248" s="9" t="n"/>
       <c r="S248" s="9" t="n"/>
+      <c r="T248" s="9" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="9" t="n"/>
@@ -6700,6 +7245,7 @@
       <c r="Q249" s="9" t="n"/>
       <c r="R249" s="9" t="n"/>
       <c r="S249" s="9" t="n"/>
+      <c r="T249" s="9" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="9" t="n"/>
@@ -6721,6 +7267,7 @@
       <c r="Q250" s="9" t="n"/>
       <c r="R250" s="9" t="n"/>
       <c r="S250" s="9" t="n"/>
+      <c r="T250" s="9" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="9" t="n"/>
@@ -6742,6 +7289,7 @@
       <c r="Q251" s="9" t="n"/>
       <c r="R251" s="9" t="n"/>
       <c r="S251" s="9" t="n"/>
+      <c r="T251" s="9" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="9" t="n"/>
@@ -6763,6 +7311,7 @@
       <c r="Q252" s="9" t="n"/>
       <c r="R252" s="9" t="n"/>
       <c r="S252" s="9" t="n"/>
+      <c r="T252" s="9" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="9" t="n"/>
@@ -6784,6 +7333,7 @@
       <c r="Q253" s="9" t="n"/>
       <c r="R253" s="9" t="n"/>
       <c r="S253" s="9" t="n"/>
+      <c r="T253" s="9" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="9" t="n"/>
@@ -6805,6 +7355,7 @@
       <c r="Q254" s="9" t="n"/>
       <c r="R254" s="9" t="n"/>
       <c r="S254" s="9" t="n"/>
+      <c r="T254" s="9" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="9" t="n"/>
@@ -6826,6 +7377,7 @@
       <c r="Q255" s="9" t="n"/>
       <c r="R255" s="9" t="n"/>
       <c r="S255" s="9" t="n"/>
+      <c r="T255" s="9" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="9" t="n"/>
@@ -6847,6 +7399,7 @@
       <c r="Q256" s="9" t="n"/>
       <c r="R256" s="9" t="n"/>
       <c r="S256" s="9" t="n"/>
+      <c r="T256" s="9" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="9" t="n"/>
@@ -6868,6 +7421,7 @@
       <c r="Q257" s="9" t="n"/>
       <c r="R257" s="9" t="n"/>
       <c r="S257" s="9" t="n"/>
+      <c r="T257" s="9" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="9" t="n"/>
@@ -6889,6 +7443,7 @@
       <c r="Q258" s="9" t="n"/>
       <c r="R258" s="9" t="n"/>
       <c r="S258" s="9" t="n"/>
+      <c r="T258" s="9" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="9" t="n"/>
@@ -6910,6 +7465,7 @@
       <c r="Q259" s="9" t="n"/>
       <c r="R259" s="9" t="n"/>
       <c r="S259" s="9" t="n"/>
+      <c r="T259" s="9" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="9" t="n"/>
@@ -6931,6 +7487,7 @@
       <c r="Q260" s="9" t="n"/>
       <c r="R260" s="9" t="n"/>
       <c r="S260" s="9" t="n"/>
+      <c r="T260" s="9" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="9" t="n"/>
@@ -6952,6 +7509,7 @@
       <c r="Q261" s="9" t="n"/>
       <c r="R261" s="9" t="n"/>
       <c r="S261" s="9" t="n"/>
+      <c r="T261" s="9" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="9" t="n"/>
@@ -6973,6 +7531,7 @@
       <c r="Q262" s="9" t="n"/>
       <c r="R262" s="9" t="n"/>
       <c r="S262" s="9" t="n"/>
+      <c r="T262" s="9" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="9" t="n"/>
@@ -6994,6 +7553,7 @@
       <c r="Q263" s="9" t="n"/>
       <c r="R263" s="9" t="n"/>
       <c r="S263" s="9" t="n"/>
+      <c r="T263" s="9" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="9" t="n"/>
@@ -7015,6 +7575,7 @@
       <c r="Q264" s="9" t="n"/>
       <c r="R264" s="9" t="n"/>
       <c r="S264" s="9" t="n"/>
+      <c r="T264" s="9" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="9" t="n"/>
@@ -7036,6 +7597,7 @@
       <c r="Q265" s="9" t="n"/>
       <c r="R265" s="9" t="n"/>
       <c r="S265" s="9" t="n"/>
+      <c r="T265" s="9" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="9" t="n"/>
@@ -7057,6 +7619,7 @@
       <c r="Q266" s="9" t="n"/>
       <c r="R266" s="9" t="n"/>
       <c r="S266" s="9" t="n"/>
+      <c r="T266" s="9" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="9" t="n"/>
@@ -7078,6 +7641,7 @@
       <c r="Q267" s="9" t="n"/>
       <c r="R267" s="9" t="n"/>
       <c r="S267" s="9" t="n"/>
+      <c r="T267" s="9" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="9" t="n"/>
@@ -7099,6 +7663,7 @@
       <c r="Q268" s="9" t="n"/>
       <c r="R268" s="9" t="n"/>
       <c r="S268" s="9" t="n"/>
+      <c r="T268" s="9" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="9" t="n"/>
@@ -7120,6 +7685,7 @@
       <c r="Q269" s="9" t="n"/>
       <c r="R269" s="9" t="n"/>
       <c r="S269" s="9" t="n"/>
+      <c r="T269" s="9" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="9" t="n"/>
@@ -7141,6 +7707,7 @@
       <c r="Q270" s="9" t="n"/>
       <c r="R270" s="9" t="n"/>
       <c r="S270" s="9" t="n"/>
+      <c r="T270" s="9" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="9" t="n"/>
@@ -7162,6 +7729,7 @@
       <c r="Q271" s="9" t="n"/>
       <c r="R271" s="9" t="n"/>
       <c r="S271" s="9" t="n"/>
+      <c r="T271" s="9" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="9" t="n"/>
@@ -7183,6 +7751,7 @@
       <c r="Q272" s="9" t="n"/>
       <c r="R272" s="9" t="n"/>
       <c r="S272" s="9" t="n"/>
+      <c r="T272" s="9" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="9" t="n"/>
@@ -7204,6 +7773,7 @@
       <c r="Q273" s="9" t="n"/>
       <c r="R273" s="9" t="n"/>
       <c r="S273" s="9" t="n"/>
+      <c r="T273" s="9" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="9" t="n"/>
@@ -7225,6 +7795,7 @@
       <c r="Q274" s="9" t="n"/>
       <c r="R274" s="9" t="n"/>
       <c r="S274" s="9" t="n"/>
+      <c r="T274" s="9" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="9" t="n"/>
@@ -7246,6 +7817,7 @@
       <c r="Q275" s="9" t="n"/>
       <c r="R275" s="9" t="n"/>
       <c r="S275" s="9" t="n"/>
+      <c r="T275" s="9" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="9" t="n"/>
@@ -7267,6 +7839,7 @@
       <c r="Q276" s="9" t="n"/>
       <c r="R276" s="9" t="n"/>
       <c r="S276" s="9" t="n"/>
+      <c r="T276" s="9" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="9" t="n"/>
@@ -7288,6 +7861,7 @@
       <c r="Q277" s="9" t="n"/>
       <c r="R277" s="9" t="n"/>
       <c r="S277" s="9" t="n"/>
+      <c r="T277" s="9" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="9" t="n"/>
@@ -7309,6 +7883,7 @@
       <c r="Q278" s="9" t="n"/>
       <c r="R278" s="9" t="n"/>
       <c r="S278" s="9" t="n"/>
+      <c r="T278" s="9" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="9" t="n"/>
@@ -7330,6 +7905,7 @@
       <c r="Q279" s="9" t="n"/>
       <c r="R279" s="9" t="n"/>
       <c r="S279" s="9" t="n"/>
+      <c r="T279" s="9" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="9" t="n"/>
@@ -7351,6 +7927,7 @@
       <c r="Q280" s="9" t="n"/>
       <c r="R280" s="9" t="n"/>
       <c r="S280" s="9" t="n"/>
+      <c r="T280" s="9" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="9" t="n"/>
@@ -7372,6 +7949,7 @@
       <c r="Q281" s="9" t="n"/>
       <c r="R281" s="9" t="n"/>
       <c r="S281" s="9" t="n"/>
+      <c r="T281" s="9" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="9" t="n"/>
@@ -7393,6 +7971,7 @@
       <c r="Q282" s="9" t="n"/>
       <c r="R282" s="9" t="n"/>
       <c r="S282" s="9" t="n"/>
+      <c r="T282" s="9" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="9" t="n"/>
@@ -7414,6 +7993,7 @@
       <c r="Q283" s="9" t="n"/>
       <c r="R283" s="9" t="n"/>
       <c r="S283" s="9" t="n"/>
+      <c r="T283" s="9" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="9" t="n"/>
@@ -7435,6 +8015,7 @@
       <c r="Q284" s="9" t="n"/>
       <c r="R284" s="9" t="n"/>
       <c r="S284" s="9" t="n"/>
+      <c r="T284" s="9" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="9" t="n"/>
@@ -7456,6 +8037,7 @@
       <c r="Q285" s="9" t="n"/>
       <c r="R285" s="9" t="n"/>
       <c r="S285" s="9" t="n"/>
+      <c r="T285" s="9" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="9" t="n"/>
@@ -7477,6 +8059,7 @@
       <c r="Q286" s="9" t="n"/>
       <c r="R286" s="9" t="n"/>
       <c r="S286" s="9" t="n"/>
+      <c r="T286" s="9" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="9" t="n"/>
@@ -7498,6 +8081,7 @@
       <c r="Q287" s="9" t="n"/>
       <c r="R287" s="9" t="n"/>
       <c r="S287" s="9" t="n"/>
+      <c r="T287" s="9" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="9" t="n"/>
@@ -7519,6 +8103,7 @@
       <c r="Q288" s="9" t="n"/>
       <c r="R288" s="9" t="n"/>
       <c r="S288" s="9" t="n"/>
+      <c r="T288" s="9" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="9" t="n"/>
@@ -7540,6 +8125,7 @@
       <c r="Q289" s="9" t="n"/>
       <c r="R289" s="9" t="n"/>
       <c r="S289" s="9" t="n"/>
+      <c r="T289" s="9" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="9" t="n"/>
@@ -7561,6 +8147,7 @@
       <c r="Q290" s="9" t="n"/>
       <c r="R290" s="9" t="n"/>
       <c r="S290" s="9" t="n"/>
+      <c r="T290" s="9" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="9" t="n"/>
@@ -7582,6 +8169,7 @@
       <c r="Q291" s="9" t="n"/>
       <c r="R291" s="9" t="n"/>
       <c r="S291" s="9" t="n"/>
+      <c r="T291" s="9" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="9" t="n"/>
@@ -7603,6 +8191,7 @@
       <c r="Q292" s="9" t="n"/>
       <c r="R292" s="9" t="n"/>
       <c r="S292" s="9" t="n"/>
+      <c r="T292" s="9" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="9" t="n"/>
@@ -7624,6 +8213,7 @@
       <c r="Q293" s="9" t="n"/>
       <c r="R293" s="9" t="n"/>
       <c r="S293" s="9" t="n"/>
+      <c r="T293" s="9" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="9" t="n"/>
@@ -7645,6 +8235,7 @@
       <c r="Q294" s="9" t="n"/>
       <c r="R294" s="9" t="n"/>
       <c r="S294" s="9" t="n"/>
+      <c r="T294" s="9" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="9" t="n"/>
@@ -7666,6 +8257,7 @@
       <c r="Q295" s="9" t="n"/>
       <c r="R295" s="9" t="n"/>
       <c r="S295" s="9" t="n"/>
+      <c r="T295" s="9" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="9" t="n"/>
@@ -7687,6 +8279,7 @@
       <c r="Q296" s="9" t="n"/>
       <c r="R296" s="9" t="n"/>
       <c r="S296" s="9" t="n"/>
+      <c r="T296" s="9" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="9" t="n"/>
@@ -7708,6 +8301,7 @@
       <c r="Q297" s="9" t="n"/>
       <c r="R297" s="9" t="n"/>
       <c r="S297" s="9" t="n"/>
+      <c r="T297" s="9" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="9" t="n"/>
@@ -7729,6 +8323,7 @@
       <c r="Q298" s="9" t="n"/>
       <c r="R298" s="9" t="n"/>
       <c r="S298" s="9" t="n"/>
+      <c r="T298" s="9" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="9" t="n"/>
@@ -7750,6 +8345,7 @@
       <c r="Q299" s="9" t="n"/>
       <c r="R299" s="9" t="n"/>
       <c r="S299" s="9" t="n"/>
+      <c r="T299" s="9" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="9" t="n"/>
@@ -7771,6 +8367,7 @@
       <c r="Q300" s="9" t="n"/>
       <c r="R300" s="9" t="n"/>
       <c r="S300" s="9" t="n"/>
+      <c r="T300" s="9" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="9" t="n"/>
@@ -7792,6 +8389,7 @@
       <c r="Q301" s="9" t="n"/>
       <c r="R301" s="9" t="n"/>
       <c r="S301" s="9" t="n"/>
+      <c r="T301" s="9" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="9" t="n"/>
@@ -7813,6 +8411,7 @@
       <c r="Q302" s="9" t="n"/>
       <c r="R302" s="9" t="n"/>
       <c r="S302" s="9" t="n"/>
+      <c r="T302" s="9" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="9" t="n"/>
@@ -7834,6 +8433,7 @@
       <c r="Q303" s="9" t="n"/>
       <c r="R303" s="9" t="n"/>
       <c r="S303" s="9" t="n"/>
+      <c r="T303" s="9" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="9" t="n"/>
@@ -7855,6 +8455,7 @@
       <c r="Q304" s="9" t="n"/>
       <c r="R304" s="9" t="n"/>
       <c r="S304" s="9" t="n"/>
+      <c r="T304" s="9" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="9" t="n"/>
@@ -7876,6 +8477,7 @@
       <c r="Q305" s="9" t="n"/>
       <c r="R305" s="9" t="n"/>
       <c r="S305" s="9" t="n"/>
+      <c r="T305" s="9" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="9" t="n"/>
@@ -7897,6 +8499,7 @@
       <c r="Q306" s="9" t="n"/>
       <c r="R306" s="9" t="n"/>
       <c r="S306" s="9" t="n"/>
+      <c r="T306" s="9" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="9" t="n"/>
@@ -7918,6 +8521,7 @@
       <c r="Q307" s="9" t="n"/>
       <c r="R307" s="9" t="n"/>
       <c r="S307" s="9" t="n"/>
+      <c r="T307" s="9" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="9" t="n"/>
@@ -7939,6 +8543,7 @@
       <c r="Q308" s="9" t="n"/>
       <c r="R308" s="9" t="n"/>
       <c r="S308" s="9" t="n"/>
+      <c r="T308" s="9" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="9" t="n"/>
@@ -7960,6 +8565,7 @@
       <c r="Q309" s="9" t="n"/>
       <c r="R309" s="9" t="n"/>
       <c r="S309" s="9" t="n"/>
+      <c r="T309" s="9" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="9" t="n"/>
@@ -7981,6 +8587,7 @@
       <c r="Q310" s="9" t="n"/>
       <c r="R310" s="9" t="n"/>
       <c r="S310" s="9" t="n"/>
+      <c r="T310" s="9" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="9" t="n"/>
@@ -8002,6 +8609,7 @@
       <c r="Q311" s="9" t="n"/>
       <c r="R311" s="9" t="n"/>
       <c r="S311" s="9" t="n"/>
+      <c r="T311" s="9" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="9" t="n"/>
@@ -8023,6 +8631,7 @@
       <c r="Q312" s="9" t="n"/>
       <c r="R312" s="9" t="n"/>
       <c r="S312" s="9" t="n"/>
+      <c r="T312" s="9" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="9" t="n"/>
@@ -8044,6 +8653,7 @@
       <c r="Q313" s="9" t="n"/>
       <c r="R313" s="9" t="n"/>
       <c r="S313" s="9" t="n"/>
+      <c r="T313" s="9" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="9" t="n"/>
@@ -8065,6 +8675,7 @@
       <c r="Q314" s="9" t="n"/>
       <c r="R314" s="9" t="n"/>
       <c r="S314" s="9" t="n"/>
+      <c r="T314" s="9" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="9" t="n"/>
@@ -8086,6 +8697,7 @@
       <c r="Q315" s="9" t="n"/>
       <c r="R315" s="9" t="n"/>
       <c r="S315" s="9" t="n"/>
+      <c r="T315" s="9" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="9" t="n"/>
@@ -8107,6 +8719,7 @@
       <c r="Q316" s="9" t="n"/>
       <c r="R316" s="9" t="n"/>
       <c r="S316" s="9" t="n"/>
+      <c r="T316" s="9" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="9" t="n"/>
@@ -8128,6 +8741,7 @@
       <c r="Q317" s="9" t="n"/>
       <c r="R317" s="9" t="n"/>
       <c r="S317" s="9" t="n"/>
+      <c r="T317" s="9" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="9" t="n"/>
@@ -8149,6 +8763,7 @@
       <c r="Q318" s="9" t="n"/>
       <c r="R318" s="9" t="n"/>
       <c r="S318" s="9" t="n"/>
+      <c r="T318" s="9" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="9" t="n"/>
@@ -8170,6 +8785,7 @@
       <c r="Q319" s="9" t="n"/>
       <c r="R319" s="9" t="n"/>
       <c r="S319" s="9" t="n"/>
+      <c r="T319" s="9" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="9" t="n"/>
@@ -8191,6 +8807,7 @@
       <c r="Q320" s="9" t="n"/>
       <c r="R320" s="9" t="n"/>
       <c r="S320" s="9" t="n"/>
+      <c r="T320" s="9" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="9" t="n"/>
@@ -8212,6 +8829,7 @@
       <c r="Q321" s="9" t="n"/>
       <c r="R321" s="9" t="n"/>
       <c r="S321" s="9" t="n"/>
+      <c r="T321" s="9" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="9" t="n"/>
@@ -8233,6 +8851,7 @@
       <c r="Q322" s="9" t="n"/>
       <c r="R322" s="9" t="n"/>
       <c r="S322" s="9" t="n"/>
+      <c r="T322" s="9" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="9" t="n"/>
@@ -8254,6 +8873,7 @@
       <c r="Q323" s="9" t="n"/>
       <c r="R323" s="9" t="n"/>
       <c r="S323" s="9" t="n"/>
+      <c r="T323" s="9" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="9" t="n"/>
@@ -8275,6 +8895,7 @@
       <c r="Q324" s="9" t="n"/>
       <c r="R324" s="9" t="n"/>
       <c r="S324" s="9" t="n"/>
+      <c r="T324" s="9" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="9" t="n"/>
@@ -8296,6 +8917,7 @@
       <c r="Q325" s="9" t="n"/>
       <c r="R325" s="9" t="n"/>
       <c r="S325" s="9" t="n"/>
+      <c r="T325" s="9" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="9" t="n"/>
@@ -8317,6 +8939,7 @@
       <c r="Q326" s="9" t="n"/>
       <c r="R326" s="9" t="n"/>
       <c r="S326" s="9" t="n"/>
+      <c r="T326" s="9" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="9" t="n"/>
@@ -8338,6 +8961,7 @@
       <c r="Q327" s="9" t="n"/>
       <c r="R327" s="9" t="n"/>
       <c r="S327" s="9" t="n"/>
+      <c r="T327" s="9" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="9" t="n"/>
@@ -8359,6 +8983,7 @@
       <c r="Q328" s="9" t="n"/>
       <c r="R328" s="9" t="n"/>
       <c r="S328" s="9" t="n"/>
+      <c r="T328" s="9" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="9" t="n"/>
@@ -8380,6 +9005,7 @@
       <c r="Q329" s="9" t="n"/>
       <c r="R329" s="9" t="n"/>
       <c r="S329" s="9" t="n"/>
+      <c r="T329" s="9" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="9" t="n"/>
@@ -8401,6 +9027,7 @@
       <c r="Q330" s="9" t="n"/>
       <c r="R330" s="9" t="n"/>
       <c r="S330" s="9" t="n"/>
+      <c r="T330" s="9" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="9" t="n"/>
@@ -8422,6 +9049,7 @@
       <c r="Q331" s="9" t="n"/>
       <c r="R331" s="9" t="n"/>
       <c r="S331" s="9" t="n"/>
+      <c r="T331" s="9" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="9" t="n"/>
@@ -8443,6 +9071,7 @@
       <c r="Q332" s="9" t="n"/>
       <c r="R332" s="9" t="n"/>
       <c r="S332" s="9" t="n"/>
+      <c r="T332" s="9" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="9" t="n"/>
@@ -8464,6 +9093,7 @@
       <c r="Q333" s="9" t="n"/>
       <c r="R333" s="9" t="n"/>
       <c r="S333" s="9" t="n"/>
+      <c r="T333" s="9" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="9" t="n"/>
@@ -8485,6 +9115,7 @@
       <c r="Q334" s="9" t="n"/>
       <c r="R334" s="9" t="n"/>
       <c r="S334" s="9" t="n"/>
+      <c r="T334" s="9" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="9" t="n"/>
@@ -8506,6 +9137,7 @@
       <c r="Q335" s="9" t="n"/>
       <c r="R335" s="9" t="n"/>
       <c r="S335" s="9" t="n"/>
+      <c r="T335" s="9" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="9" t="n"/>
@@ -8527,6 +9159,7 @@
       <c r="Q336" s="9" t="n"/>
       <c r="R336" s="9" t="n"/>
       <c r="S336" s="9" t="n"/>
+      <c r="T336" s="9" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="9" t="n"/>
@@ -8548,6 +9181,7 @@
       <c r="Q337" s="9" t="n"/>
       <c r="R337" s="9" t="n"/>
       <c r="S337" s="9" t="n"/>
+      <c r="T337" s="9" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="9" t="n"/>
@@ -8569,6 +9203,7 @@
       <c r="Q338" s="9" t="n"/>
       <c r="R338" s="9" t="n"/>
       <c r="S338" s="9" t="n"/>
+      <c r="T338" s="9" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="9" t="n"/>
@@ -8590,6 +9225,7 @@
       <c r="Q339" s="9" t="n"/>
       <c r="R339" s="9" t="n"/>
       <c r="S339" s="9" t="n"/>
+      <c r="T339" s="9" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="9" t="n"/>
@@ -8611,6 +9247,7 @@
       <c r="Q340" s="9" t="n"/>
       <c r="R340" s="9" t="n"/>
       <c r="S340" s="9" t="n"/>
+      <c r="T340" s="9" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="9" t="n"/>
@@ -8632,6 +9269,7 @@
       <c r="Q341" s="9" t="n"/>
       <c r="R341" s="9" t="n"/>
       <c r="S341" s="9" t="n"/>
+      <c r="T341" s="9" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="9" t="n"/>
@@ -8653,6 +9291,7 @@
       <c r="Q342" s="9" t="n"/>
       <c r="R342" s="9" t="n"/>
       <c r="S342" s="9" t="n"/>
+      <c r="T342" s="9" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="9" t="n"/>
@@ -8674,6 +9313,7 @@
       <c r="Q343" s="9" t="n"/>
       <c r="R343" s="9" t="n"/>
       <c r="S343" s="9" t="n"/>
+      <c r="T343" s="9" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="9" t="n"/>
@@ -8695,6 +9335,7 @@
       <c r="Q344" s="9" t="n"/>
       <c r="R344" s="9" t="n"/>
       <c r="S344" s="9" t="n"/>
+      <c r="T344" s="9" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="9" t="n"/>
@@ -8716,6 +9357,7 @@
       <c r="Q345" s="9" t="n"/>
       <c r="R345" s="9" t="n"/>
       <c r="S345" s="9" t="n"/>
+      <c r="T345" s="9" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="9" t="n"/>
@@ -8737,6 +9379,7 @@
       <c r="Q346" s="9" t="n"/>
       <c r="R346" s="9" t="n"/>
       <c r="S346" s="9" t="n"/>
+      <c r="T346" s="9" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="9" t="n"/>
@@ -8758,6 +9401,7 @@
       <c r="Q347" s="9" t="n"/>
       <c r="R347" s="9" t="n"/>
       <c r="S347" s="9" t="n"/>
+      <c r="T347" s="9" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="9" t="n"/>
@@ -8779,6 +9423,7 @@
       <c r="Q348" s="9" t="n"/>
       <c r="R348" s="9" t="n"/>
       <c r="S348" s="9" t="n"/>
+      <c r="T348" s="9" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="9" t="n"/>
@@ -8800,6 +9445,7 @@
       <c r="Q349" s="9" t="n"/>
       <c r="R349" s="9" t="n"/>
       <c r="S349" s="9" t="n"/>
+      <c r="T349" s="9" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="9" t="n"/>
@@ -8821,6 +9467,7 @@
       <c r="Q350" s="9" t="n"/>
       <c r="R350" s="9" t="n"/>
       <c r="S350" s="9" t="n"/>
+      <c r="T350" s="9" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="9" t="n"/>
@@ -8842,6 +9489,7 @@
       <c r="Q351" s="9" t="n"/>
       <c r="R351" s="9" t="n"/>
       <c r="S351" s="9" t="n"/>
+      <c r="T351" s="9" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="9" t="n"/>
@@ -8863,6 +9511,7 @@
       <c r="Q352" s="9" t="n"/>
       <c r="R352" s="9" t="n"/>
       <c r="S352" s="9" t="n"/>
+      <c r="T352" s="9" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="9" t="n"/>
@@ -8884,6 +9533,7 @@
       <c r="Q353" s="9" t="n"/>
       <c r="R353" s="9" t="n"/>
       <c r="S353" s="9" t="n"/>
+      <c r="T353" s="9" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="9" t="n"/>
@@ -8905,6 +9555,7 @@
       <c r="Q354" s="9" t="n"/>
       <c r="R354" s="9" t="n"/>
       <c r="S354" s="9" t="n"/>
+      <c r="T354" s="9" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="9" t="n"/>
@@ -8926,6 +9577,7 @@
       <c r="Q355" s="9" t="n"/>
       <c r="R355" s="9" t="n"/>
       <c r="S355" s="9" t="n"/>
+      <c r="T355" s="9" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="9" t="n"/>
@@ -8947,6 +9599,7 @@
       <c r="Q356" s="9" t="n"/>
       <c r="R356" s="9" t="n"/>
       <c r="S356" s="9" t="n"/>
+      <c r="T356" s="9" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="9" t="n"/>
@@ -8968,6 +9621,7 @@
       <c r="Q357" s="9" t="n"/>
       <c r="R357" s="9" t="n"/>
       <c r="S357" s="9" t="n"/>
+      <c r="T357" s="9" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="9" t="n"/>
@@ -8989,6 +9643,7 @@
       <c r="Q358" s="9" t="n"/>
       <c r="R358" s="9" t="n"/>
       <c r="S358" s="9" t="n"/>
+      <c r="T358" s="9" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="9" t="n"/>
@@ -9010,6 +9665,7 @@
       <c r="Q359" s="9" t="n"/>
       <c r="R359" s="9" t="n"/>
       <c r="S359" s="9" t="n"/>
+      <c r="T359" s="9" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="9" t="n"/>
@@ -9031,6 +9687,7 @@
       <c r="Q360" s="9" t="n"/>
       <c r="R360" s="9" t="n"/>
       <c r="S360" s="9" t="n"/>
+      <c r="T360" s="9" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="9" t="n"/>
@@ -9052,6 +9709,7 @@
       <c r="Q361" s="9" t="n"/>
       <c r="R361" s="9" t="n"/>
       <c r="S361" s="9" t="n"/>
+      <c r="T361" s="9" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="9" t="n"/>
@@ -9073,6 +9731,7 @@
       <c r="Q362" s="9" t="n"/>
       <c r="R362" s="9" t="n"/>
       <c r="S362" s="9" t="n"/>
+      <c r="T362" s="9" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="9" t="n"/>
@@ -9094,6 +9753,7 @@
       <c r="Q363" s="9" t="n"/>
       <c r="R363" s="9" t="n"/>
       <c r="S363" s="9" t="n"/>
+      <c r="T363" s="9" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="9" t="n"/>
@@ -9115,6 +9775,7 @@
       <c r="Q364" s="9" t="n"/>
       <c r="R364" s="9" t="n"/>
       <c r="S364" s="9" t="n"/>
+      <c r="T364" s="9" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="9" t="n"/>
@@ -9136,6 +9797,7 @@
       <c r="Q365" s="9" t="n"/>
       <c r="R365" s="9" t="n"/>
       <c r="S365" s="9" t="n"/>
+      <c r="T365" s="9" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="9" t="n"/>
@@ -9157,6 +9819,7 @@
       <c r="Q366" s="9" t="n"/>
       <c r="R366" s="9" t="n"/>
       <c r="S366" s="9" t="n"/>
+      <c r="T366" s="9" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="9" t="n"/>
@@ -9178,6 +9841,7 @@
       <c r="Q367" s="9" t="n"/>
       <c r="R367" s="9" t="n"/>
       <c r="S367" s="9" t="n"/>
+      <c r="T367" s="9" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="9" t="n"/>
@@ -9199,6 +9863,7 @@
       <c r="Q368" s="9" t="n"/>
       <c r="R368" s="9" t="n"/>
       <c r="S368" s="9" t="n"/>
+      <c r="T368" s="9" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="9" t="n"/>
@@ -9220,6 +9885,7 @@
       <c r="Q369" s="9" t="n"/>
       <c r="R369" s="9" t="n"/>
       <c r="S369" s="9" t="n"/>
+      <c r="T369" s="9" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="9" t="n"/>
@@ -9241,6 +9907,7 @@
       <c r="Q370" s="9" t="n"/>
       <c r="R370" s="9" t="n"/>
       <c r="S370" s="9" t="n"/>
+      <c r="T370" s="9" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="9" t="n"/>
@@ -9262,6 +9929,7 @@
       <c r="Q371" s="9" t="n"/>
       <c r="R371" s="9" t="n"/>
       <c r="S371" s="9" t="n"/>
+      <c r="T371" s="9" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="9" t="n"/>
@@ -9283,6 +9951,7 @@
       <c r="Q372" s="9" t="n"/>
       <c r="R372" s="9" t="n"/>
       <c r="S372" s="9" t="n"/>
+      <c r="T372" s="9" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="9" t="n"/>
@@ -9304,6 +9973,7 @@
       <c r="Q373" s="9" t="n"/>
       <c r="R373" s="9" t="n"/>
       <c r="S373" s="9" t="n"/>
+      <c r="T373" s="9" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="9" t="n"/>
@@ -9325,6 +9995,7 @@
       <c r="Q374" s="9" t="n"/>
       <c r="R374" s="9" t="n"/>
       <c r="S374" s="9" t="n"/>
+      <c r="T374" s="9" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="9" t="n"/>
@@ -9346,6 +10017,7 @@
       <c r="Q375" s="9" t="n"/>
       <c r="R375" s="9" t="n"/>
       <c r="S375" s="9" t="n"/>
+      <c r="T375" s="9" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="9" t="n"/>
@@ -9367,6 +10039,7 @@
       <c r="Q376" s="9" t="n"/>
       <c r="R376" s="9" t="n"/>
       <c r="S376" s="9" t="n"/>
+      <c r="T376" s="9" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="9" t="n"/>
@@ -9388,6 +10061,7 @@
       <c r="Q377" s="9" t="n"/>
       <c r="R377" s="9" t="n"/>
       <c r="S377" s="9" t="n"/>
+      <c r="T377" s="9" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="9" t="n"/>
@@ -9409,6 +10083,7 @@
       <c r="Q378" s="9" t="n"/>
       <c r="R378" s="9" t="n"/>
       <c r="S378" s="9" t="n"/>
+      <c r="T378" s="9" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="9" t="n"/>
@@ -9430,6 +10105,7 @@
       <c r="Q379" s="9" t="n"/>
       <c r="R379" s="9" t="n"/>
       <c r="S379" s="9" t="n"/>
+      <c r="T379" s="9" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="9" t="n"/>
@@ -9451,6 +10127,7 @@
       <c r="Q380" s="9" t="n"/>
       <c r="R380" s="9" t="n"/>
       <c r="S380" s="9" t="n"/>
+      <c r="T380" s="9" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="9" t="n"/>
@@ -9472,6 +10149,7 @@
       <c r="Q381" s="9" t="n"/>
       <c r="R381" s="9" t="n"/>
       <c r="S381" s="9" t="n"/>
+      <c r="T381" s="9" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="9" t="n"/>
@@ -9493,6 +10171,7 @@
       <c r="Q382" s="9" t="n"/>
       <c r="R382" s="9" t="n"/>
       <c r="S382" s="9" t="n"/>
+      <c r="T382" s="9" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="9" t="n"/>
@@ -9514,6 +10193,7 @@
       <c r="Q383" s="9" t="n"/>
       <c r="R383" s="9" t="n"/>
       <c r="S383" s="9" t="n"/>
+      <c r="T383" s="9" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="9" t="n"/>
@@ -9535,6 +10215,7 @@
       <c r="Q384" s="9" t="n"/>
       <c r="R384" s="9" t="n"/>
       <c r="S384" s="9" t="n"/>
+      <c r="T384" s="9" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="9" t="n"/>
@@ -9556,6 +10237,7 @@
       <c r="Q385" s="9" t="n"/>
       <c r="R385" s="9" t="n"/>
       <c r="S385" s="9" t="n"/>
+      <c r="T385" s="9" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="9" t="n"/>
@@ -9577,6 +10259,7 @@
       <c r="Q386" s="9" t="n"/>
       <c r="R386" s="9" t="n"/>
       <c r="S386" s="9" t="n"/>
+      <c r="T386" s="9" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="9" t="n"/>
@@ -9598,6 +10281,7 @@
       <c r="Q387" s="9" t="n"/>
       <c r="R387" s="9" t="n"/>
       <c r="S387" s="9" t="n"/>
+      <c r="T387" s="9" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="9" t="n"/>
@@ -9619,6 +10303,7 @@
       <c r="Q388" s="9" t="n"/>
       <c r="R388" s="9" t="n"/>
       <c r="S388" s="9" t="n"/>
+      <c r="T388" s="9" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="9" t="n"/>
@@ -9640,6 +10325,7 @@
       <c r="Q389" s="9" t="n"/>
       <c r="R389" s="9" t="n"/>
       <c r="S389" s="9" t="n"/>
+      <c r="T389" s="9" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="9" t="n"/>
@@ -9661,6 +10347,7 @@
       <c r="Q390" s="9" t="n"/>
       <c r="R390" s="9" t="n"/>
       <c r="S390" s="9" t="n"/>
+      <c r="T390" s="9" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="9" t="n"/>
@@ -9682,6 +10369,7 @@
       <c r="Q391" s="9" t="n"/>
       <c r="R391" s="9" t="n"/>
       <c r="S391" s="9" t="n"/>
+      <c r="T391" s="9" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="9" t="n"/>
@@ -9703,6 +10391,7 @@
       <c r="Q392" s="9" t="n"/>
       <c r="R392" s="9" t="n"/>
       <c r="S392" s="9" t="n"/>
+      <c r="T392" s="9" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="9" t="n"/>
@@ -9724,6 +10413,7 @@
       <c r="Q393" s="9" t="n"/>
       <c r="R393" s="9" t="n"/>
       <c r="S393" s="9" t="n"/>
+      <c r="T393" s="9" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="9" t="n"/>
@@ -9745,6 +10435,7 @@
       <c r="Q394" s="9" t="n"/>
       <c r="R394" s="9" t="n"/>
       <c r="S394" s="9" t="n"/>
+      <c r="T394" s="9" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="9" t="n"/>
@@ -9766,6 +10457,7 @@
       <c r="Q395" s="9" t="n"/>
       <c r="R395" s="9" t="n"/>
       <c r="S395" s="9" t="n"/>
+      <c r="T395" s="9" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="9" t="n"/>
@@ -9787,6 +10479,7 @@
       <c r="Q396" s="9" t="n"/>
       <c r="R396" s="9" t="n"/>
       <c r="S396" s="9" t="n"/>
+      <c r="T396" s="9" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="9" t="n"/>
@@ -9808,6 +10501,7 @@
       <c r="Q397" s="9" t="n"/>
       <c r="R397" s="9" t="n"/>
       <c r="S397" s="9" t="n"/>
+      <c r="T397" s="9" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="9" t="n"/>
@@ -9829,6 +10523,7 @@
       <c r="Q398" s="9" t="n"/>
       <c r="R398" s="9" t="n"/>
       <c r="S398" s="9" t="n"/>
+      <c r="T398" s="9" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="9" t="n"/>
@@ -9850,6 +10545,7 @@
       <c r="Q399" s="9" t="n"/>
       <c r="R399" s="9" t="n"/>
       <c r="S399" s="9" t="n"/>
+      <c r="T399" s="9" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="9" t="n"/>
@@ -9871,6 +10567,7 @@
       <c r="Q400" s="9" t="n"/>
       <c r="R400" s="9" t="n"/>
       <c r="S400" s="9" t="n"/>
+      <c r="T400" s="9" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="9" t="n"/>
@@ -9892,6 +10589,7 @@
       <c r="Q401" s="9" t="n"/>
       <c r="R401" s="9" t="n"/>
       <c r="S401" s="9" t="n"/>
+      <c r="T401" s="9" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="9" t="n"/>
@@ -9913,6 +10611,7 @@
       <c r="Q402" s="9" t="n"/>
       <c r="R402" s="9" t="n"/>
       <c r="S402" s="9" t="n"/>
+      <c r="T402" s="9" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="9" t="n"/>
@@ -9934,6 +10633,7 @@
       <c r="Q403" s="9" t="n"/>
       <c r="R403" s="9" t="n"/>
       <c r="S403" s="9" t="n"/>
+      <c r="T403" s="9" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="9" t="n"/>
@@ -9955,6 +10655,7 @@
       <c r="Q404" s="9" t="n"/>
       <c r="R404" s="9" t="n"/>
       <c r="S404" s="9" t="n"/>
+      <c r="T404" s="9" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="9" t="n"/>
@@ -9976,6 +10677,7 @@
       <c r="Q405" s="9" t="n"/>
       <c r="R405" s="9" t="n"/>
       <c r="S405" s="9" t="n"/>
+      <c r="T405" s="9" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="9" t="n"/>
@@ -9997,6 +10699,7 @@
       <c r="Q406" s="9" t="n"/>
       <c r="R406" s="9" t="n"/>
       <c r="S406" s="9" t="n"/>
+      <c r="T406" s="9" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="9" t="n"/>
@@ -10018,6 +10721,7 @@
       <c r="Q407" s="9" t="n"/>
       <c r="R407" s="9" t="n"/>
       <c r="S407" s="9" t="n"/>
+      <c r="T407" s="9" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="9" t="n"/>
@@ -10039,6 +10743,7 @@
       <c r="Q408" s="9" t="n"/>
       <c r="R408" s="9" t="n"/>
       <c r="S408" s="9" t="n"/>
+      <c r="T408" s="9" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="9" t="n"/>
@@ -10060,6 +10765,7 @@
       <c r="Q409" s="9" t="n"/>
       <c r="R409" s="9" t="n"/>
       <c r="S409" s="9" t="n"/>
+      <c r="T409" s="9" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="9" t="n"/>
@@ -10081,6 +10787,7 @@
       <c r="Q410" s="9" t="n"/>
       <c r="R410" s="9" t="n"/>
       <c r="S410" s="9" t="n"/>
+      <c r="T410" s="9" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="9" t="n"/>
@@ -10102,6 +10809,7 @@
       <c r="Q411" s="9" t="n"/>
       <c r="R411" s="9" t="n"/>
       <c r="S411" s="9" t="n"/>
+      <c r="T411" s="9" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="9" t="n"/>
@@ -10123,6 +10831,7 @@
       <c r="Q412" s="9" t="n"/>
       <c r="R412" s="9" t="n"/>
       <c r="S412" s="9" t="n"/>
+      <c r="T412" s="9" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="9" t="n"/>
@@ -10144,6 +10853,7 @@
       <c r="Q413" s="9" t="n"/>
       <c r="R413" s="9" t="n"/>
       <c r="S413" s="9" t="n"/>
+      <c r="T413" s="9" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="9" t="n"/>
@@ -10165,6 +10875,7 @@
       <c r="Q414" s="9" t="n"/>
       <c r="R414" s="9" t="n"/>
       <c r="S414" s="9" t="n"/>
+      <c r="T414" s="9" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="9" t="n"/>
@@ -10186,6 +10897,7 @@
       <c r="Q415" s="9" t="n"/>
       <c r="R415" s="9" t="n"/>
       <c r="S415" s="9" t="n"/>
+      <c r="T415" s="9" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="9" t="n"/>
@@ -10207,6 +10919,7 @@
       <c r="Q416" s="9" t="n"/>
       <c r="R416" s="9" t="n"/>
       <c r="S416" s="9" t="n"/>
+      <c r="T416" s="9" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="9" t="n"/>
@@ -10228,6 +10941,7 @@
       <c r="Q417" s="9" t="n"/>
       <c r="R417" s="9" t="n"/>
       <c r="S417" s="9" t="n"/>
+      <c r="T417" s="9" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="9" t="n"/>
@@ -10249,6 +10963,7 @@
       <c r="Q418" s="9" t="n"/>
       <c r="R418" s="9" t="n"/>
       <c r="S418" s="9" t="n"/>
+      <c r="T418" s="9" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="9" t="n"/>
@@ -10270,6 +10985,7 @@
       <c r="Q419" s="9" t="n"/>
       <c r="R419" s="9" t="n"/>
       <c r="S419" s="9" t="n"/>
+      <c r="T419" s="9" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="9" t="n"/>
@@ -10291,6 +11007,7 @@
       <c r="Q420" s="9" t="n"/>
       <c r="R420" s="9" t="n"/>
       <c r="S420" s="9" t="n"/>
+      <c r="T420" s="9" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="9" t="n"/>
@@ -10312,6 +11029,7 @@
       <c r="Q421" s="9" t="n"/>
       <c r="R421" s="9" t="n"/>
       <c r="S421" s="9" t="n"/>
+      <c r="T421" s="9" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="9" t="n"/>
@@ -10333,6 +11051,7 @@
       <c r="Q422" s="9" t="n"/>
       <c r="R422" s="9" t="n"/>
       <c r="S422" s="9" t="n"/>
+      <c r="T422" s="9" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="9" t="n"/>
@@ -10354,6 +11073,7 @@
       <c r="Q423" s="9" t="n"/>
       <c r="R423" s="9" t="n"/>
       <c r="S423" s="9" t="n"/>
+      <c r="T423" s="9" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="9" t="n"/>
@@ -10375,6 +11095,7 @@
       <c r="Q424" s="9" t="n"/>
       <c r="R424" s="9" t="n"/>
       <c r="S424" s="9" t="n"/>
+      <c r="T424" s="9" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="9" t="n"/>
@@ -10396,6 +11117,7 @@
       <c r="Q425" s="9" t="n"/>
       <c r="R425" s="9" t="n"/>
       <c r="S425" s="9" t="n"/>
+      <c r="T425" s="9" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="9" t="n"/>
@@ -10417,6 +11139,7 @@
       <c r="Q426" s="9" t="n"/>
       <c r="R426" s="9" t="n"/>
       <c r="S426" s="9" t="n"/>
+      <c r="T426" s="9" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="9" t="n"/>
@@ -10438,6 +11161,7 @@
       <c r="Q427" s="9" t="n"/>
       <c r="R427" s="9" t="n"/>
       <c r="S427" s="9" t="n"/>
+      <c r="T427" s="9" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="9" t="n"/>
@@ -10459,6 +11183,7 @@
       <c r="Q428" s="9" t="n"/>
       <c r="R428" s="9" t="n"/>
       <c r="S428" s="9" t="n"/>
+      <c r="T428" s="9" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="9" t="n"/>
@@ -10480,6 +11205,7 @@
       <c r="Q429" s="9" t="n"/>
       <c r="R429" s="9" t="n"/>
       <c r="S429" s="9" t="n"/>
+      <c r="T429" s="9" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="9" t="n"/>
@@ -10501,6 +11227,7 @@
       <c r="Q430" s="9" t="n"/>
       <c r="R430" s="9" t="n"/>
       <c r="S430" s="9" t="n"/>
+      <c r="T430" s="9" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="9" t="n"/>
@@ -10522,6 +11249,7 @@
       <c r="Q431" s="9" t="n"/>
       <c r="R431" s="9" t="n"/>
       <c r="S431" s="9" t="n"/>
+      <c r="T431" s="9" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="9" t="n"/>
@@ -10543,6 +11271,7 @@
       <c r="Q432" s="9" t="n"/>
       <c r="R432" s="9" t="n"/>
       <c r="S432" s="9" t="n"/>
+      <c r="T432" s="9" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="9" t="n"/>
@@ -10564,6 +11293,7 @@
       <c r="Q433" s="9" t="n"/>
       <c r="R433" s="9" t="n"/>
       <c r="S433" s="9" t="n"/>
+      <c r="T433" s="9" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="9" t="n"/>
@@ -10585,6 +11315,7 @@
       <c r="Q434" s="9" t="n"/>
       <c r="R434" s="9" t="n"/>
       <c r="S434" s="9" t="n"/>
+      <c r="T434" s="9" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="9" t="n"/>
@@ -10606,6 +11337,7 @@
       <c r="Q435" s="9" t="n"/>
       <c r="R435" s="9" t="n"/>
       <c r="S435" s="9" t="n"/>
+      <c r="T435" s="9" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="9" t="n"/>
@@ -10627,6 +11359,7 @@
       <c r="Q436" s="9" t="n"/>
       <c r="R436" s="9" t="n"/>
       <c r="S436" s="9" t="n"/>
+      <c r="T436" s="9" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="9" t="n"/>
@@ -10648,6 +11381,7 @@
       <c r="Q437" s="9" t="n"/>
       <c r="R437" s="9" t="n"/>
       <c r="S437" s="9" t="n"/>
+      <c r="T437" s="9" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="9" t="n"/>
@@ -10669,6 +11403,7 @@
       <c r="Q438" s="9" t="n"/>
       <c r="R438" s="9" t="n"/>
       <c r="S438" s="9" t="n"/>
+      <c r="T438" s="9" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="9" t="n"/>
@@ -10690,6 +11425,7 @@
       <c r="Q439" s="9" t="n"/>
       <c r="R439" s="9" t="n"/>
       <c r="S439" s="9" t="n"/>
+      <c r="T439" s="9" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="9" t="n"/>
@@ -10711,6 +11447,7 @@
       <c r="Q440" s="9" t="n"/>
       <c r="R440" s="9" t="n"/>
       <c r="S440" s="9" t="n"/>
+      <c r="T440" s="9" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="9" t="n"/>
@@ -10732,6 +11469,7 @@
       <c r="Q441" s="9" t="n"/>
       <c r="R441" s="9" t="n"/>
       <c r="S441" s="9" t="n"/>
+      <c r="T441" s="9" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="9" t="n"/>
@@ -10753,6 +11491,7 @@
       <c r="Q442" s="9" t="n"/>
       <c r="R442" s="9" t="n"/>
       <c r="S442" s="9" t="n"/>
+      <c r="T442" s="9" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="9" t="n"/>
@@ -10774,6 +11513,7 @@
       <c r="Q443" s="9" t="n"/>
       <c r="R443" s="9" t="n"/>
       <c r="S443" s="9" t="n"/>
+      <c r="T443" s="9" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="9" t="n"/>
@@ -10795,6 +11535,7 @@
       <c r="Q444" s="9" t="n"/>
       <c r="R444" s="9" t="n"/>
       <c r="S444" s="9" t="n"/>
+      <c r="T444" s="9" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="9" t="n"/>
@@ -10816,6 +11557,7 @@
       <c r="Q445" s="9" t="n"/>
       <c r="R445" s="9" t="n"/>
       <c r="S445" s="9" t="n"/>
+      <c r="T445" s="9" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="9" t="n"/>
@@ -10837,6 +11579,7 @@
       <c r="Q446" s="9" t="n"/>
       <c r="R446" s="9" t="n"/>
       <c r="S446" s="9" t="n"/>
+      <c r="T446" s="9" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="9" t="n"/>
@@ -10858,6 +11601,7 @@
       <c r="Q447" s="9" t="n"/>
       <c r="R447" s="9" t="n"/>
       <c r="S447" s="9" t="n"/>
+      <c r="T447" s="9" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="9" t="n"/>
@@ -10879,6 +11623,7 @@
       <c r="Q448" s="9" t="n"/>
       <c r="R448" s="9" t="n"/>
       <c r="S448" s="9" t="n"/>
+      <c r="T448" s="9" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="9" t="n"/>
@@ -10900,6 +11645,7 @@
       <c r="Q449" s="9" t="n"/>
       <c r="R449" s="9" t="n"/>
       <c r="S449" s="9" t="n"/>
+      <c r="T449" s="9" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="9" t="n"/>
@@ -10921,6 +11667,7 @@
       <c r="Q450" s="9" t="n"/>
       <c r="R450" s="9" t="n"/>
       <c r="S450" s="9" t="n"/>
+      <c r="T450" s="9" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="9" t="n"/>
@@ -10942,6 +11689,7 @@
       <c r="Q451" s="9" t="n"/>
       <c r="R451" s="9" t="n"/>
       <c r="S451" s="9" t="n"/>
+      <c r="T451" s="9" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="9" t="n"/>
@@ -10963,6 +11711,7 @@
       <c r="Q452" s="9" t="n"/>
       <c r="R452" s="9" t="n"/>
       <c r="S452" s="9" t="n"/>
+      <c r="T452" s="9" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="9" t="n"/>
@@ -10984,6 +11733,7 @@
       <c r="Q453" s="9" t="n"/>
       <c r="R453" s="9" t="n"/>
       <c r="S453" s="9" t="n"/>
+      <c r="T453" s="9" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="9" t="n"/>
@@ -11005,6 +11755,7 @@
       <c r="Q454" s="9" t="n"/>
       <c r="R454" s="9" t="n"/>
       <c r="S454" s="9" t="n"/>
+      <c r="T454" s="9" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="9" t="n"/>
@@ -11026,6 +11777,7 @@
       <c r="Q455" s="9" t="n"/>
       <c r="R455" s="9" t="n"/>
       <c r="S455" s="9" t="n"/>
+      <c r="T455" s="9" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="9" t="n"/>
@@ -11047,6 +11799,7 @@
       <c r="Q456" s="9" t="n"/>
       <c r="R456" s="9" t="n"/>
       <c r="S456" s="9" t="n"/>
+      <c r="T456" s="9" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="9" t="n"/>
@@ -11068,6 +11821,7 @@
       <c r="Q457" s="9" t="n"/>
       <c r="R457" s="9" t="n"/>
       <c r="S457" s="9" t="n"/>
+      <c r="T457" s="9" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="9" t="n"/>
@@ -11089,6 +11843,7 @@
       <c r="Q458" s="9" t="n"/>
       <c r="R458" s="9" t="n"/>
       <c r="S458" s="9" t="n"/>
+      <c r="T458" s="9" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="9" t="n"/>
@@ -11110,6 +11865,7 @@
       <c r="Q459" s="9" t="n"/>
       <c r="R459" s="9" t="n"/>
       <c r="S459" s="9" t="n"/>
+      <c r="T459" s="9" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="9" t="n"/>
@@ -11131,6 +11887,7 @@
       <c r="Q460" s="9" t="n"/>
       <c r="R460" s="9" t="n"/>
       <c r="S460" s="9" t="n"/>
+      <c r="T460" s="9" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="9" t="n"/>
@@ -11152,6 +11909,7 @@
       <c r="Q461" s="9" t="n"/>
       <c r="R461" s="9" t="n"/>
       <c r="S461" s="9" t="n"/>
+      <c r="T461" s="9" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="9" t="n"/>
@@ -11173,6 +11931,7 @@
       <c r="Q462" s="9" t="n"/>
       <c r="R462" s="9" t="n"/>
       <c r="S462" s="9" t="n"/>
+      <c r="T462" s="9" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="9" t="n"/>
@@ -11194,6 +11953,7 @@
       <c r="Q463" s="9" t="n"/>
       <c r="R463" s="9" t="n"/>
       <c r="S463" s="9" t="n"/>
+      <c r="T463" s="9" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="9" t="n"/>
@@ -11215,6 +11975,7 @@
       <c r="Q464" s="9" t="n"/>
       <c r="R464" s="9" t="n"/>
       <c r="S464" s="9" t="n"/>
+      <c r="T464" s="9" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="9" t="n"/>
@@ -11236,6 +11997,7 @@
       <c r="Q465" s="9" t="n"/>
       <c r="R465" s="9" t="n"/>
       <c r="S465" s="9" t="n"/>
+      <c r="T465" s="9" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="9" t="n"/>
@@ -11257,6 +12019,7 @@
       <c r="Q466" s="9" t="n"/>
       <c r="R466" s="9" t="n"/>
       <c r="S466" s="9" t="n"/>
+      <c r="T466" s="9" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="9" t="n"/>
@@ -11278,6 +12041,7 @@
       <c r="Q467" s="9" t="n"/>
       <c r="R467" s="9" t="n"/>
       <c r="S467" s="9" t="n"/>
+      <c r="T467" s="9" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="9" t="n"/>
@@ -11299,6 +12063,7 @@
       <c r="Q468" s="9" t="n"/>
       <c r="R468" s="9" t="n"/>
       <c r="S468" s="9" t="n"/>
+      <c r="T468" s="9" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="9" t="n"/>
@@ -11320,6 +12085,7 @@
       <c r="Q469" s="9" t="n"/>
       <c r="R469" s="9" t="n"/>
       <c r="S469" s="9" t="n"/>
+      <c r="T469" s="9" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="9" t="n"/>
@@ -11341,6 +12107,7 @@
       <c r="Q470" s="9" t="n"/>
       <c r="R470" s="9" t="n"/>
       <c r="S470" s="9" t="n"/>
+      <c r="T470" s="9" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="9" t="n"/>
@@ -11362,6 +12129,7 @@
       <c r="Q471" s="9" t="n"/>
       <c r="R471" s="9" t="n"/>
       <c r="S471" s="9" t="n"/>
+      <c r="T471" s="9" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="9" t="n"/>
@@ -11383,6 +12151,7 @@
       <c r="Q472" s="9" t="n"/>
       <c r="R472" s="9" t="n"/>
       <c r="S472" s="9" t="n"/>
+      <c r="T472" s="9" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="9" t="n"/>
@@ -11404,6 +12173,7 @@
       <c r="Q473" s="9" t="n"/>
       <c r="R473" s="9" t="n"/>
       <c r="S473" s="9" t="n"/>
+      <c r="T473" s="9" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="9" t="n"/>
@@ -11425,6 +12195,7 @@
       <c r="Q474" s="9" t="n"/>
       <c r="R474" s="9" t="n"/>
       <c r="S474" s="9" t="n"/>
+      <c r="T474" s="9" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="9" t="n"/>
@@ -11446,6 +12217,7 @@
       <c r="Q475" s="9" t="n"/>
       <c r="R475" s="9" t="n"/>
       <c r="S475" s="9" t="n"/>
+      <c r="T475" s="9" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="9" t="n"/>
@@ -11467,6 +12239,7 @@
       <c r="Q476" s="9" t="n"/>
       <c r="R476" s="9" t="n"/>
       <c r="S476" s="9" t="n"/>
+      <c r="T476" s="9" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="9" t="n"/>
@@ -11488,6 +12261,7 @@
       <c r="Q477" s="9" t="n"/>
       <c r="R477" s="9" t="n"/>
       <c r="S477" s="9" t="n"/>
+      <c r="T477" s="9" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="9" t="n"/>
@@ -11509,6 +12283,7 @@
       <c r="Q478" s="9" t="n"/>
       <c r="R478" s="9" t="n"/>
       <c r="S478" s="9" t="n"/>
+      <c r="T478" s="9" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="9" t="n"/>
@@ -11530,6 +12305,7 @@
       <c r="Q479" s="9" t="n"/>
       <c r="R479" s="9" t="n"/>
       <c r="S479" s="9" t="n"/>
+      <c r="T479" s="9" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="9" t="n"/>
@@ -11551,6 +12327,7 @@
       <c r="Q480" s="9" t="n"/>
       <c r="R480" s="9" t="n"/>
       <c r="S480" s="9" t="n"/>
+      <c r="T480" s="9" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="9" t="n"/>
@@ -11572,6 +12349,7 @@
       <c r="Q481" s="9" t="n"/>
       <c r="R481" s="9" t="n"/>
       <c r="S481" s="9" t="n"/>
+      <c r="T481" s="9" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="9" t="n"/>
@@ -11593,6 +12371,7 @@
       <c r="Q482" s="9" t="n"/>
       <c r="R482" s="9" t="n"/>
       <c r="S482" s="9" t="n"/>
+      <c r="T482" s="9" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="9" t="n"/>
@@ -11614,6 +12393,7 @@
       <c r="Q483" s="9" t="n"/>
       <c r="R483" s="9" t="n"/>
       <c r="S483" s="9" t="n"/>
+      <c r="T483" s="9" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="9" t="n"/>
@@ -11635,6 +12415,7 @@
       <c r="Q484" s="9" t="n"/>
       <c r="R484" s="9" t="n"/>
       <c r="S484" s="9" t="n"/>
+      <c r="T484" s="9" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="9" t="n"/>
@@ -11656,6 +12437,7 @@
       <c r="Q485" s="9" t="n"/>
       <c r="R485" s="9" t="n"/>
       <c r="S485" s="9" t="n"/>
+      <c r="T485" s="9" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="9" t="n"/>
@@ -11677,6 +12459,7 @@
       <c r="Q486" s="9" t="n"/>
       <c r="R486" s="9" t="n"/>
       <c r="S486" s="9" t="n"/>
+      <c r="T486" s="9" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="9" t="n"/>
@@ -11698,6 +12481,7 @@
       <c r="Q487" s="9" t="n"/>
       <c r="R487" s="9" t="n"/>
       <c r="S487" s="9" t="n"/>
+      <c r="T487" s="9" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="9" t="n"/>
@@ -11719,6 +12503,7 @@
       <c r="Q488" s="9" t="n"/>
       <c r="R488" s="9" t="n"/>
       <c r="S488" s="9" t="n"/>
+      <c r="T488" s="9" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="9" t="n"/>
@@ -11740,6 +12525,7 @@
       <c r="Q489" s="9" t="n"/>
       <c r="R489" s="9" t="n"/>
       <c r="S489" s="9" t="n"/>
+      <c r="T489" s="9" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="9" t="n"/>
@@ -11761,6 +12547,7 @@
       <c r="Q490" s="9" t="n"/>
       <c r="R490" s="9" t="n"/>
       <c r="S490" s="9" t="n"/>
+      <c r="T490" s="9" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="9" t="n"/>
@@ -11782,6 +12569,7 @@
       <c r="Q491" s="9" t="n"/>
       <c r="R491" s="9" t="n"/>
       <c r="S491" s="9" t="n"/>
+      <c r="T491" s="9" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="9" t="n"/>
@@ -11803,6 +12591,7 @@
       <c r="Q492" s="9" t="n"/>
       <c r="R492" s="9" t="n"/>
       <c r="S492" s="9" t="n"/>
+      <c r="T492" s="9" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="9" t="n"/>
@@ -11824,6 +12613,7 @@
       <c r="Q493" s="9" t="n"/>
       <c r="R493" s="9" t="n"/>
       <c r="S493" s="9" t="n"/>
+      <c r="T493" s="9" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="9" t="n"/>
@@ -11845,6 +12635,7 @@
       <c r="Q494" s="9" t="n"/>
       <c r="R494" s="9" t="n"/>
       <c r="S494" s="9" t="n"/>
+      <c r="T494" s="9" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="9" t="n"/>
@@ -11866,6 +12657,7 @@
       <c r="Q495" s="9" t="n"/>
       <c r="R495" s="9" t="n"/>
       <c r="S495" s="9" t="n"/>
+      <c r="T495" s="9" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="9" t="n"/>
@@ -11887,6 +12679,7 @@
       <c r="Q496" s="9" t="n"/>
       <c r="R496" s="9" t="n"/>
       <c r="S496" s="9" t="n"/>
+      <c r="T496" s="9" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="9" t="n"/>
@@ -11908,6 +12701,7 @@
       <c r="Q497" s="9" t="n"/>
       <c r="R497" s="9" t="n"/>
       <c r="S497" s="9" t="n"/>
+      <c r="T497" s="9" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="9" t="n"/>
@@ -11929,6 +12723,7 @@
       <c r="Q498" s="9" t="n"/>
       <c r="R498" s="9" t="n"/>
       <c r="S498" s="9" t="n"/>
+      <c r="T498" s="9" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="9" t="n"/>
@@ -11950,6 +12745,7 @@
       <c r="Q499" s="9" t="n"/>
       <c r="R499" s="9" t="n"/>
       <c r="S499" s="9" t="n"/>
+      <c r="T499" s="9" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="9" t="n"/>
@@ -11971,6 +12767,7 @@
       <c r="Q500" s="9" t="n"/>
       <c r="R500" s="9" t="n"/>
       <c r="S500" s="9" t="n"/>
+      <c r="T500" s="9" t="n"/>
     </row>
     <row r="501">
       <c r="A501" s="9" t="n"/>
@@ -11992,6 +12789,7 @@
       <c r="Q501" s="9" t="n"/>
       <c r="R501" s="9" t="n"/>
       <c r="S501" s="9" t="n"/>
+      <c r="T501" s="9" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="9">
@@ -12034,7 +12832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S5"/>
+  <dimension ref="A1:T5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12056,6 +12854,7 @@
     <col width="9" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
     <col width="28" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12154,6 +12953,11 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="T1" s="5" t="inlineStr">
+        <is>
+          <t>verified by</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -12247,6 +13051,11 @@
           <t>Unstuck: gear-and-circuit milestone at step 15 (6 steps later).</t>
         </is>
       </c>
+      <c r="T2" s="10" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -12334,6 +13143,11 @@
       <c r="S3" s="10" t="inlineStr">
         <is>
           <t>Not unstuck: detector fired again at step 29; next milestone at step 75.</t>
+        </is>
+      </c>
+      <c r="T3" s="10" t="inlineStr">
+        <is>
+          <t>pending</t>
         </is>
       </c>
     </row>
@@ -12415,6 +13229,11 @@
           <t>Not unstuck: detector fired again at step 65.</t>
         </is>
       </c>
+      <c r="T4" s="10" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -12506,6 +13325,11 @@
       <c r="S5" s="10" t="inlineStr">
         <is>
           <t>Unstuck: steam-power milestone at step 75 (10 steps later). Guidance text truncated here for display; the trajectory holds it in full.</t>
+        </is>
+      </c>
+      <c r="T5" s="10" t="inlineStr">
+        <is>
+          <t>pending</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add error code E10, no error (backstop)
D75. The step backstop asks for help every 20 quiet steps whether or not
the agent is stuck; E10 codes those requests instead of swelling E09.
The validator allows it only on a backstop request and with no
secondary code. The workbook gains the row, its drop-downs, and a
Summary rebuilt for ten codes; the pilot's steps 19 and 39 are
re-drafted as E10. Grid stuck events are pre-coded by Claude by hand in
a working session.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/codebook-v0.xlsx
+++ b/docs/codebook-v0.xlsx
@@ -592,7 +592,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>v0 (draft, 2026-10-19). Revised once after the E1 pilot (build-plan 5b); every annotation row carries the version it was coded under.</t>
+          <t>v0 (draft, 2026-10-19; E10 'No error (backstop)' added 2026-10-21, D75). Revised once after the E1 pilot (build-plan 5b); every annotation row carries the version it was coded under.</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1118,7 +1118,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Does not fit E01-E08. Describe it in the note; recurring 'other' notes become new codes in v1.</t>
+          <t>Does not fit any other code. Describe it in the note; recurring 'other' notes become new codes in v1.</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -1144,6 +1144,48 @@
       <c r="H10" s="7" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>No error (backstop)</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>The step backstop (D67) asked for help, but the agent was not stuck: it was making progress, and no error in the steps before explains the request.</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>The stuck reason is the backstop's ('N steps without a request for help') and the ~5 steps before show normal progress: no repeated failure, no misread, no environment fault.</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Any identifiable error in that window - code the error instead, even though the backstop fired. Never with a repeated-error stuck reason. No secondary code.</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Stuck reason '20 steps without a request for help'; clean steps; inventory, entities or milestones growing.</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Harness (detector)</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Cell 5 pilot 20261021T162318-3e77267c, step 19: building drills and furnaces and collecting plates when the backstop fired.</t>
         </is>
       </c>
     </row>
@@ -1536,13 +1578,13 @@
       </c>
       <c r="I2" s="8" t="inlineStr">
         <is>
-          <t>E09</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="J2" s="8" t="n"/>
       <c r="K2" s="8" t="inlineStr">
         <is>
-          <t>No error found: steps 15-19 the agent was building copper/iron drills and furnaces and collecting plates normally. The 20-step backstop fired (D67) without the agent being stuck - candidate for a v1 'false alarm' code.</t>
+          <t>Steps 15-19: building copper/iron drills and furnaces and collecting plates normally when the 20-step backstop fired (D67).</t>
         </is>
       </c>
       <c r="L2" s="8" t="n"/>
@@ -1604,13 +1646,13 @@
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
-          <t>E09</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="J3" s="8" t="n"/>
       <c r="K3" s="8" t="inlineStr">
         <is>
-          <t>No clear error: steps 35-39 normal progress (automation researched at step 33, logistics research running, assemblers crafted); coal ran out (coal=0) at step 39. Backstop fired (D67) - candidate for a v1 'false alarm' code.</t>
+          <t>Steps 35-39: normal progress - automation researched at step 33, logistics research running, assemblers crafted. Coal ran out (coal=0) at step 39 but nothing was failing. Backstop fired (D67).</t>
         </is>
       </c>
       <c r="L3" s="8" t="n"/>
@@ -12793,12 +12835,6 @@
     </row>
   </sheetData>
   <dataValidations count="9">
-    <dataValidation sqref="I2:I501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Codebook value" error="Pick a value from the list." type="list">
-      <formula1>'Error codebook'!$A$2:$A$10</formula1>
-    </dataValidation>
-    <dataValidation sqref="J2:J501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Codebook value" error="Pick a value from the list." type="list">
-      <formula1>'Error codebook'!$A$2:$A$10</formula1>
-    </dataValidation>
     <dataValidation sqref="L2:L501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Codebook value" error="Pick a value from the list." type="list">
       <formula1>'Guidance codebook'!$A$2:$A$6</formula1>
     </dataValidation>
@@ -12819,6 +12855,12 @@
     </dataValidation>
     <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1,2,3,4,5,6,7,8,5',6',7',8',pilot"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'Error codebook'!$A$2:$A$11</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'Error codebook'!$A$2:$A$11</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13345,7 +13387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -13403,7 +13445,7 @@
         <v/>
       </c>
       <c r="D4" s="14">
-        <f>IFERROR(B4/SUM($B$4:$B$12),0)</f>
+        <f>IFERROR(B4/SUM($B$4:$B$13),0)</f>
         <v/>
       </c>
       <c r="E4" s="13" t="n"/>
@@ -13423,7 +13465,7 @@
         <v/>
       </c>
       <c r="D5" s="14">
-        <f>IFERROR(B5/SUM($B$4:$B$12),0)</f>
+        <f>IFERROR(B5/SUM($B$4:$B$13),0)</f>
         <v/>
       </c>
       <c r="E5" s="13" t="n"/>
@@ -13443,7 +13485,7 @@
         <v/>
       </c>
       <c r="D6" s="14">
-        <f>IFERROR(B6/SUM($B$4:$B$12),0)</f>
+        <f>IFERROR(B6/SUM($B$4:$B$13),0)</f>
         <v/>
       </c>
       <c r="E6" s="13" t="n"/>
@@ -13463,7 +13505,7 @@
         <v/>
       </c>
       <c r="D7" s="14">
-        <f>IFERROR(B7/SUM($B$4:$B$12),0)</f>
+        <f>IFERROR(B7/SUM($B$4:$B$13),0)</f>
         <v/>
       </c>
       <c r="E7" s="13" t="n"/>
@@ -13483,7 +13525,7 @@
         <v/>
       </c>
       <c r="D8" s="14">
-        <f>IFERROR(B8/SUM($B$4:$B$12),0)</f>
+        <f>IFERROR(B8/SUM($B$4:$B$13),0)</f>
         <v/>
       </c>
       <c r="E8" s="13" t="n"/>
@@ -13503,7 +13545,7 @@
         <v/>
       </c>
       <c r="D9" s="14">
-        <f>IFERROR(B9/SUM($B$4:$B$12),0)</f>
+        <f>IFERROR(B9/SUM($B$4:$B$13),0)</f>
         <v/>
       </c>
       <c r="E9" s="13" t="n"/>
@@ -13523,7 +13565,7 @@
         <v/>
       </c>
       <c r="D10" s="14">
-        <f>IFERROR(B10/SUM($B$4:$B$12),0)</f>
+        <f>IFERROR(B10/SUM($B$4:$B$13),0)</f>
         <v/>
       </c>
       <c r="E10" s="13" t="n"/>
@@ -13543,7 +13585,7 @@
         <v/>
       </c>
       <c r="D11" s="14">
-        <f>IFERROR(B11/SUM($B$4:$B$12),0)</f>
+        <f>IFERROR(B11/SUM($B$4:$B$13),0)</f>
         <v/>
       </c>
       <c r="E11" s="13" t="n"/>
@@ -13563,90 +13605,90 @@
         <v/>
       </c>
       <c r="D12" s="14">
-        <f>IFERROR(B12/SUM($B$4:$B$12),0)</f>
+        <f>IFERROR(B12/SUM($B$4:$B$13),0)</f>
         <v/>
       </c>
       <c r="E12" s="13" t="n"/>
       <c r="F12" s="13" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Total stuck events coded</t>
-        </is>
+      <c r="A13" s="13">
+        <f>'Error codebook'!A11&amp;" "&amp;'Error codebook'!B11</f>
+        <v/>
       </c>
       <c r="B13" s="13">
-        <f>SUM(B4:B12)</f>
+        <f>COUNTIF(Annotations!$I$2:$I$501,'Error codebook'!A11)</f>
         <v/>
       </c>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="13" t="n"/>
+      <c r="C13" s="13">
+        <f>COUNTIF(Annotations!$J$2:$J$501,'Error codebook'!A11)</f>
+        <v/>
+      </c>
+      <c r="D13" s="14">
+        <f>IFERROR(B13/SUM($B$4:$B$13),0)</f>
+        <v/>
+      </c>
       <c r="E13" s="13" t="n"/>
       <c r="F13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="n"/>
-      <c r="B14" s="13" t="n"/>
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Total stuck events coded</t>
+        </is>
+      </c>
+      <c r="B14" s="13">
+        <f>SUM(B4:B13)</f>
+        <v/>
+      </c>
       <c r="C14" s="13" t="n"/>
       <c r="D14" s="13" t="n"/>
       <c r="E14" s="13" t="n"/>
       <c r="F14" s="13" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>Guidance code</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Primary</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>Unstuck (yes)</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>Unstuck rate</t>
-        </is>
-      </c>
+      <c r="A15" s="12" t="n"/>
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="12" t="n"/>
       <c r="E15" s="13" t="n"/>
       <c r="F15" s="13" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="13">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Guidance code</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Unstuck (yes)</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Unstuck rate</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13">
         <f>'Guidance codebook'!A2&amp;" "&amp;'Guidance codebook'!B2</f>
         <v/>
       </c>
-      <c r="B16" s="13">
+      <c r="B17" s="13">
         <f>COUNTIF(Annotations!$L$2:$L$501,'Guidance codebook'!A2)</f>
         <v/>
       </c>
-      <c r="C16" s="13">
+      <c r="C17" s="13">
         <f>COUNTIFS(Annotations!$L$2:$L$501,'Guidance codebook'!A2,Annotations!$P$2:$P$501,"yes")</f>
-        <v/>
-      </c>
-      <c r="D16" s="14">
-        <f>IFERROR(C16/B16,0)</f>
-        <v/>
-      </c>
-      <c r="E16" s="13" t="n"/>
-      <c r="F16" s="13" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="13">
-        <f>'Guidance codebook'!A3&amp;" "&amp;'Guidance codebook'!B3</f>
-        <v/>
-      </c>
-      <c r="B17" s="13">
-        <f>COUNTIF(Annotations!$L$2:$L$501,'Guidance codebook'!A3)</f>
-        <v/>
-      </c>
-      <c r="C17" s="13">
-        <f>COUNTIFS(Annotations!$L$2:$L$501,'Guidance codebook'!A3,Annotations!$P$2:$P$501,"yes")</f>
         <v/>
       </c>
       <c r="D17" s="14">
@@ -13658,15 +13700,15 @@
     </row>
     <row r="18">
       <c r="A18" s="13">
-        <f>'Guidance codebook'!A4&amp;" "&amp;'Guidance codebook'!B4</f>
+        <f>'Guidance codebook'!A3&amp;" "&amp;'Guidance codebook'!B3</f>
         <v/>
       </c>
       <c r="B18" s="13">
-        <f>COUNTIF(Annotations!$L$2:$L$501,'Guidance codebook'!A4)</f>
+        <f>COUNTIF(Annotations!$L$2:$L$501,'Guidance codebook'!A3)</f>
         <v/>
       </c>
       <c r="C18" s="13">
-        <f>COUNTIFS(Annotations!$L$2:$L$501,'Guidance codebook'!A4,Annotations!$P$2:$P$501,"yes")</f>
+        <f>COUNTIFS(Annotations!$L$2:$L$501,'Guidance codebook'!A3,Annotations!$P$2:$P$501,"yes")</f>
         <v/>
       </c>
       <c r="D18" s="14">
@@ -13678,15 +13720,15 @@
     </row>
     <row r="19">
       <c r="A19" s="13">
-        <f>'Guidance codebook'!A5&amp;" "&amp;'Guidance codebook'!B5</f>
+        <f>'Guidance codebook'!A4&amp;" "&amp;'Guidance codebook'!B4</f>
         <v/>
       </c>
       <c r="B19" s="13">
-        <f>COUNTIF(Annotations!$L$2:$L$501,'Guidance codebook'!A5)</f>
+        <f>COUNTIF(Annotations!$L$2:$L$501,'Guidance codebook'!A4)</f>
         <v/>
       </c>
       <c r="C19" s="13">
-        <f>COUNTIFS(Annotations!$L$2:$L$501,'Guidance codebook'!A5,Annotations!$P$2:$P$501,"yes")</f>
+        <f>COUNTIFS(Annotations!$L$2:$L$501,'Guidance codebook'!A4,Annotations!$P$2:$P$501,"yes")</f>
         <v/>
       </c>
       <c r="D19" s="14">
@@ -13698,15 +13740,15 @@
     </row>
     <row r="20">
       <c r="A20" s="13">
-        <f>'Guidance codebook'!A6&amp;" "&amp;'Guidance codebook'!B6</f>
+        <f>'Guidance codebook'!A5&amp;" "&amp;'Guidance codebook'!B5</f>
         <v/>
       </c>
       <c r="B20" s="13">
-        <f>COUNTIF(Annotations!$L$2:$L$501,'Guidance codebook'!A6)</f>
+        <f>COUNTIF(Annotations!$L$2:$L$501,'Guidance codebook'!A5)</f>
         <v/>
       </c>
       <c r="C20" s="13">
-        <f>COUNTIFS(Annotations!$L$2:$L$501,'Guidance codebook'!A6,Annotations!$P$2:$P$501,"yes")</f>
+        <f>COUNTIFS(Annotations!$L$2:$L$501,'Guidance codebook'!A5,Annotations!$P$2:$P$501,"yes")</f>
         <v/>
       </c>
       <c r="D20" s="14">
@@ -13717,28 +13759,33 @@
       <c r="F20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>Declined / no guidance</t>
-        </is>
+      <c r="A21" s="13">
+        <f>'Guidance codebook'!A6&amp;" "&amp;'Guidance codebook'!B6</f>
+        <v/>
       </c>
       <c r="B21" s="13">
-        <f>SUMPRODUCT((Annotations!$E$2:$E$501="yes")*(Annotations!$I$2:$I$501&lt;&gt;"")*(Annotations!$L$2:$L$501=""))</f>
+        <f>COUNTIF(Annotations!$L$2:$L$501,'Guidance codebook'!A6)</f>
         <v/>
       </c>
-      <c r="C21" s="13" t="n"/>
-      <c r="D21" s="13" t="n"/>
+      <c r="C21" s="13">
+        <f>COUNTIFS(Annotations!$L$2:$L$501,'Guidance codebook'!A6,Annotations!$P$2:$P$501,"yes")</f>
+        <v/>
+      </c>
+      <c r="D21" s="14">
+        <f>IFERROR(C21/B21,0)</f>
+        <v/>
+      </c>
       <c r="E21" s="13" t="n"/>
       <c r="F21" s="13" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>Hints mentioning API calls</t>
+          <t>Declined / no guidance</t>
         </is>
       </c>
       <c r="B22" s="13">
-        <f>COUNTIF(Annotations!$O$2:$O$501,"yes")</f>
+        <f>SUMPRODUCT((Annotations!$E$2:$E$501="yes")*(Annotations!$I$2:$I$501&lt;&gt;"")*(Annotations!$L$2:$L$501=""))</f>
         <v/>
       </c>
       <c r="C22" s="13" t="n"/>
@@ -13747,19 +13794,22 @@
       <c r="F22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="n"/>
-      <c r="B23" s="13" t="n"/>
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Hints mentioning API calls</t>
+        </is>
+      </c>
+      <c r="B23" s="13">
+        <f>COUNTIF(Annotations!$O$2:$O$501,"yes")</f>
+        <v/>
+      </c>
       <c r="C23" s="13" t="n"/>
       <c r="D23" s="13" t="n"/>
       <c r="E23" s="13" t="n"/>
       <c r="F23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>Error (rows) x guidance (columns), primary codes</t>
-        </is>
-      </c>
+      <c r="A24" s="12" t="n"/>
       <c r="B24" s="13" t="n"/>
       <c r="C24" s="13" t="n"/>
       <c r="D24" s="13" t="n"/>
@@ -13767,264 +13817,303 @@
       <c r="F24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="n"/>
-      <c r="B25" s="12">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Error (rows) x guidance (columns), primary codes</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="n"/>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="12" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="n"/>
+      <c r="B26" s="12">
         <f>'Guidance codebook'!A2</f>
         <v/>
       </c>
-      <c r="C25" s="12">
+      <c r="C26" s="12">
         <f>'Guidance codebook'!A3</f>
         <v/>
       </c>
-      <c r="D25" s="12">
+      <c r="D26" s="12">
         <f>'Guidance codebook'!A4</f>
         <v/>
       </c>
-      <c r="E25" s="12">
+      <c r="E26" s="12">
         <f>'Guidance codebook'!A5</f>
         <v/>
       </c>
-      <c r="F25" s="12">
+      <c r="F26" s="12">
         <f>'Guidance codebook'!A6</f>
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="13">
+    <row r="27">
+      <c r="A27" s="13">
         <f>'Error codebook'!A2</f>
         <v/>
       </c>
-      <c r="B26" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A26,Annotations!$L$2:$L$501,B$25)</f>
+      <c r="B27" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A27,Annotations!$L$2:$L$501,B$26)</f>
         <v/>
       </c>
-      <c r="C26" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A26,Annotations!$L$2:$L$501,C$25)</f>
+      <c r="C27" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A27,Annotations!$L$2:$L$501,C$26)</f>
         <v/>
       </c>
-      <c r="D26" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A26,Annotations!$L$2:$L$501,D$25)</f>
+      <c r="D27" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A27,Annotations!$L$2:$L$501,D$26)</f>
         <v/>
       </c>
-      <c r="E26" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A26,Annotations!$L$2:$L$501,E$25)</f>
+      <c r="E27" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A27,Annotations!$L$2:$L$501,E$26)</f>
         <v/>
       </c>
-      <c r="F26" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A26,Annotations!$L$2:$L$501,F$25)</f>
+      <c r="F27" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A27,Annotations!$L$2:$L$501,F$26)</f>
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="13">
+    <row r="28">
+      <c r="A28" s="13">
         <f>'Error codebook'!A3</f>
         <v/>
       </c>
-      <c r="B27" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A27,Annotations!$L$2:$L$501,B$25)</f>
+      <c r="B28" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A28,Annotations!$L$2:$L$501,B$26)</f>
         <v/>
       </c>
-      <c r="C27" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A27,Annotations!$L$2:$L$501,C$25)</f>
+      <c r="C28" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A28,Annotations!$L$2:$L$501,C$26)</f>
         <v/>
       </c>
-      <c r="D27" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A27,Annotations!$L$2:$L$501,D$25)</f>
+      <c r="D28" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A28,Annotations!$L$2:$L$501,D$26)</f>
         <v/>
       </c>
-      <c r="E27" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A27,Annotations!$L$2:$L$501,E$25)</f>
+      <c r="E28" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A28,Annotations!$L$2:$L$501,E$26)</f>
         <v/>
       </c>
-      <c r="F27" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A27,Annotations!$L$2:$L$501,F$25)</f>
+      <c r="F28" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A28,Annotations!$L$2:$L$501,F$26)</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="13">
+    <row r="29">
+      <c r="A29" s="13">
         <f>'Error codebook'!A4</f>
         <v/>
       </c>
-      <c r="B28" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A28,Annotations!$L$2:$L$501,B$25)</f>
+      <c r="B29" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A29,Annotations!$L$2:$L$501,B$26)</f>
         <v/>
       </c>
-      <c r="C28" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A28,Annotations!$L$2:$L$501,C$25)</f>
+      <c r="C29" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A29,Annotations!$L$2:$L$501,C$26)</f>
         <v/>
       </c>
-      <c r="D28" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A28,Annotations!$L$2:$L$501,D$25)</f>
+      <c r="D29" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A29,Annotations!$L$2:$L$501,D$26)</f>
         <v/>
       </c>
-      <c r="E28" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A28,Annotations!$L$2:$L$501,E$25)</f>
+      <c r="E29" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A29,Annotations!$L$2:$L$501,E$26)</f>
         <v/>
       </c>
-      <c r="F28" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A28,Annotations!$L$2:$L$501,F$25)</f>
+      <c r="F29" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A29,Annotations!$L$2:$L$501,F$26)</f>
         <v/>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="13">
+    <row r="30">
+      <c r="A30" s="13">
         <f>'Error codebook'!A5</f>
         <v/>
       </c>
-      <c r="B29" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A29,Annotations!$L$2:$L$501,B$25)</f>
+      <c r="B30" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A30,Annotations!$L$2:$L$501,B$26)</f>
         <v/>
       </c>
-      <c r="C29" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A29,Annotations!$L$2:$L$501,C$25)</f>
+      <c r="C30" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A30,Annotations!$L$2:$L$501,C$26)</f>
         <v/>
       </c>
-      <c r="D29" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A29,Annotations!$L$2:$L$501,D$25)</f>
+      <c r="D30" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A30,Annotations!$L$2:$L$501,D$26)</f>
         <v/>
       </c>
-      <c r="E29" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A29,Annotations!$L$2:$L$501,E$25)</f>
+      <c r="E30" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A30,Annotations!$L$2:$L$501,E$26)</f>
         <v/>
       </c>
-      <c r="F29" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A29,Annotations!$L$2:$L$501,F$25)</f>
+      <c r="F30" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A30,Annotations!$L$2:$L$501,F$26)</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="13">
+    <row r="31">
+      <c r="A31" s="13">
         <f>'Error codebook'!A6</f>
         <v/>
       </c>
-      <c r="B30" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A30,Annotations!$L$2:$L$501,B$25)</f>
+      <c r="B31" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A31,Annotations!$L$2:$L$501,B$26)</f>
         <v/>
       </c>
-      <c r="C30" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A30,Annotations!$L$2:$L$501,C$25)</f>
+      <c r="C31" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A31,Annotations!$L$2:$L$501,C$26)</f>
         <v/>
       </c>
-      <c r="D30" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A30,Annotations!$L$2:$L$501,D$25)</f>
+      <c r="D31" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A31,Annotations!$L$2:$L$501,D$26)</f>
         <v/>
       </c>
-      <c r="E30" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A30,Annotations!$L$2:$L$501,E$25)</f>
+      <c r="E31" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A31,Annotations!$L$2:$L$501,E$26)</f>
         <v/>
       </c>
-      <c r="F30" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A30,Annotations!$L$2:$L$501,F$25)</f>
+      <c r="F31" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A31,Annotations!$L$2:$L$501,F$26)</f>
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="13">
+    <row r="32">
+      <c r="A32" s="13">
         <f>'Error codebook'!A7</f>
         <v/>
       </c>
-      <c r="B31" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A31,Annotations!$L$2:$L$501,B$25)</f>
+      <c r="B32" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A32,Annotations!$L$2:$L$501,B$26)</f>
         <v/>
       </c>
-      <c r="C31" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A31,Annotations!$L$2:$L$501,C$25)</f>
+      <c r="C32" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A32,Annotations!$L$2:$L$501,C$26)</f>
         <v/>
       </c>
-      <c r="D31" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A31,Annotations!$L$2:$L$501,D$25)</f>
+      <c r="D32" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A32,Annotations!$L$2:$L$501,D$26)</f>
         <v/>
       </c>
-      <c r="E31" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A31,Annotations!$L$2:$L$501,E$25)</f>
+      <c r="E32" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A32,Annotations!$L$2:$L$501,E$26)</f>
         <v/>
       </c>
-      <c r="F31" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A31,Annotations!$L$2:$L$501,F$25)</f>
+      <c r="F32" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A32,Annotations!$L$2:$L$501,F$26)</f>
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="13">
+    <row r="33">
+      <c r="A33" s="13">
         <f>'Error codebook'!A8</f>
         <v/>
       </c>
-      <c r="B32" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A32,Annotations!$L$2:$L$501,B$25)</f>
+      <c r="B33" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A33,Annotations!$L$2:$L$501,B$26)</f>
         <v/>
       </c>
-      <c r="C32" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A32,Annotations!$L$2:$L$501,C$25)</f>
+      <c r="C33" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A33,Annotations!$L$2:$L$501,C$26)</f>
         <v/>
       </c>
-      <c r="D32" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A32,Annotations!$L$2:$L$501,D$25)</f>
+      <c r="D33" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A33,Annotations!$L$2:$L$501,D$26)</f>
         <v/>
       </c>
-      <c r="E32" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A32,Annotations!$L$2:$L$501,E$25)</f>
+      <c r="E33" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A33,Annotations!$L$2:$L$501,E$26)</f>
         <v/>
       </c>
-      <c r="F32" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A32,Annotations!$L$2:$L$501,F$25)</f>
+      <c r="F33" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A33,Annotations!$L$2:$L$501,F$26)</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="13">
+    <row r="34">
+      <c r="A34" s="13">
         <f>'Error codebook'!A9</f>
         <v/>
       </c>
-      <c r="B33" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A33,Annotations!$L$2:$L$501,B$25)</f>
+      <c r="B34" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A34,Annotations!$L$2:$L$501,B$26)</f>
         <v/>
       </c>
-      <c r="C33" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A33,Annotations!$L$2:$L$501,C$25)</f>
+      <c r="C34" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A34,Annotations!$L$2:$L$501,C$26)</f>
         <v/>
       </c>
-      <c r="D33" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A33,Annotations!$L$2:$L$501,D$25)</f>
+      <c r="D34" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A34,Annotations!$L$2:$L$501,D$26)</f>
         <v/>
       </c>
-      <c r="E33" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A33,Annotations!$L$2:$L$501,E$25)</f>
+      <c r="E34" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A34,Annotations!$L$2:$L$501,E$26)</f>
         <v/>
       </c>
-      <c r="F33" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A33,Annotations!$L$2:$L$501,F$25)</f>
+      <c r="F34" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A34,Annotations!$L$2:$L$501,F$26)</f>
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="13">
+    <row r="35">
+      <c r="A35" s="13">
         <f>'Error codebook'!A10</f>
         <v/>
       </c>
-      <c r="B34" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A34,Annotations!$L$2:$L$501,B$25)</f>
+      <c r="B35" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A35,Annotations!$L$2:$L$501,B$26)</f>
         <v/>
       </c>
-      <c r="C34" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A34,Annotations!$L$2:$L$501,C$25)</f>
+      <c r="C35" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A35,Annotations!$L$2:$L$501,C$26)</f>
         <v/>
       </c>
-      <c r="D34" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A34,Annotations!$L$2:$L$501,D$25)</f>
+      <c r="D35" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A35,Annotations!$L$2:$L$501,D$26)</f>
         <v/>
       </c>
-      <c r="E34" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A34,Annotations!$L$2:$L$501,E$25)</f>
+      <c r="E35" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A35,Annotations!$L$2:$L$501,E$26)</f>
         <v/>
       </c>
-      <c r="F34" s="13">
-        <f>COUNTIFS(Annotations!$I$2:$I$501,$A34,Annotations!$L$2:$L$501,F$25)</f>
+      <c r="F35" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A35,Annotations!$L$2:$L$501,F$26)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="15" t="inlineStr">
+      <c r="A36" s="13">
+        <f>'Error codebook'!A11</f>
+        <v/>
+      </c>
+      <c r="B36" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A36,Annotations!$L$2:$L$501,B$26)</f>
+        <v/>
+      </c>
+      <c r="C36" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A36,Annotations!$L$2:$L$501,C$26)</f>
+        <v/>
+      </c>
+      <c r="D36" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A36,Annotations!$L$2:$L$501,D$26)</f>
+        <v/>
+      </c>
+      <c r="E36" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A36,Annotations!$L$2:$L$501,E$26)</f>
+        <v/>
+      </c>
+      <c r="F36" s="13">
+        <f>COUNTIFS(Annotations!$I$2:$I$501,$A36,Annotations!$L$2:$L$501,F$26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>Counts cover Annotations rows 2-501. Worked examples are not counted.</t>
         </is>

</xml_diff>

<commit_message>
data: annotate the cell-5 runs, log B6, complete E0 step 24
The full cell-5 run (20261021T172150-ba5dcf0a) stopped at its 300-step
cap: 13/24 highest, 9/24 contiguous, 19 technologies (1,137 units),
~$1.01. Its 15 backstop requests are drafted in the workbook (13 E10,
one E01, one E02), as pre-freeze; with the stopped run's 6 they export
to annotations/ and validate, awaiting the research lead's verification.
B6: FLE's score is a per-step delta and its automated score counts
consumed hand-made science against the run - explained, not a bug.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/codebook-v0.xlsx
+++ b/docs/codebook-v0.xlsx
@@ -1966,333 +1966,1023 @@
       <c r="T7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="n"/>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="8" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="8" t="n"/>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>19</v>
+      </c>
       <c r="G8" s="8" t="n"/>
-      <c r="H8" s="8" t="n"/>
-      <c r="I8" s="8" t="n"/>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J8" s="8" t="n"/>
-      <c r="K8" s="8" t="n"/>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>Steps 15-19: building iron drills and furnaces, extracting plates, crafting pipes and gears - normal early progress when the backstop fired.</t>
+        </is>
+      </c>
       <c r="L8" s="8" t="n"/>
       <c r="M8" s="8" t="n"/>
       <c r="N8" s="8" t="n"/>
       <c r="O8" s="8" t="n"/>
       <c r="P8" s="16" t="n"/>
-      <c r="Q8" s="8" t="n"/>
-      <c r="R8" s="8" t="n"/>
-      <c r="S8" s="8" t="n"/>
+      <c r="Q8" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R8" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S8" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T8" s="8" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="n"/>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>39</v>
+      </c>
       <c r="G9" s="8" t="n"/>
-      <c r="H9" s="8" t="n"/>
-      <c r="I9" s="8" t="n"/>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
       <c r="J9" s="8" t="n"/>
-      <c r="K9" s="8" t="n"/>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>Step 38: AttributeError - 'PipeGroup' object has no attribute 'fluid' (read a field the API does not have). Recovered at once; steps 35-39 otherwise assembling steam power (boiler, pipes, pole, engine).</t>
+        </is>
+      </c>
       <c r="L9" s="8" t="n"/>
       <c r="M9" s="8" t="n"/>
       <c r="N9" s="8" t="n"/>
       <c r="O9" s="8" t="n"/>
       <c r="P9" s="16" t="n"/>
-      <c r="Q9" s="8" t="n"/>
-      <c r="R9" s="8" t="n"/>
-      <c r="S9" s="8" t="n"/>
+      <c r="Q9" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R9" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S9" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="n"/>
-      <c r="B10" s="8" t="n"/>
-      <c r="C10" s="8" t="n"/>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="8" t="n"/>
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>59</v>
+      </c>
       <c r="G10" s="8" t="n"/>
-      <c r="H10" s="8" t="n"/>
-      <c r="I10" s="8" t="n"/>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
       <c r="J10" s="8" t="n"/>
-      <c r="K10" s="8" t="n"/>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>Step 59: 'Could not place burner-mining-drill', caught by the agent's own try block. Steps 55-58 otherwise normal: red packs, drills, furnaces.</t>
+        </is>
+      </c>
       <c r="L10" s="8" t="n"/>
       <c r="M10" s="8" t="n"/>
       <c r="N10" s="8" t="n"/>
       <c r="O10" s="8" t="n"/>
       <c r="P10" s="16" t="n"/>
-      <c r="Q10" s="8" t="n"/>
-      <c r="R10" s="8" t="n"/>
-      <c r="S10" s="8" t="n"/>
+      <c r="Q10" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R10" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S10" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T10" s="8" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="n"/>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="8" t="n"/>
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>79</v>
+      </c>
       <c r="G11" s="8" t="n"/>
-      <c r="H11" s="8" t="n"/>
-      <c r="I11" s="8" t="n"/>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J11" s="8" t="n"/>
-      <c r="K11" s="8" t="n"/>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>Steps 75-79: harvesting, extracting plates; logistics research finished at step 78 and the labs briefly idle (no research set) - a transition, not an error.</t>
+        </is>
+      </c>
       <c r="L11" s="8" t="n"/>
       <c r="M11" s="8" t="n"/>
       <c r="N11" s="8" t="n"/>
       <c r="O11" s="8" t="n"/>
       <c r="P11" s="16" t="n"/>
-      <c r="Q11" s="8" t="n"/>
-      <c r="R11" s="8" t="n"/>
-      <c r="S11" s="8" t="n"/>
+      <c r="Q11" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R11" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S11" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="n"/>
-      <c r="B12" s="8" t="n"/>
-      <c r="C12" s="8" t="n"/>
-      <c r="D12" s="8" t="n"/>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="8" t="n"/>
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>99</v>
+      </c>
       <c r="G12" s="8" t="n"/>
-      <c r="H12" s="8" t="n"/>
-      <c r="I12" s="8" t="n"/>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J12" s="8" t="n"/>
-      <c r="K12" s="8" t="n"/>
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>Steps 95-99: crafting 30 red packs, refuelling drills, coal from the chest, harvesting stone - normal progress.</t>
+        </is>
+      </c>
       <c r="L12" s="8" t="n"/>
       <c r="M12" s="8" t="n"/>
       <c r="N12" s="8" t="n"/>
       <c r="O12" s="8" t="n"/>
       <c r="P12" s="16" t="n"/>
-      <c r="Q12" s="8" t="n"/>
-      <c r="R12" s="8" t="n"/>
-      <c r="S12" s="8" t="n"/>
+      <c r="Q12" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R12" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S12" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T12" s="8" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="n"/>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="8" t="n"/>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>119</v>
+      </c>
       <c r="G13" s="8" t="n"/>
-      <c r="H13" s="8" t="n"/>
-      <c r="I13" s="8" t="n"/>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J13" s="8" t="n"/>
-      <c r="K13" s="8" t="n"/>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>Steps 115-119: no error in the window. Manual loop: carrying plates and coal, hand-crafting science, feeding labs; no assemblers, belts or inserters placed - why the ladder stalled at 13 (v1 candidate).</t>
+        </is>
+      </c>
       <c r="L13" s="8" t="n"/>
       <c r="M13" s="8" t="n"/>
       <c r="N13" s="8" t="n"/>
       <c r="O13" s="8" t="n"/>
       <c r="P13" s="16" t="n"/>
-      <c r="Q13" s="8" t="n"/>
-      <c r="R13" s="8" t="n"/>
-      <c r="S13" s="8" t="n"/>
+      <c r="Q13" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R13" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S13" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="n"/>
-      <c r="B14" s="8" t="n"/>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="8" t="n"/>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="8" t="n"/>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>139</v>
+      </c>
       <c r="G14" s="8" t="n"/>
-      <c r="H14" s="8" t="n"/>
-      <c r="I14" s="8" t="n"/>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J14" s="8" t="n"/>
-      <c r="K14" s="8" t="n"/>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>Steps 135-139: no error in the window. Manual loop: carrying plates and coal, hand-crafting science, feeding labs; no assemblers, belts or inserters placed - why the ladder stalled at 13 (v1 candidate).</t>
+        </is>
+      </c>
       <c r="L14" s="8" t="n"/>
       <c r="M14" s="8" t="n"/>
       <c r="N14" s="8" t="n"/>
       <c r="O14" s="8" t="n"/>
       <c r="P14" s="16" t="n"/>
-      <c r="Q14" s="8" t="n"/>
-      <c r="R14" s="8" t="n"/>
-      <c r="S14" s="8" t="n"/>
+      <c r="Q14" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R14" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S14" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T14" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="n"/>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="8" t="n"/>
-      <c r="E15" s="8" t="n"/>
-      <c r="F15" s="8" t="n"/>
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>159</v>
+      </c>
       <c r="G15" s="8" t="n"/>
-      <c r="H15" s="8" t="n"/>
-      <c r="I15" s="8" t="n"/>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J15" s="8" t="n"/>
-      <c r="K15" s="8" t="n"/>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>Steps 155-159: no error in the window. Manual loop: carrying plates and coal, hand-crafting science, feeding labs; no assemblers, belts or inserters placed - why the ladder stalled at 13 (v1 candidate).</t>
+        </is>
+      </c>
       <c r="L15" s="8" t="n"/>
       <c r="M15" s="8" t="n"/>
       <c r="N15" s="8" t="n"/>
       <c r="O15" s="8" t="n"/>
       <c r="P15" s="16" t="n"/>
-      <c r="Q15" s="8" t="n"/>
-      <c r="R15" s="8" t="n"/>
-      <c r="S15" s="8" t="n"/>
+      <c r="Q15" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R15" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S15" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T15" s="8" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="n"/>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="n"/>
-      <c r="F16" s="8" t="n"/>
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>179</v>
+      </c>
       <c r="G16" s="8" t="n"/>
-      <c r="H16" s="8" t="n"/>
-      <c r="I16" s="8" t="n"/>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J16" s="8" t="n"/>
-      <c r="K16" s="8" t="n"/>
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>Steps 175-179: no error in the window. Manual loop: carrying plates and coal, hand-crafting science, feeding labs; no assemblers, belts or inserters placed - why the ladder stalled at 13 (v1 candidate).</t>
+        </is>
+      </c>
       <c r="L16" s="8" t="n"/>
       <c r="M16" s="8" t="n"/>
       <c r="N16" s="8" t="n"/>
       <c r="O16" s="8" t="n"/>
       <c r="P16" s="16" t="n"/>
-      <c r="Q16" s="8" t="n"/>
-      <c r="R16" s="8" t="n"/>
-      <c r="S16" s="8" t="n"/>
+      <c r="Q16" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R16" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S16" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T16" s="8" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="n"/>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="8" t="n"/>
-      <c r="E17" s="8" t="n"/>
-      <c r="F17" s="8" t="n"/>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>199</v>
+      </c>
       <c r="G17" s="8" t="n"/>
-      <c r="H17" s="8" t="n"/>
-      <c r="I17" s="8" t="n"/>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J17" s="8" t="n"/>
-      <c r="K17" s="8" t="n"/>
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>Steps 195-199: no error in the window. Manual loop: carrying plates and coal, hand-crafting science, feeding labs; no assemblers, belts or inserters placed - why the ladder stalled at 13 (v1 candidate).</t>
+        </is>
+      </c>
       <c r="L17" s="8" t="n"/>
       <c r="M17" s="8" t="n"/>
       <c r="N17" s="8" t="n"/>
       <c r="O17" s="8" t="n"/>
       <c r="P17" s="16" t="n"/>
-      <c r="Q17" s="8" t="n"/>
-      <c r="R17" s="8" t="n"/>
-      <c r="S17" s="8" t="n"/>
+      <c r="Q17" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R17" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S17" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T17" s="8" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="n"/>
-      <c r="B18" s="8" t="n"/>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="8" t="n"/>
-      <c r="E18" s="8" t="n"/>
-      <c r="F18" s="8" t="n"/>
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>219</v>
+      </c>
       <c r="G18" s="8" t="n"/>
-      <c r="H18" s="8" t="n"/>
-      <c r="I18" s="8" t="n"/>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J18" s="8" t="n"/>
-      <c r="K18" s="8" t="n"/>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>Steps 215-219: no error in the window. Manual loop: carrying plates and coal, hand-crafting science, feeding labs; no assemblers, belts or inserters placed - why the ladder stalled at 13 (v1 candidate).</t>
+        </is>
+      </c>
       <c r="L18" s="8" t="n"/>
       <c r="M18" s="8" t="n"/>
       <c r="N18" s="8" t="n"/>
       <c r="O18" s="8" t="n"/>
       <c r="P18" s="16" t="n"/>
-      <c r="Q18" s="8" t="n"/>
-      <c r="R18" s="8" t="n"/>
-      <c r="S18" s="8" t="n"/>
+      <c r="Q18" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R18" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S18" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T18" s="8" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="8" t="n"/>
-      <c r="E19" s="8" t="n"/>
-      <c r="F19" s="8" t="n"/>
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>239</v>
+      </c>
       <c r="G19" s="8" t="n"/>
-      <c r="H19" s="8" t="n"/>
-      <c r="I19" s="8" t="n"/>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J19" s="8" t="n"/>
-      <c r="K19" s="8" t="n"/>
+      <c r="K19" s="8" t="inlineStr">
+        <is>
+          <t>Steps 235-239: no error in the window. Manual loop: carrying plates and coal, hand-crafting science, feeding labs; no assemblers, belts or inserters placed - why the ladder stalled at 13 (v1 candidate).</t>
+        </is>
+      </c>
       <c r="L19" s="8" t="n"/>
       <c r="M19" s="8" t="n"/>
       <c r="N19" s="8" t="n"/>
       <c r="O19" s="8" t="n"/>
       <c r="P19" s="16" t="n"/>
-      <c r="Q19" s="8" t="n"/>
-      <c r="R19" s="8" t="n"/>
-      <c r="S19" s="8" t="n"/>
+      <c r="Q19" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R19" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S19" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T19" s="8" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="n"/>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="8" t="n"/>
-      <c r="E20" s="8" t="n"/>
-      <c r="F20" s="8" t="n"/>
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>259</v>
+      </c>
       <c r="G20" s="8" t="n"/>
-      <c r="H20" s="8" t="n"/>
-      <c r="I20" s="8" t="n"/>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J20" s="8" t="n"/>
-      <c r="K20" s="8" t="n"/>
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>Steps 255-259: no error in the window. Manual loop: carrying plates and coal, hand-crafting science, feeding labs; no assemblers, belts or inserters placed - why the ladder stalled at 13 (v1 candidate).</t>
+        </is>
+      </c>
       <c r="L20" s="8" t="n"/>
       <c r="M20" s="8" t="n"/>
       <c r="N20" s="8" t="n"/>
       <c r="O20" s="8" t="n"/>
       <c r="P20" s="16" t="n"/>
-      <c r="Q20" s="8" t="n"/>
-      <c r="R20" s="8" t="n"/>
-      <c r="S20" s="8" t="n"/>
+      <c r="Q20" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R20" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S20" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T20" s="8" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="n"/>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="8" t="n"/>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="8" t="n"/>
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>279</v>
+      </c>
       <c r="G21" s="8" t="n"/>
-      <c r="H21" s="8" t="n"/>
-      <c r="I21" s="8" t="n"/>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J21" s="8" t="n"/>
-      <c r="K21" s="8" t="n"/>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>Steps 275-279: no error in the window. Manual loop: carrying plates and coal, hand-crafting science, feeding labs; no assemblers, belts or inserters placed - why the ladder stalled at 13 (v1 candidate).</t>
+        </is>
+      </c>
       <c r="L21" s="8" t="n"/>
       <c r="M21" s="8" t="n"/>
       <c r="N21" s="8" t="n"/>
       <c r="O21" s="8" t="n"/>
       <c r="P21" s="16" t="n"/>
-      <c r="Q21" s="8" t="n"/>
-      <c r="R21" s="8" t="n"/>
-      <c r="S21" s="8" t="n"/>
+      <c r="Q21" s="8" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R21" s="8" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S21" s="8" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T21" s="8" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="n"/>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9" t="n"/>
-      <c r="F22" s="9" t="n"/>
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>20261021T172150-ba5dcf0a</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>claude-haiku-5-5</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>299</v>
+      </c>
       <c r="G22" s="9" t="n"/>
-      <c r="H22" s="9" t="n"/>
-      <c r="I22" s="9" t="n"/>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>20 steps without a request for help</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
       <c r="J22" s="9" t="n"/>
-      <c r="K22" s="9" t="n"/>
+      <c r="K22" s="9" t="inlineStr">
+        <is>
+          <t>Steps 295-299: no error in the window. Manual loop: carrying plates and coal, hand-crafting science, feeding labs; no assemblers, belts or inserters placed - why the ladder stalled at 13 (v1 candidate).</t>
+        </is>
+      </c>
       <c r="L22" s="9" t="n"/>
       <c r="M22" s="9" t="n"/>
       <c r="N22" s="9" t="n"/>
       <c r="O22" s="9" t="n"/>
       <c r="P22" s="17" t="n"/>
-      <c r="Q22" s="9" t="n"/>
-      <c r="R22" s="9" t="n"/>
-      <c r="S22" s="9" t="n"/>
+      <c r="Q22" s="9" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="R22" s="9" t="inlineStr">
+        <is>
+          <t>Claude (draft)</t>
+        </is>
+      </c>
+      <c r="S22" s="9" t="inlineStr">
+        <is>
+          <t>Pre-freeze run (harness c3fab47, D66 instructions); exclude from grid analysis.</t>
+        </is>
+      </c>
       <c r="T22" s="9" t="n"/>
     </row>
     <row r="23">
@@ -13387,7 +14077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -14111,7 +14801,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="15" t="inlineStr">
         <is>

</xml_diff>